<commit_message>
fix(cbr): align header injection with updated template and sync templates
</commit_message>
<xml_diff>
--- a/app/templates/Temp_CBR_ASTM.xlsx
+++ b/app/templates/Temp_CBR_ASTM.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24332"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27928"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Mi unidad\4.0 Área de Sistemas\8. FORMATO ENSAYO NUEVO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20CA5E50-FFBE-46CC-A411-2CD93B7256ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{125A63E1-FFBC-475F-B49D-22BDB4BA5FA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="151" uniqueCount="139">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="143">
   <si>
     <t>FC</t>
   </si>
@@ -508,6 +508,18 @@
   <si>
     <t>INS-000</t>
   </si>
+  <si>
+    <t>MUESTRA</t>
+  </si>
+  <si>
+    <t>N° OT</t>
+  </si>
+  <si>
+    <t>FECHA DE ENSAYO</t>
+  </si>
+  <si>
+    <t>REALIZADO</t>
+  </si>
 </sst>
 </file>
 
@@ -519,7 +531,7 @@
     <numFmt numFmtId="166" formatCode="&quot;FORMATO F-LEM-P-SU-11.01&quot;"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
-  <fonts count="19" x14ac:knownFonts="1">
+  <fonts count="20" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
@@ -631,6 +643,12 @@
       <color rgb="FF000000"/>
       <name val="Times New Roman"/>
       <family val="1"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -861,7 +879,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="185">
+  <cellXfs count="195">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1173,6 +1191,218 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="8" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="11" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="4" borderId="16" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1221,223 +1451,41 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="8" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="11" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="16" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -1702,576 +1750,6 @@
         </a:extLst>
       </xdr:spPr>
     </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>301623</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>361133</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>153987</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="11" name="5 CuadroTexto">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4704CA25-5610-47AA-9E8E-F64DFE6F59E0}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="984248" y="1508125"/>
-          <a:ext cx="1520010" cy="257175"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-PE" sz="900">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>MUESTRA</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>408938</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>315910</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>153987</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="12" name="6 CuadroTexto">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{809DA074-925A-4CF3-891A-7FC6B52F6C9D}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2552063" y="1508125"/>
-          <a:ext cx="1518285" cy="257175"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-PE" sz="900">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>N°</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="es-PE" sz="900" baseline="0">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> OT</a:t>
-          </a:r>
-          <a:endParaRPr lang="es-PE" sz="900">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>390205</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>35378</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>153987</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="13" name="8 CuadroTexto">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{09887C65-D022-4AEC-A518-FC7BBF765B65}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4144643" y="1508125"/>
-          <a:ext cx="1558110" cy="257175"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-PE" sz="900">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>FECHA DE</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="es-PE" sz="900" baseline="0">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t> ENSAYO</a:t>
-          </a:r>
-          <a:endParaRPr lang="es-PE" sz="900">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>1</xdr:col>
-      <xdr:colOff>301623</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>192405</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>361133</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>107950</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="21" name="4 Rectángulo">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AB98F895-CD54-4986-9A1B-9A6B3E090744}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="984248" y="1803718"/>
-          <a:ext cx="1520010" cy="312420"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="3175">
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="dk1"/>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="lt1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="es-PE" sz="900">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>422273</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>1588</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>315910</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>107950</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="22" name="4 Rectángulo">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EA0E0A20-6E31-4AB4-954E-82FF837BBD4E}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="2565398" y="1811338"/>
-          <a:ext cx="1504950" cy="304800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="3175">
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="dk1"/>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="lt1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="es-PE" sz="900">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>6</xdr:col>
-      <xdr:colOff>390205</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>3175</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>35378</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>109537</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="23" name="4 Rectángulo">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{4A61A1DA-C2AA-41D7-A7F7-C0964547BBC6}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="4144643" y="1812925"/>
-          <a:ext cx="1558110" cy="304800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="3175">
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="dk1"/>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="lt1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="es-PE" sz="900">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>85723</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>95250</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>411160</xdr:colOff>
-      <xdr:row>7</xdr:row>
-      <xdr:rowOff>153987</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="24" name="6 CuadroTexto">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{18B21773-6BEF-4556-A46B-81E14107B91B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5753098" y="1508125"/>
-          <a:ext cx="2047875" cy="257175"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="lt1"/>
-        </a:solidFill>
-        <a:ln w="9525" cmpd="sng">
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="square" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="es-PE" sz="900">
-              <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            </a:rPr>
-            <a:t>REALIZADO</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>91120</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>1588</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>14</xdr:col>
-      <xdr:colOff>401308</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>107950</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="25" name="4 Rectángulo">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7F5355A1-6563-46F4-A774-0231D355375C}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="5758495" y="1811338"/>
-          <a:ext cx="2032626" cy="304800"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="3175">
-          <a:solidFill>
-            <a:sysClr val="windowText" lastClr="000000"/>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="dk1"/>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="lt1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="dk1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="dk1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="t"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:endParaRPr lang="es-PE" sz="900">
-            <a:latin typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-            <a:cs typeface="Arial" panose="020B0604020202020204" pitchFamily="34" charset="0"/>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
@@ -2930,43 +2408,43 @@
       <c r="A2" s="81"/>
       <c r="B2" s="82"/>
       <c r="C2" s="83"/>
-      <c r="D2" s="103" t="s">
+      <c r="D2" s="170" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="104"/>
-      <c r="F2" s="104"/>
-      <c r="G2" s="104"/>
-      <c r="H2" s="104"/>
-      <c r="I2" s="104"/>
-      <c r="J2" s="104"/>
-      <c r="K2" s="104"/>
-      <c r="L2" s="104"/>
-      <c r="M2" s="104"/>
-      <c r="N2" s="104"/>
-      <c r="O2" s="104"/>
-      <c r="P2" s="104"/>
-      <c r="Q2" s="105"/>
+      <c r="E2" s="171"/>
+      <c r="F2" s="171"/>
+      <c r="G2" s="171"/>
+      <c r="H2" s="171"/>
+      <c r="I2" s="171"/>
+      <c r="J2" s="171"/>
+      <c r="K2" s="171"/>
+      <c r="L2" s="171"/>
+      <c r="M2" s="171"/>
+      <c r="N2" s="171"/>
+      <c r="O2" s="171"/>
+      <c r="P2" s="171"/>
+      <c r="Q2" s="172"/>
     </row>
     <row r="3" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="81"/>
       <c r="B3" s="82"/>
       <c r="C3" s="83"/>
-      <c r="D3" s="106" t="s">
+      <c r="D3" s="173" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="107"/>
-      <c r="F3" s="107"/>
-      <c r="G3" s="107"/>
-      <c r="H3" s="107"/>
-      <c r="I3" s="107"/>
-      <c r="J3" s="107"/>
-      <c r="K3" s="107"/>
-      <c r="L3" s="107"/>
-      <c r="M3" s="107"/>
-      <c r="N3" s="107"/>
-      <c r="O3" s="107"/>
-      <c r="P3" s="107"/>
-      <c r="Q3" s="108"/>
+      <c r="E3" s="174"/>
+      <c r="F3" s="174"/>
+      <c r="G3" s="174"/>
+      <c r="H3" s="174"/>
+      <c r="I3" s="174"/>
+      <c r="J3" s="174"/>
+      <c r="K3" s="174"/>
+      <c r="L3" s="174"/>
+      <c r="M3" s="174"/>
+      <c r="N3" s="174"/>
+      <c r="O3" s="174"/>
+      <c r="P3" s="174"/>
+      <c r="Q3" s="175"/>
     </row>
     <row r="4" spans="1:17" ht="3" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="81"/>
@@ -3045,16 +2523,24 @@
     <row r="8" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="32"/>
       <c r="C8" s="32"/>
-      <c r="D8" s="32"/>
-      <c r="E8" s="32"/>
-      <c r="F8" s="32"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="32"/>
-      <c r="J8" s="32"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="15"/>
+      <c r="D8" s="190" t="s">
+        <v>139</v>
+      </c>
+      <c r="E8" s="191"/>
+      <c r="F8" s="189" t="s">
+        <v>140</v>
+      </c>
+      <c r="G8" s="185"/>
+      <c r="H8" s="186" t="s">
+        <v>141</v>
+      </c>
+      <c r="I8" s="187"/>
+      <c r="J8" s="185"/>
+      <c r="K8" s="186" t="s">
+        <v>142</v>
+      </c>
+      <c r="L8" s="188"/>
+      <c r="M8" s="60"/>
       <c r="N8" s="15"/>
       <c r="O8" s="15"/>
     </row>
@@ -3062,16 +2548,16 @@
       <c r="A9" s="32"/>
       <c r="B9" s="32"/>
       <c r="C9" s="32"/>
-      <c r="D9" s="32"/>
-      <c r="E9" s="32"/>
-      <c r="F9" s="32"/>
-      <c r="G9" s="32"/>
-      <c r="H9" s="32"/>
-      <c r="I9" s="32"/>
-      <c r="J9" s="32"/>
-      <c r="K9" s="14"/>
-      <c r="L9" s="14"/>
-      <c r="M9" s="14"/>
+      <c r="D9" s="185"/>
+      <c r="E9" s="187"/>
+      <c r="F9" s="192"/>
+      <c r="G9" s="185"/>
+      <c r="H9" s="193"/>
+      <c r="I9" s="187"/>
+      <c r="J9" s="185"/>
+      <c r="K9" s="59"/>
+      <c r="L9" s="59"/>
+      <c r="M9" s="194"/>
       <c r="N9" s="14"/>
       <c r="O9" s="14"/>
     </row>
@@ -3093,46 +2579,46 @@
       <c r="O10" s="35"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="110" t="s">
+      <c r="A11" s="177" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="111"/>
-      <c r="C11" s="111"/>
-      <c r="D11" s="111"/>
-      <c r="E11" s="111"/>
-      <c r="F11" s="111"/>
-      <c r="G11" s="111"/>
-      <c r="H11" s="111"/>
-      <c r="I11" s="111"/>
-      <c r="J11" s="111"/>
-      <c r="K11" s="111"/>
-      <c r="L11" s="111"/>
-      <c r="M11" s="111"/>
-      <c r="N11" s="111"/>
-      <c r="O11" s="111"/>
-      <c r="P11" s="111"/>
-      <c r="Q11" s="112"/>
+      <c r="B11" s="178"/>
+      <c r="C11" s="178"/>
+      <c r="D11" s="178"/>
+      <c r="E11" s="178"/>
+      <c r="F11" s="178"/>
+      <c r="G11" s="178"/>
+      <c r="H11" s="178"/>
+      <c r="I11" s="178"/>
+      <c r="J11" s="178"/>
+      <c r="K11" s="178"/>
+      <c r="L11" s="178"/>
+      <c r="M11" s="178"/>
+      <c r="N11" s="178"/>
+      <c r="O11" s="178"/>
+      <c r="P11" s="178"/>
+      <c r="Q11" s="179"/>
     </row>
     <row r="12" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="113" t="s">
+      <c r="A12" s="180" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="114"/>
-      <c r="C12" s="114"/>
-      <c r="D12" s="114"/>
-      <c r="E12" s="114"/>
-      <c r="F12" s="114"/>
-      <c r="G12" s="114"/>
-      <c r="H12" s="114"/>
-      <c r="I12" s="114"/>
-      <c r="J12" s="114"/>
-      <c r="K12" s="114"/>
-      <c r="L12" s="114"/>
-      <c r="M12" s="114"/>
-      <c r="N12" s="114"/>
-      <c r="O12" s="114"/>
-      <c r="P12" s="114"/>
-      <c r="Q12" s="115"/>
+      <c r="B12" s="181"/>
+      <c r="C12" s="181"/>
+      <c r="D12" s="181"/>
+      <c r="E12" s="181"/>
+      <c r="F12" s="181"/>
+      <c r="G12" s="181"/>
+      <c r="H12" s="181"/>
+      <c r="I12" s="181"/>
+      <c r="J12" s="181"/>
+      <c r="K12" s="181"/>
+      <c r="L12" s="181"/>
+      <c r="M12" s="181"/>
+      <c r="N12" s="181"/>
+      <c r="O12" s="181"/>
+      <c r="P12" s="181"/>
+      <c r="Q12" s="182"/>
     </row>
     <row r="13" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="36"/>
@@ -3160,8 +2646,8 @@
       <c r="B14" s="14"/>
       <c r="C14" s="43"/>
       <c r="D14" s="14"/>
-      <c r="E14" s="179"/>
-      <c r="F14" s="179"/>
+      <c r="E14" s="124"/>
+      <c r="F14" s="124"/>
       <c r="G14" s="87" t="s">
         <v>23</v>
       </c>
@@ -3171,8 +2657,8 @@
       <c r="N14" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="O14" s="175"/>
-      <c r="P14" s="176"/>
+      <c r="O14" s="122"/>
+      <c r="P14" s="123"/>
       <c r="Q14" s="27"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -3182,8 +2668,8 @@
       <c r="B15" s="14"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
-      <c r="E15" s="179"/>
-      <c r="F15" s="179"/>
+      <c r="E15" s="124"/>
+      <c r="F15" s="124"/>
       <c r="G15" s="87" t="s">
         <v>25</v>
       </c>
@@ -3193,8 +2679,8 @@
       <c r="N15" s="45" t="s">
         <v>68</v>
       </c>
-      <c r="O15" s="175"/>
-      <c r="P15" s="176"/>
+      <c r="O15" s="122"/>
+      <c r="P15" s="123"/>
       <c r="Q15" s="27"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -3206,7 +2692,7 @@
       <c r="D16" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="E16" s="180"/>
+      <c r="E16" s="116"/>
       <c r="G16" s="72"/>
       <c r="H16" s="14"/>
       <c r="K16" s="14"/>
@@ -3214,8 +2700,8 @@
       <c r="N16" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="O16" s="175"/>
-      <c r="P16" s="176"/>
+      <c r="O16" s="122"/>
+      <c r="P16" s="123"/>
       <c r="Q16" s="27"/>
     </row>
     <row r="17" spans="1:20" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
@@ -3225,7 +2711,7 @@
       <c r="D17" s="88" t="s">
         <v>61</v>
       </c>
-      <c r="E17" s="163"/>
+      <c r="E17" s="106"/>
       <c r="F17" s="14"/>
       <c r="H17" s="14"/>
       <c r="K17" s="14"/>
@@ -3233,8 +2719,8 @@
       <c r="N17" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="O17" s="175"/>
-      <c r="P17" s="176"/>
+      <c r="O17" s="122"/>
+      <c r="P17" s="123"/>
       <c r="Q17" s="27"/>
     </row>
     <row r="18" spans="1:20" ht="6" customHeight="1" x14ac:dyDescent="0.2">
@@ -3265,8 +2751,8 @@
       <c r="D19" s="90"/>
       <c r="E19" s="98"/>
       <c r="F19" s="98"/>
-      <c r="G19" s="174"/>
-      <c r="H19" s="174"/>
+      <c r="G19" s="137"/>
+      <c r="H19" s="137"/>
       <c r="I19" s="91"/>
       <c r="J19" s="91"/>
       <c r="K19" s="90"/>
@@ -3284,243 +2770,243 @@
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
       <c r="D20" s="48"/>
-      <c r="E20" s="132" t="s">
+      <c r="E20" s="158" t="s">
         <v>36</v>
       </c>
-      <c r="F20" s="132"/>
-      <c r="G20" s="132"/>
-      <c r="H20" s="132"/>
-      <c r="I20" s="132"/>
-      <c r="J20" s="132"/>
-      <c r="K20" s="132"/>
-      <c r="L20" s="132"/>
-      <c r="M20" s="132"/>
-      <c r="N20" s="132"/>
-      <c r="O20" s="132"/>
-      <c r="P20" s="132"/>
-      <c r="Q20" s="133"/>
+      <c r="F20" s="158"/>
+      <c r="G20" s="158"/>
+      <c r="H20" s="158"/>
+      <c r="I20" s="158"/>
+      <c r="J20" s="158"/>
+      <c r="K20" s="158"/>
+      <c r="L20" s="158"/>
+      <c r="M20" s="158"/>
+      <c r="N20" s="158"/>
+      <c r="O20" s="158"/>
+      <c r="P20" s="158"/>
+      <c r="Q20" s="159"/>
     </row>
     <row r="21" spans="1:20" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="160" t="s">
+      <c r="A21" s="183" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="160"/>
-      <c r="C21" s="160"/>
-      <c r="D21" s="160" t="s">
+      <c r="B21" s="183"/>
+      <c r="C21" s="183"/>
+      <c r="D21" s="183" t="s">
         <v>27</v>
       </c>
-      <c r="E21" s="160"/>
-      <c r="F21" s="160"/>
-      <c r="G21" s="160"/>
-      <c r="H21" s="160" t="s">
+      <c r="E21" s="183"/>
+      <c r="F21" s="183"/>
+      <c r="G21" s="183"/>
+      <c r="H21" s="183" t="s">
         <v>28</v>
       </c>
-      <c r="I21" s="160"/>
-      <c r="J21" s="160"/>
-      <c r="K21" s="160"/>
-      <c r="L21" s="160" t="s">
+      <c r="I21" s="183"/>
+      <c r="J21" s="183"/>
+      <c r="K21" s="183"/>
+      <c r="L21" s="183" t="s">
         <v>29</v>
       </c>
-      <c r="M21" s="160"/>
-      <c r="N21" s="160"/>
-      <c r="O21" s="160"/>
-      <c r="P21" s="160"/>
-      <c r="Q21" s="160"/>
+      <c r="M21" s="183"/>
+      <c r="N21" s="183"/>
+      <c r="O21" s="183"/>
+      <c r="P21" s="183"/>
+      <c r="Q21" s="183"/>
       <c r="R21" s="13"/>
     </row>
     <row r="22" spans="1:20" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="160" t="s">
+      <c r="A22" s="183" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="160"/>
-      <c r="C22" s="160"/>
-      <c r="D22" s="160" t="s">
+      <c r="B22" s="183"/>
+      <c r="C22" s="183"/>
+      <c r="D22" s="183" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="160"/>
-      <c r="F22" s="160" t="s">
+      <c r="E22" s="183"/>
+      <c r="F22" s="183" t="s">
         <v>32</v>
       </c>
-      <c r="G22" s="160"/>
-      <c r="H22" s="160" t="s">
+      <c r="G22" s="183"/>
+      <c r="H22" s="183" t="s">
         <v>31</v>
       </c>
-      <c r="I22" s="160"/>
-      <c r="J22" s="160" t="s">
+      <c r="I22" s="183"/>
+      <c r="J22" s="183" t="s">
         <v>32</v>
       </c>
-      <c r="K22" s="160"/>
-      <c r="L22" s="160" t="s">
+      <c r="K22" s="183"/>
+      <c r="L22" s="183" t="s">
         <v>31</v>
       </c>
-      <c r="M22" s="160"/>
-      <c r="N22" s="160"/>
-      <c r="O22" s="160" t="s">
+      <c r="M22" s="183"/>
+      <c r="N22" s="183"/>
+      <c r="O22" s="183" t="s">
         <v>32</v>
       </c>
-      <c r="P22" s="160"/>
-      <c r="Q22" s="160"/>
+      <c r="P22" s="183"/>
+      <c r="Q22" s="183"/>
       <c r="R22" s="13"/>
     </row>
     <row r="23" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="122" t="s">
+      <c r="A23" s="151" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="122"/>
-      <c r="C23" s="122"/>
-      <c r="D23" s="181" t="s">
+      <c r="B23" s="151"/>
+      <c r="C23" s="151"/>
+      <c r="D23" s="167" t="s">
         <v>137</v>
       </c>
-      <c r="E23" s="181"/>
-      <c r="F23" s="181"/>
-      <c r="G23" s="181"/>
-      <c r="H23" s="125">
+      <c r="E23" s="167"/>
+      <c r="F23" s="167"/>
+      <c r="G23" s="167"/>
+      <c r="H23" s="144">
         <v>25</v>
       </c>
-      <c r="I23" s="125"/>
-      <c r="J23" s="125"/>
-      <c r="K23" s="125"/>
-      <c r="L23" s="125">
+      <c r="I23" s="144"/>
+      <c r="J23" s="144"/>
+      <c r="K23" s="144"/>
+      <c r="L23" s="144">
         <v>10</v>
       </c>
-      <c r="M23" s="125"/>
-      <c r="N23" s="125"/>
-      <c r="O23" s="125"/>
-      <c r="P23" s="125"/>
-      <c r="Q23" s="125"/>
+      <c r="M23" s="144"/>
+      <c r="N23" s="144"/>
+      <c r="O23" s="144"/>
+      <c r="P23" s="144"/>
+      <c r="Q23" s="144"/>
     </row>
     <row r="24" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="122" t="s">
+      <c r="A24" s="151" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="122"/>
-      <c r="C24" s="122"/>
-      <c r="D24" s="181" t="s">
+      <c r="B24" s="151"/>
+      <c r="C24" s="151"/>
+      <c r="D24" s="167" t="s">
         <v>138</v>
       </c>
-      <c r="E24" s="181"/>
-      <c r="F24" s="181"/>
-      <c r="G24" s="181"/>
-      <c r="H24" s="181" t="s">
+      <c r="E24" s="167"/>
+      <c r="F24" s="167"/>
+      <c r="G24" s="167"/>
+      <c r="H24" s="167" t="s">
         <v>138</v>
       </c>
-      <c r="I24" s="181"/>
-      <c r="J24" s="181"/>
-      <c r="K24" s="181"/>
-      <c r="L24" s="125" t="s">
+      <c r="I24" s="167"/>
+      <c r="J24" s="167"/>
+      <c r="K24" s="167"/>
+      <c r="L24" s="144" t="s">
         <v>138</v>
       </c>
-      <c r="M24" s="125"/>
-      <c r="N24" s="125"/>
-      <c r="O24" s="125"/>
-      <c r="P24" s="125"/>
-      <c r="Q24" s="125"/>
+      <c r="M24" s="144"/>
+      <c r="N24" s="144"/>
+      <c r="O24" s="144"/>
+      <c r="P24" s="144"/>
+      <c r="Q24" s="144"/>
     </row>
     <row r="25" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="134" t="s">
+      <c r="A25" s="160" t="s">
         <v>69</v>
       </c>
-      <c r="B25" s="135"/>
-      <c r="C25" s="136"/>
-      <c r="D25" s="127"/>
-      <c r="E25" s="129"/>
-      <c r="F25" s="129"/>
-      <c r="G25" s="128"/>
-      <c r="H25" s="127"/>
-      <c r="I25" s="129"/>
-      <c r="J25" s="129"/>
-      <c r="K25" s="128"/>
-      <c r="L25" s="119"/>
-      <c r="M25" s="120"/>
-      <c r="N25" s="120"/>
-      <c r="O25" s="120"/>
-      <c r="P25" s="120"/>
-      <c r="Q25" s="121"/>
+      <c r="B25" s="161"/>
+      <c r="C25" s="162"/>
+      <c r="D25" s="145"/>
+      <c r="E25" s="147"/>
+      <c r="F25" s="147"/>
+      <c r="G25" s="146"/>
+      <c r="H25" s="145"/>
+      <c r="I25" s="147"/>
+      <c r="J25" s="147"/>
+      <c r="K25" s="146"/>
+      <c r="L25" s="141"/>
+      <c r="M25" s="142"/>
+      <c r="N25" s="142"/>
+      <c r="O25" s="142"/>
+      <c r="P25" s="142"/>
+      <c r="Q25" s="143"/>
     </row>
     <row r="26" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="134" t="s">
+      <c r="A26" s="160" t="s">
         <v>47</v>
       </c>
-      <c r="B26" s="135"/>
-      <c r="C26" s="136"/>
-      <c r="D26" s="127"/>
-      <c r="E26" s="129"/>
-      <c r="F26" s="129"/>
-      <c r="G26" s="128"/>
-      <c r="H26" s="127"/>
-      <c r="I26" s="129"/>
-      <c r="J26" s="129"/>
-      <c r="K26" s="128"/>
-      <c r="L26" s="119"/>
-      <c r="M26" s="120"/>
-      <c r="N26" s="120"/>
-      <c r="O26" s="120"/>
-      <c r="P26" s="120"/>
-      <c r="Q26" s="121"/>
+      <c r="B26" s="161"/>
+      <c r="C26" s="162"/>
+      <c r="D26" s="145"/>
+      <c r="E26" s="147"/>
+      <c r="F26" s="147"/>
+      <c r="G26" s="146"/>
+      <c r="H26" s="145"/>
+      <c r="I26" s="147"/>
+      <c r="J26" s="147"/>
+      <c r="K26" s="146"/>
+      <c r="L26" s="141"/>
+      <c r="M26" s="142"/>
+      <c r="N26" s="142"/>
+      <c r="O26" s="142"/>
+      <c r="P26" s="142"/>
+      <c r="Q26" s="143"/>
     </row>
     <row r="27" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="122" t="s">
+      <c r="A27" s="151" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="122"/>
-      <c r="C27" s="122"/>
-      <c r="D27" s="126"/>
-      <c r="E27" s="126"/>
-      <c r="F27" s="125"/>
-      <c r="G27" s="125"/>
-      <c r="H27" s="127"/>
-      <c r="I27" s="128"/>
-      <c r="J27" s="125"/>
-      <c r="K27" s="125"/>
-      <c r="L27" s="125"/>
-      <c r="M27" s="125"/>
-      <c r="N27" s="125"/>
-      <c r="O27" s="125"/>
-      <c r="P27" s="125"/>
-      <c r="Q27" s="125"/>
+      <c r="B27" s="151"/>
+      <c r="C27" s="151"/>
+      <c r="D27" s="140"/>
+      <c r="E27" s="140"/>
+      <c r="F27" s="144"/>
+      <c r="G27" s="144"/>
+      <c r="H27" s="145"/>
+      <c r="I27" s="146"/>
+      <c r="J27" s="144"/>
+      <c r="K27" s="144"/>
+      <c r="L27" s="144"/>
+      <c r="M27" s="144"/>
+      <c r="N27" s="144"/>
+      <c r="O27" s="144"/>
+      <c r="P27" s="144"/>
+      <c r="Q27" s="144"/>
     </row>
     <row r="28" spans="1:20" ht="11.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="137" t="s">
+      <c r="A28" s="163" t="s">
         <v>40</v>
       </c>
-      <c r="B28" s="138"/>
-      <c r="C28" s="138"/>
-      <c r="D28" s="138"/>
-      <c r="E28" s="138"/>
-      <c r="F28" s="138"/>
-      <c r="G28" s="138"/>
-      <c r="H28" s="138"/>
-      <c r="I28" s="138"/>
-      <c r="J28" s="138"/>
-      <c r="K28" s="138"/>
-      <c r="L28" s="138"/>
-      <c r="M28" s="138"/>
-      <c r="N28" s="138"/>
-      <c r="O28" s="138"/>
-      <c r="P28" s="138"/>
-      <c r="Q28" s="139"/>
+      <c r="B28" s="164"/>
+      <c r="C28" s="164"/>
+      <c r="D28" s="164"/>
+      <c r="E28" s="164"/>
+      <c r="F28" s="164"/>
+      <c r="G28" s="164"/>
+      <c r="H28" s="164"/>
+      <c r="I28" s="164"/>
+      <c r="J28" s="164"/>
+      <c r="K28" s="164"/>
+      <c r="L28" s="164"/>
+      <c r="M28" s="164"/>
+      <c r="N28" s="164"/>
+      <c r="O28" s="164"/>
+      <c r="P28" s="164"/>
+      <c r="Q28" s="165"/>
     </row>
     <row r="29" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="122" t="s">
+      <c r="A29" s="151" t="s">
         <v>48</v>
       </c>
-      <c r="B29" s="122"/>
-      <c r="C29" s="122"/>
-      <c r="D29" s="126"/>
-      <c r="E29" s="126"/>
-      <c r="F29" s="125"/>
-      <c r="G29" s="125"/>
-      <c r="H29" s="127"/>
-      <c r="I29" s="128"/>
-      <c r="J29" s="125"/>
-      <c r="K29" s="125"/>
-      <c r="L29" s="127"/>
-      <c r="M29" s="129"/>
-      <c r="N29" s="128"/>
-      <c r="O29" s="127"/>
-      <c r="P29" s="129"/>
-      <c r="Q29" s="128"/>
-      <c r="S29" s="173" t="s">
+      <c r="B29" s="151"/>
+      <c r="C29" s="151"/>
+      <c r="D29" s="140"/>
+      <c r="E29" s="140"/>
+      <c r="F29" s="144"/>
+      <c r="G29" s="144"/>
+      <c r="H29" s="145"/>
+      <c r="I29" s="146"/>
+      <c r="J29" s="144"/>
+      <c r="K29" s="144"/>
+      <c r="L29" s="145"/>
+      <c r="M29" s="147"/>
+      <c r="N29" s="146"/>
+      <c r="O29" s="145"/>
+      <c r="P29" s="147"/>
+      <c r="Q29" s="146"/>
+      <c r="S29" s="113" t="s">
         <v>90</v>
       </c>
       <c r="T29" s="73">
@@ -3528,26 +3014,26 @@
       </c>
     </row>
     <row r="30" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="122" t="s">
+      <c r="A30" s="151" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="122"/>
-      <c r="C30" s="122"/>
-      <c r="D30" s="126"/>
-      <c r="E30" s="126"/>
-      <c r="F30" s="125"/>
-      <c r="G30" s="125"/>
-      <c r="H30" s="127"/>
-      <c r="I30" s="128"/>
-      <c r="J30" s="125"/>
-      <c r="K30" s="125"/>
-      <c r="L30" s="127"/>
-      <c r="M30" s="129"/>
-      <c r="N30" s="128"/>
-      <c r="O30" s="127"/>
-      <c r="P30" s="129"/>
-      <c r="Q30" s="128"/>
-      <c r="S30" s="159" t="e">
+      <c r="B30" s="151"/>
+      <c r="C30" s="151"/>
+      <c r="D30" s="140"/>
+      <c r="E30" s="140"/>
+      <c r="F30" s="144"/>
+      <c r="G30" s="144"/>
+      <c r="H30" s="145"/>
+      <c r="I30" s="146"/>
+      <c r="J30" s="144"/>
+      <c r="K30" s="144"/>
+      <c r="L30" s="145"/>
+      <c r="M30" s="147"/>
+      <c r="N30" s="146"/>
+      <c r="O30" s="145"/>
+      <c r="P30" s="147"/>
+      <c r="Q30" s="146"/>
+      <c r="S30" s="103" t="e">
         <f>+(D32-(D34-D30))/(D34-D30)*100</f>
         <v>#DIV/0!</v>
       </c>
@@ -3557,26 +3043,26 @@
       </c>
     </row>
     <row r="31" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="122" t="s">
+      <c r="A31" s="151" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="122"/>
-      <c r="C31" s="122"/>
-      <c r="D31" s="126"/>
-      <c r="E31" s="126"/>
-      <c r="F31" s="125"/>
-      <c r="G31" s="125"/>
-      <c r="H31" s="127"/>
-      <c r="I31" s="128"/>
-      <c r="J31" s="125"/>
-      <c r="K31" s="125"/>
-      <c r="L31" s="127"/>
-      <c r="M31" s="129"/>
-      <c r="N31" s="128"/>
-      <c r="O31" s="127"/>
-      <c r="P31" s="129"/>
-      <c r="Q31" s="128"/>
-      <c r="S31" s="159" t="e">
+      <c r="B31" s="151"/>
+      <c r="C31" s="151"/>
+      <c r="D31" s="140"/>
+      <c r="E31" s="140"/>
+      <c r="F31" s="144"/>
+      <c r="G31" s="144"/>
+      <c r="H31" s="145"/>
+      <c r="I31" s="146"/>
+      <c r="J31" s="144"/>
+      <c r="K31" s="144"/>
+      <c r="L31" s="145"/>
+      <c r="M31" s="147"/>
+      <c r="N31" s="146"/>
+      <c r="O31" s="145"/>
+      <c r="P31" s="147"/>
+      <c r="Q31" s="146"/>
+      <c r="S31" s="103" t="e">
         <f>+(H32-(H34-H30))/(H34-H30)*100</f>
         <v>#DIV/0!</v>
       </c>
@@ -3586,44 +3072,44 @@
       </c>
     </row>
     <row r="32" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="140" t="s">
+      <c r="A32" s="166" t="s">
         <v>86</v>
       </c>
-      <c r="B32" s="140"/>
-      <c r="C32" s="140"/>
-      <c r="D32" s="126">
+      <c r="B32" s="166"/>
+      <c r="C32" s="166"/>
+      <c r="D32" s="140">
         <f>+D31-D30</f>
         <v>0</v>
       </c>
-      <c r="E32" s="126"/>
-      <c r="F32" s="126">
+      <c r="E32" s="140"/>
+      <c r="F32" s="140">
         <f>+F31-F30</f>
         <v>0</v>
       </c>
-      <c r="G32" s="126"/>
-      <c r="H32" s="126">
+      <c r="G32" s="140"/>
+      <c r="H32" s="140">
         <f>+H31-H30</f>
         <v>0</v>
       </c>
-      <c r="I32" s="126"/>
-      <c r="J32" s="126">
+      <c r="I32" s="140"/>
+      <c r="J32" s="140">
         <f>+J31-J30</f>
         <v>0</v>
       </c>
-      <c r="K32" s="126"/>
-      <c r="L32" s="119">
+      <c r="K32" s="140"/>
+      <c r="L32" s="141">
         <f>+L31-L30</f>
         <v>0</v>
       </c>
-      <c r="M32" s="120"/>
-      <c r="N32" s="121"/>
-      <c r="O32" s="119">
+      <c r="M32" s="142"/>
+      <c r="N32" s="143"/>
+      <c r="O32" s="141">
         <f>+O31-O30</f>
         <v>0</v>
       </c>
-      <c r="P32" s="120"/>
-      <c r="Q32" s="121"/>
-      <c r="S32" s="159" t="e">
+      <c r="P32" s="142"/>
+      <c r="Q32" s="143"/>
+      <c r="S32" s="103" t="e">
         <f>+(L32-(L34-L30))/(L34-L30)*100</f>
         <v>#DIV/0!</v>
       </c>
@@ -3633,50 +3119,50 @@
       </c>
     </row>
     <row r="33" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="122" t="s">
+      <c r="A33" s="151" t="s">
         <v>51</v>
       </c>
-      <c r="B33" s="122"/>
-      <c r="C33" s="122"/>
-      <c r="D33" s="126"/>
-      <c r="E33" s="126"/>
-      <c r="F33" s="125"/>
-      <c r="G33" s="125"/>
-      <c r="H33" s="127"/>
-      <c r="I33" s="128"/>
-      <c r="J33" s="125"/>
-      <c r="K33" s="125"/>
-      <c r="L33" s="127"/>
-      <c r="M33" s="129"/>
-      <c r="N33" s="128"/>
-      <c r="O33" s="127"/>
-      <c r="P33" s="129"/>
-      <c r="Q33" s="128"/>
+      <c r="B33" s="151"/>
+      <c r="C33" s="151"/>
+      <c r="D33" s="140"/>
+      <c r="E33" s="140"/>
+      <c r="F33" s="144"/>
+      <c r="G33" s="144"/>
+      <c r="H33" s="145"/>
+      <c r="I33" s="146"/>
+      <c r="J33" s="144"/>
+      <c r="K33" s="144"/>
+      <c r="L33" s="145"/>
+      <c r="M33" s="147"/>
+      <c r="N33" s="146"/>
+      <c r="O33" s="145"/>
+      <c r="P33" s="147"/>
+      <c r="Q33" s="146"/>
       <c r="S33" s="73" t="s">
         <v>91</v>
       </c>
     </row>
     <row r="34" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="122" t="s">
+      <c r="A34" s="151" t="s">
         <v>52</v>
       </c>
-      <c r="B34" s="122"/>
-      <c r="C34" s="122"/>
-      <c r="D34" s="126"/>
-      <c r="E34" s="126"/>
-      <c r="F34" s="125"/>
-      <c r="G34" s="125"/>
-      <c r="H34" s="127"/>
-      <c r="I34" s="128"/>
-      <c r="J34" s="125"/>
-      <c r="K34" s="125"/>
-      <c r="L34" s="127"/>
-      <c r="M34" s="129"/>
-      <c r="N34" s="128"/>
-      <c r="O34" s="127"/>
-      <c r="P34" s="129"/>
-      <c r="Q34" s="128"/>
-      <c r="S34" s="159" t="e">
+      <c r="B34" s="151"/>
+      <c r="C34" s="151"/>
+      <c r="D34" s="140"/>
+      <c r="E34" s="140"/>
+      <c r="F34" s="144"/>
+      <c r="G34" s="144"/>
+      <c r="H34" s="145"/>
+      <c r="I34" s="146"/>
+      <c r="J34" s="144"/>
+      <c r="K34" s="144"/>
+      <c r="L34" s="145"/>
+      <c r="M34" s="147"/>
+      <c r="N34" s="146"/>
+      <c r="O34" s="145"/>
+      <c r="P34" s="147"/>
+      <c r="Q34" s="146"/>
+      <c r="S34" s="103" t="e">
         <f>+(F32-(F34-F30))/(F34-F30)*100</f>
         <v>#DIV/0!</v>
       </c>
@@ -3701,7 +3187,7 @@
       <c r="O35" s="95"/>
       <c r="P35" s="95"/>
       <c r="Q35" s="96"/>
-      <c r="S35" s="159" t="e">
+      <c r="S35" s="103" t="e">
         <f>+(J32-(J34-J30))/(J34-J30)*100</f>
         <v>#DIV/0!</v>
       </c>
@@ -3726,69 +3212,69 @@
       <c r="O36" s="26"/>
       <c r="P36" s="26"/>
       <c r="Q36" s="27"/>
-      <c r="S36" s="159" t="e">
+      <c r="S36" s="103" t="e">
         <f>+(O32-(O34-O30))/(O34-O30)*100</f>
         <v>#DIV/0!</v>
       </c>
     </row>
     <row r="37" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="142" t="s">
+      <c r="A37" s="152" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="116" t="s">
+      <c r="B37" s="118" t="s">
         <v>17</v>
       </c>
-      <c r="C37" s="118"/>
+      <c r="C37" s="119"/>
       <c r="D37" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E37" s="116" t="s">
+      <c r="E37" s="118" t="s">
         <v>45</v>
       </c>
-      <c r="F37" s="117"/>
-      <c r="G37" s="117"/>
-      <c r="H37" s="117"/>
-      <c r="I37" s="117"/>
-      <c r="J37" s="118"/>
+      <c r="F37" s="157"/>
+      <c r="G37" s="157"/>
+      <c r="H37" s="157"/>
+      <c r="I37" s="157"/>
+      <c r="J37" s="119"/>
       <c r="K37" s="49"/>
-      <c r="L37" s="157" t="s">
+      <c r="L37" s="138" t="s">
         <v>83</v>
       </c>
-      <c r="M37" s="157"/>
-      <c r="N37" s="157"/>
-      <c r="O37" s="157"/>
-      <c r="P37" s="157"/>
-      <c r="Q37" s="157"/>
+      <c r="M37" s="138"/>
+      <c r="N37" s="138"/>
+      <c r="O37" s="138"/>
+      <c r="P37" s="138"/>
+      <c r="Q37" s="138"/>
     </row>
     <row r="38" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="143"/>
-      <c r="B38" s="145" t="s">
+      <c r="A38" s="153"/>
+      <c r="B38" s="155" t="s">
         <v>70</v>
       </c>
-      <c r="C38" s="145" t="s">
+      <c r="C38" s="155" t="s">
         <v>71</v>
       </c>
       <c r="D38" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E38" s="147" t="s">
+      <c r="E38" s="133" t="s">
         <v>44</v>
       </c>
-      <c r="F38" s="148"/>
-      <c r="G38" s="147" t="s">
+      <c r="F38" s="134"/>
+      <c r="G38" s="133" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="148"/>
-      <c r="I38" s="147" t="s">
+      <c r="H38" s="134"/>
+      <c r="I38" s="133" t="s">
         <v>44</v>
       </c>
-      <c r="J38" s="148"/>
+      <c r="J38" s="134"/>
       <c r="K38" s="49"/>
-      <c r="L38" s="147" t="s">
+      <c r="L38" s="133" t="s">
         <v>19</v>
       </c>
-      <c r="M38" s="148"/>
-      <c r="N38" s="130" t="s">
+      <c r="M38" s="134"/>
+      <c r="N38" s="168" t="s">
         <v>34</v>
       </c>
       <c r="O38" s="73" t="s">
@@ -3800,40 +3286,40 @@
       <c r="Q38" s="73" t="s">
         <v>56</v>
       </c>
-      <c r="S38" s="178" t="s">
+      <c r="S38" s="115" t="s">
         <v>92</v>
       </c>
-      <c r="T38" s="178" t="s">
+      <c r="T38" s="115" t="s">
         <v>111</v>
       </c>
     </row>
     <row r="39" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="144"/>
-      <c r="B39" s="146"/>
-      <c r="C39" s="146"/>
+      <c r="A39" s="154"/>
+      <c r="B39" s="156"/>
+      <c r="C39" s="156"/>
       <c r="D39" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="E39" s="149"/>
-      <c r="F39" s="150"/>
-      <c r="G39" s="149"/>
-      <c r="H39" s="150"/>
-      <c r="I39" s="149"/>
-      <c r="J39" s="150"/>
+      <c r="E39" s="135"/>
+      <c r="F39" s="136"/>
+      <c r="G39" s="135"/>
+      <c r="H39" s="136"/>
+      <c r="I39" s="135"/>
+      <c r="J39" s="136"/>
       <c r="K39" s="49"/>
-      <c r="L39" s="149"/>
-      <c r="M39" s="150"/>
-      <c r="N39" s="131"/>
-      <c r="O39" s="116" t="s">
+      <c r="L39" s="135"/>
+      <c r="M39" s="136"/>
+      <c r="N39" s="169"/>
+      <c r="O39" s="118" t="s">
         <v>73</v>
       </c>
-      <c r="P39" s="117"/>
-      <c r="Q39" s="118"/>
+      <c r="P39" s="157"/>
+      <c r="Q39" s="119"/>
       <c r="R39" s="50"/>
-      <c r="S39" s="184" t="s">
+      <c r="S39" s="117" t="s">
         <v>93</v>
       </c>
-      <c r="T39" s="177" t="s">
+      <c r="T39" s="114" t="s">
         <v>112</v>
       </c>
     </row>
@@ -3848,24 +3334,24 @@
         <v>0</v>
       </c>
       <c r="D40" s="23"/>
-      <c r="E40" s="116"/>
-      <c r="F40" s="118"/>
-      <c r="G40" s="116"/>
-      <c r="H40" s="118"/>
-      <c r="I40" s="116"/>
-      <c r="J40" s="118"/>
+      <c r="E40" s="118"/>
+      <c r="F40" s="119"/>
+      <c r="G40" s="118"/>
+      <c r="H40" s="119"/>
+      <c r="I40" s="118"/>
+      <c r="J40" s="119"/>
       <c r="K40" s="49"/>
-      <c r="L40" s="123"/>
-      <c r="M40" s="124"/>
+      <c r="L40" s="148"/>
+      <c r="M40" s="149"/>
       <c r="N40" s="69"/>
       <c r="O40" s="102"/>
       <c r="P40" s="102"/>
       <c r="Q40" s="70"/>
       <c r="R40" s="50"/>
-      <c r="S40" s="184" t="s">
+      <c r="S40" s="117" t="s">
         <v>94</v>
       </c>
-      <c r="T40" s="177" t="s">
+      <c r="T40" s="114" t="s">
         <v>113</v>
       </c>
     </row>
@@ -3880,24 +3366,24 @@
         <v>0.64</v>
       </c>
       <c r="D41" s="23"/>
-      <c r="E41" s="116"/>
-      <c r="F41" s="118"/>
-      <c r="G41" s="116"/>
-      <c r="H41" s="118"/>
-      <c r="I41" s="116"/>
-      <c r="J41" s="118"/>
+      <c r="E41" s="118"/>
+      <c r="F41" s="119"/>
+      <c r="G41" s="118"/>
+      <c r="H41" s="119"/>
+      <c r="I41" s="118"/>
+      <c r="J41" s="119"/>
       <c r="K41" s="51"/>
-      <c r="L41" s="123"/>
-      <c r="M41" s="124"/>
+      <c r="L41" s="148"/>
+      <c r="M41" s="149"/>
       <c r="N41" s="69"/>
       <c r="O41" s="19"/>
       <c r="P41" s="19"/>
       <c r="Q41" s="19"/>
       <c r="R41" s="52"/>
-      <c r="S41" s="184" t="s">
+      <c r="S41" s="117" t="s">
         <v>95</v>
       </c>
-      <c r="T41" s="177" t="s">
+      <c r="T41" s="114" t="s">
         <v>114</v>
       </c>
     </row>
@@ -3912,24 +3398,24 @@
         <v>1.3</v>
       </c>
       <c r="D42" s="23"/>
-      <c r="E42" s="116"/>
-      <c r="F42" s="118"/>
-      <c r="G42" s="116"/>
-      <c r="H42" s="118"/>
-      <c r="I42" s="116"/>
-      <c r="J42" s="118"/>
+      <c r="E42" s="118"/>
+      <c r="F42" s="119"/>
+      <c r="G42" s="118"/>
+      <c r="H42" s="119"/>
+      <c r="I42" s="118"/>
+      <c r="J42" s="119"/>
       <c r="K42" s="51"/>
-      <c r="L42" s="123"/>
-      <c r="M42" s="124"/>
+      <c r="L42" s="148"/>
+      <c r="M42" s="149"/>
       <c r="N42" s="69"/>
       <c r="O42" s="19"/>
       <c r="P42" s="19"/>
       <c r="Q42" s="19"/>
       <c r="R42" s="52"/>
-      <c r="S42" s="184" t="s">
+      <c r="S42" s="117" t="s">
         <v>96</v>
       </c>
-      <c r="T42" s="177" t="s">
+      <c r="T42" s="114" t="s">
         <v>115</v>
       </c>
     </row>
@@ -3944,78 +3430,78 @@
         <v>1.9</v>
       </c>
       <c r="D43" s="23"/>
-      <c r="E43" s="116"/>
-      <c r="F43" s="118"/>
-      <c r="G43" s="116"/>
-      <c r="H43" s="118"/>
-      <c r="I43" s="116"/>
-      <c r="J43" s="118"/>
+      <c r="E43" s="118"/>
+      <c r="F43" s="119"/>
+      <c r="G43" s="118"/>
+      <c r="H43" s="119"/>
+      <c r="I43" s="118"/>
+      <c r="J43" s="119"/>
       <c r="K43" s="51"/>
-      <c r="L43" s="123"/>
-      <c r="M43" s="124"/>
+      <c r="L43" s="148"/>
+      <c r="M43" s="149"/>
       <c r="N43" s="69"/>
       <c r="O43" s="19"/>
       <c r="P43" s="19"/>
       <c r="Q43" s="19"/>
       <c r="R43" s="52"/>
-      <c r="S43" s="184" t="s">
+      <c r="S43" s="117" t="s">
         <v>97</v>
       </c>
-      <c r="T43" s="177" t="s">
+      <c r="T43" s="114" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="44" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="167" t="s">
+      <c r="A44" s="108" t="s">
         <v>22</v>
       </c>
-      <c r="B44" s="168">
+      <c r="B44" s="109">
         <v>0.1</v>
       </c>
-      <c r="C44" s="169">
+      <c r="C44" s="110">
         <v>2.5</v>
       </c>
-      <c r="D44" s="170">
+      <c r="D44" s="111">
         <v>1000</v>
       </c>
-      <c r="E44" s="164"/>
-      <c r="F44" s="165"/>
-      <c r="G44" s="164"/>
-      <c r="H44" s="165"/>
-      <c r="I44" s="164"/>
-      <c r="J44" s="165"/>
+      <c r="E44" s="131"/>
+      <c r="F44" s="132"/>
+      <c r="G44" s="131"/>
+      <c r="H44" s="132"/>
+      <c r="I44" s="131"/>
+      <c r="J44" s="132"/>
       <c r="K44" s="51"/>
-      <c r="L44" s="123"/>
-      <c r="M44" s="124"/>
+      <c r="L44" s="148"/>
+      <c r="M44" s="149"/>
       <c r="N44" s="69"/>
       <c r="O44" s="19"/>
       <c r="P44" s="19"/>
       <c r="Q44" s="19"/>
       <c r="R44" s="52"/>
-      <c r="S44" s="184" t="s">
+      <c r="S44" s="117" t="s">
         <v>98</v>
       </c>
-      <c r="T44" s="177" t="s">
+      <c r="T44" s="114" t="s">
         <v>117</v>
       </c>
     </row>
     <row r="45" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="166">
+      <c r="A45" s="107">
         <v>0.10416666666666667</v>
       </c>
-      <c r="B45" s="161">
+      <c r="B45" s="104">
         <v>0.125</v>
       </c>
-      <c r="C45" s="162">
+      <c r="C45" s="105">
         <v>3.18</v>
       </c>
-      <c r="D45" s="163"/>
-      <c r="E45" s="164"/>
-      <c r="F45" s="165"/>
-      <c r="G45" s="164"/>
-      <c r="H45" s="165"/>
-      <c r="I45" s="164"/>
-      <c r="J45" s="165"/>
+      <c r="D45" s="106"/>
+      <c r="E45" s="131"/>
+      <c r="F45" s="132"/>
+      <c r="G45" s="131"/>
+      <c r="H45" s="132"/>
+      <c r="I45" s="131"/>
+      <c r="J45" s="132"/>
       <c r="K45" s="51"/>
       <c r="L45" s="40"/>
       <c r="M45" s="40"/>
@@ -4024,120 +3510,120 @@
       <c r="P45" s="40"/>
       <c r="Q45" s="41"/>
       <c r="R45" s="52"/>
-      <c r="S45" s="184" t="s">
+      <c r="S45" s="117" t="s">
         <v>99</v>
       </c>
-      <c r="T45" s="177" t="s">
+      <c r="T45" s="114" t="s">
         <v>118</v>
       </c>
     </row>
     <row r="46" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="166">
+      <c r="A46" s="107">
         <v>0.125</v>
       </c>
-      <c r="B46" s="161">
+      <c r="B46" s="104">
         <v>0.15</v>
       </c>
-      <c r="C46" s="162">
+      <c r="C46" s="105">
         <v>3.8</v>
       </c>
-      <c r="D46" s="163"/>
-      <c r="E46" s="164"/>
-      <c r="F46" s="165"/>
-      <c r="G46" s="164"/>
-      <c r="H46" s="165"/>
-      <c r="I46" s="164"/>
-      <c r="J46" s="165"/>
+      <c r="D46" s="106"/>
+      <c r="E46" s="131"/>
+      <c r="F46" s="132"/>
+      <c r="G46" s="131"/>
+      <c r="H46" s="132"/>
+      <c r="I46" s="131"/>
+      <c r="J46" s="132"/>
       <c r="K46" s="51"/>
-      <c r="L46" s="154" t="s">
+      <c r="L46" s="125" t="s">
         <v>75</v>
       </c>
-      <c r="M46" s="155"/>
-      <c r="N46" s="156"/>
-      <c r="O46" s="141" t="s">
+      <c r="M46" s="126"/>
+      <c r="N46" s="127"/>
+      <c r="O46" s="150" t="s">
         <v>76</v>
       </c>
-      <c r="P46" s="141"/>
-      <c r="Q46" s="141"/>
+      <c r="P46" s="150"/>
+      <c r="Q46" s="150"/>
       <c r="R46" s="52"/>
-      <c r="S46" s="184" t="s">
+      <c r="S46" s="117" t="s">
         <v>100</v>
       </c>
-      <c r="T46" s="177" t="s">
+      <c r="T46" s="114" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="47" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="166">
+      <c r="A47" s="107">
         <v>0.14583333333333334</v>
       </c>
-      <c r="B47" s="161">
+      <c r="B47" s="104">
         <v>0.17499999999999999</v>
       </c>
-      <c r="C47" s="162">
+      <c r="C47" s="105">
         <v>4.45</v>
       </c>
-      <c r="D47" s="163"/>
-      <c r="E47" s="164"/>
-      <c r="F47" s="165"/>
-      <c r="G47" s="164"/>
-      <c r="H47" s="165"/>
-      <c r="I47" s="164"/>
-      <c r="J47" s="165"/>
+      <c r="D47" s="106"/>
+      <c r="E47" s="131"/>
+      <c r="F47" s="132"/>
+      <c r="G47" s="131"/>
+      <c r="H47" s="132"/>
+      <c r="I47" s="131"/>
+      <c r="J47" s="132"/>
       <c r="K47" s="51"/>
-      <c r="L47" s="151" t="s">
+      <c r="L47" s="128" t="s">
         <v>80</v>
       </c>
-      <c r="M47" s="152"/>
-      <c r="N47" s="153"/>
-      <c r="O47" s="172" t="s">
+      <c r="M47" s="129"/>
+      <c r="N47" s="130"/>
+      <c r="O47" s="139" t="s">
         <v>130</v>
       </c>
-      <c r="P47" s="172"/>
-      <c r="Q47" s="172"/>
+      <c r="P47" s="139"/>
+      <c r="Q47" s="139"/>
       <c r="R47" s="52"/>
-      <c r="S47" s="184" t="s">
+      <c r="S47" s="117" t="s">
         <v>101</v>
       </c>
-      <c r="T47" s="177" t="s">
+      <c r="T47" s="114" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="48" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="171">
+      <c r="A48" s="112">
         <v>0.16666666666666666</v>
       </c>
-      <c r="B48" s="168">
+      <c r="B48" s="109">
         <v>0.2</v>
       </c>
-      <c r="C48" s="169">
+      <c r="C48" s="110">
         <v>5.0999999999999996</v>
       </c>
-      <c r="D48" s="170">
+      <c r="D48" s="111">
         <v>1500</v>
       </c>
-      <c r="E48" s="164"/>
-      <c r="F48" s="165"/>
-      <c r="G48" s="164"/>
-      <c r="H48" s="165"/>
-      <c r="I48" s="164"/>
-      <c r="J48" s="165"/>
+      <c r="E48" s="131"/>
+      <c r="F48" s="132"/>
+      <c r="G48" s="131"/>
+      <c r="H48" s="132"/>
+      <c r="I48" s="131"/>
+      <c r="J48" s="132"/>
       <c r="K48" s="51"/>
-      <c r="L48" s="151" t="s">
+      <c r="L48" s="128" t="s">
         <v>81</v>
       </c>
-      <c r="M48" s="152"/>
-      <c r="N48" s="153"/>
-      <c r="O48" s="172" t="s">
+      <c r="M48" s="129"/>
+      <c r="N48" s="130"/>
+      <c r="O48" s="139" t="s">
         <v>131</v>
       </c>
-      <c r="P48" s="172"/>
-      <c r="Q48" s="172"/>
+      <c r="P48" s="139"/>
+      <c r="Q48" s="139"/>
       <c r="R48" s="52"/>
-      <c r="S48" s="184" t="s">
+      <c r="S48" s="117" t="s">
         <v>102</v>
       </c>
-      <c r="T48" s="177" t="s">
+      <c r="T48" s="114" t="s">
         <v>121</v>
       </c>
     </row>
@@ -4152,28 +3638,28 @@
         <v>7.6</v>
       </c>
       <c r="D49" s="23"/>
-      <c r="E49" s="116"/>
-      <c r="F49" s="118"/>
-      <c r="G49" s="116"/>
-      <c r="H49" s="118"/>
-      <c r="I49" s="116"/>
-      <c r="J49" s="118"/>
+      <c r="E49" s="118"/>
+      <c r="F49" s="119"/>
+      <c r="G49" s="118"/>
+      <c r="H49" s="119"/>
+      <c r="I49" s="118"/>
+      <c r="J49" s="119"/>
       <c r="K49" s="53"/>
-      <c r="L49" s="151" t="s">
+      <c r="L49" s="128" t="s">
         <v>82</v>
       </c>
-      <c r="M49" s="152"/>
-      <c r="N49" s="153"/>
-      <c r="O49" s="172" t="s">
+      <c r="M49" s="129"/>
+      <c r="N49" s="130"/>
+      <c r="O49" s="139" t="s">
         <v>132</v>
       </c>
-      <c r="P49" s="172"/>
-      <c r="Q49" s="172"/>
+      <c r="P49" s="139"/>
+      <c r="Q49" s="139"/>
       <c r="R49" s="52"/>
-      <c r="S49" s="184" t="s">
+      <c r="S49" s="117" t="s">
         <v>103</v>
       </c>
-      <c r="T49" s="177" t="s">
+      <c r="T49" s="114" t="s">
         <v>122</v>
       </c>
     </row>
@@ -4188,28 +3674,28 @@
         <v>10</v>
       </c>
       <c r="D50" s="23"/>
-      <c r="E50" s="116"/>
-      <c r="F50" s="118"/>
-      <c r="G50" s="116"/>
-      <c r="H50" s="118"/>
-      <c r="I50" s="116"/>
-      <c r="J50" s="118"/>
+      <c r="E50" s="118"/>
+      <c r="F50" s="119"/>
+      <c r="G50" s="118"/>
+      <c r="H50" s="119"/>
+      <c r="I50" s="118"/>
+      <c r="J50" s="119"/>
       <c r="K50" s="53"/>
       <c r="L50" s="74" t="s">
         <v>78</v>
       </c>
       <c r="M50" s="75"/>
       <c r="N50" s="76"/>
-      <c r="O50" s="172" t="s">
+      <c r="O50" s="139" t="s">
         <v>133</v>
       </c>
-      <c r="P50" s="172"/>
-      <c r="Q50" s="172"/>
+      <c r="P50" s="139"/>
+      <c r="Q50" s="139"/>
       <c r="R50" s="52"/>
-      <c r="S50" s="184" t="s">
+      <c r="S50" s="117" t="s">
         <v>104</v>
       </c>
-      <c r="T50" s="177" t="s">
+      <c r="T50" s="114" t="s">
         <v>123</v>
       </c>
     </row>
@@ -4224,28 +3710,28 @@
         <v>13</v>
       </c>
       <c r="D51" s="23"/>
-      <c r="E51" s="116"/>
-      <c r="F51" s="118"/>
-      <c r="G51" s="116"/>
-      <c r="H51" s="118"/>
-      <c r="I51" s="116"/>
-      <c r="J51" s="118"/>
+      <c r="E51" s="118"/>
+      <c r="F51" s="119"/>
+      <c r="G51" s="118"/>
+      <c r="H51" s="119"/>
+      <c r="I51" s="118"/>
+      <c r="J51" s="119"/>
       <c r="K51" s="54"/>
       <c r="L51" s="74" t="s">
         <v>79</v>
       </c>
       <c r="M51" s="75"/>
       <c r="N51" s="76"/>
-      <c r="O51" s="172" t="s">
+      <c r="O51" s="139" t="s">
         <v>134</v>
       </c>
-      <c r="P51" s="172"/>
-      <c r="Q51" s="172"/>
+      <c r="P51" s="139"/>
+      <c r="Q51" s="139"/>
       <c r="R51" s="52"/>
-      <c r="S51" s="184" t="s">
+      <c r="S51" s="117" t="s">
         <v>105</v>
       </c>
-      <c r="T51" s="177" t="s">
+      <c r="T51" s="114" t="s">
         <v>124</v>
       </c>
     </row>
@@ -4261,20 +3747,20 @@
       <c r="I52" s="57"/>
       <c r="J52" s="28"/>
       <c r="K52" s="14"/>
-      <c r="L52" s="151" t="s">
+      <c r="L52" s="128" t="s">
         <v>77</v>
       </c>
-      <c r="M52" s="152"/>
-      <c r="N52" s="153"/>
-      <c r="O52" s="172" t="s">
+      <c r="M52" s="129"/>
+      <c r="N52" s="130"/>
+      <c r="O52" s="139" t="s">
         <v>135</v>
       </c>
-      <c r="P52" s="172"/>
-      <c r="Q52" s="172"/>
-      <c r="S52" s="184" t="s">
+      <c r="P52" s="139"/>
+      <c r="Q52" s="139"/>
+      <c r="S52" s="117" t="s">
         <v>106</v>
       </c>
-      <c r="T52" s="177" t="s">
+      <c r="T52" s="114" t="s">
         <v>125</v>
       </c>
     </row>
@@ -4285,27 +3771,27 @@
       <c r="B53" s="59"/>
       <c r="C53" s="59"/>
       <c r="D53" s="60"/>
-      <c r="E53" s="116"/>
-      <c r="F53" s="118"/>
-      <c r="G53" s="116"/>
-      <c r="H53" s="118"/>
-      <c r="I53" s="182"/>
-      <c r="J53" s="183"/>
+      <c r="E53" s="118"/>
+      <c r="F53" s="119"/>
+      <c r="G53" s="118"/>
+      <c r="H53" s="119"/>
+      <c r="I53" s="120"/>
+      <c r="J53" s="121"/>
       <c r="K53" s="61"/>
-      <c r="L53" s="151" t="s">
+      <c r="L53" s="128" t="s">
         <v>84</v>
       </c>
-      <c r="M53" s="152"/>
-      <c r="N53" s="153"/>
-      <c r="O53" s="172" t="s">
+      <c r="M53" s="129"/>
+      <c r="N53" s="130"/>
+      <c r="O53" s="139" t="s">
         <v>136</v>
       </c>
-      <c r="P53" s="172"/>
-      <c r="Q53" s="172"/>
-      <c r="S53" s="184" t="s">
+      <c r="P53" s="139"/>
+      <c r="Q53" s="139"/>
+      <c r="S53" s="117" t="s">
         <v>107</v>
       </c>
-      <c r="T53" s="177" t="s">
+      <c r="T53" s="114" t="s">
         <v>126</v>
       </c>
     </row>
@@ -4327,10 +3813,10 @@
       <c r="O54" s="14"/>
       <c r="P54" s="14"/>
       <c r="Q54" s="14"/>
-      <c r="S54" s="184" t="s">
+      <c r="S54" s="117" t="s">
         <v>108</v>
       </c>
-      <c r="T54" s="177" t="s">
+      <c r="T54" s="114" t="s">
         <v>127</v>
       </c>
     </row>
@@ -4352,10 +3838,10 @@
       <c r="O55" s="28"/>
       <c r="P55" s="28"/>
       <c r="Q55" s="29"/>
-      <c r="S55" s="184" t="s">
+      <c r="S55" s="117" t="s">
         <v>109</v>
       </c>
-      <c r="T55" s="177" t="s">
+      <c r="T55" s="114" t="s">
         <v>128</v>
       </c>
     </row>
@@ -4379,10 +3865,10 @@
       <c r="O56" s="63"/>
       <c r="P56" s="63"/>
       <c r="Q56" s="66"/>
-      <c r="S56" s="184" t="s">
+      <c r="S56" s="117" t="s">
         <v>110</v>
       </c>
-      <c r="T56" s="177" t="s">
+      <c r="T56" s="114" t="s">
         <v>129</v>
       </c>
     </row>
@@ -4448,25 +3934,25 @@
     </row>
     <row r="62" spans="1:20" ht="7.2" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="63" spans="1:20" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="109" t="s">
+      <c r="A63" s="176" t="s">
         <v>85</v>
       </c>
-      <c r="B63" s="109"/>
-      <c r="C63" s="109"/>
-      <c r="D63" s="109"/>
-      <c r="E63" s="109"/>
-      <c r="F63" s="109"/>
-      <c r="G63" s="109"/>
-      <c r="H63" s="109"/>
-      <c r="I63" s="109"/>
-      <c r="J63" s="109"/>
-      <c r="K63" s="109"/>
-      <c r="L63" s="109"/>
-      <c r="M63" s="109"/>
-      <c r="N63" s="109"/>
-      <c r="O63" s="109"/>
-      <c r="P63" s="109"/>
-      <c r="Q63" s="109"/>
+      <c r="B63" s="176"/>
+      <c r="C63" s="176"/>
+      <c r="D63" s="176"/>
+      <c r="E63" s="176"/>
+      <c r="F63" s="176"/>
+      <c r="G63" s="176"/>
+      <c r="H63" s="176"/>
+      <c r="I63" s="176"/>
+      <c r="J63" s="176"/>
+      <c r="K63" s="176"/>
+      <c r="L63" s="176"/>
+      <c r="M63" s="176"/>
+      <c r="N63" s="176"/>
+      <c r="O63" s="176"/>
+      <c r="P63" s="176"/>
+      <c r="Q63" s="176"/>
     </row>
     <row r="64" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="65" ht="15.9" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -4475,7 +3961,144 @@
     <protectedRange sqref="C10 C13" name="Rango3_3_1_1_1_1_1_1_1_1"/>
     <protectedRange sqref="C8:C9" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
-  <mergeCells count="160">
+  <mergeCells count="161">
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D2:Q2"/>
+    <mergeCell ref="D3:Q3"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="L24:Q24"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="L23:Q23"/>
+    <mergeCell ref="A63:Q63"/>
+    <mergeCell ref="A11:Q11"/>
+    <mergeCell ref="A12:Q12"/>
+    <mergeCell ref="O39:Q39"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="L21:Q21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="L25:Q25"/>
+    <mergeCell ref="L26:Q26"/>
+    <mergeCell ref="L22:N22"/>
+    <mergeCell ref="O22:Q22"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="L44:M44"/>
+    <mergeCell ref="O30:Q30"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="H26:K26"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="O33:Q33"/>
+    <mergeCell ref="N38:N39"/>
+    <mergeCell ref="O27:Q27"/>
+    <mergeCell ref="O29:Q29"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="E20:Q20"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="O31:Q31"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="G49:H49"/>
+    <mergeCell ref="G50:H50"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="A37:A39"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="E37:J37"/>
+    <mergeCell ref="E38:F39"/>
+    <mergeCell ref="G38:H39"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="L32:N32"/>
+    <mergeCell ref="O32:Q32"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="O34:Q34"/>
+    <mergeCell ref="I38:J39"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="O50:Q50"/>
+    <mergeCell ref="L53:N53"/>
+    <mergeCell ref="O53:Q53"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="O47:Q47"/>
+    <mergeCell ref="O48:Q48"/>
+    <mergeCell ref="O49:Q49"/>
+    <mergeCell ref="O52:Q52"/>
+    <mergeCell ref="O51:Q51"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="O46:Q46"/>
+    <mergeCell ref="G48:H48"/>
     <mergeCell ref="E53:F53"/>
     <mergeCell ref="G53:H53"/>
     <mergeCell ref="I53:J53"/>
@@ -4500,142 +4123,6 @@
     <mergeCell ref="E50:F50"/>
     <mergeCell ref="E43:F43"/>
     <mergeCell ref="E44:F44"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="O50:Q50"/>
-    <mergeCell ref="L53:N53"/>
-    <mergeCell ref="O53:Q53"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="O47:Q47"/>
-    <mergeCell ref="O48:Q48"/>
-    <mergeCell ref="O49:Q49"/>
-    <mergeCell ref="O52:Q52"/>
-    <mergeCell ref="O51:Q51"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="L32:N32"/>
-    <mergeCell ref="O32:Q32"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="L34:N34"/>
-    <mergeCell ref="O34:Q34"/>
-    <mergeCell ref="I38:J39"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="L41:M41"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="L43:M43"/>
-    <mergeCell ref="O46:Q46"/>
-    <mergeCell ref="G48:H48"/>
-    <mergeCell ref="G49:H49"/>
-    <mergeCell ref="G50:H50"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="A37:A39"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="E37:J37"/>
-    <mergeCell ref="E38:F39"/>
-    <mergeCell ref="G38:H39"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="E20:Q20"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="A28:Q28"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="L44:M44"/>
-    <mergeCell ref="O30:Q30"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="H25:K25"/>
-    <mergeCell ref="H26:K26"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="O33:Q33"/>
-    <mergeCell ref="N38:N39"/>
-    <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="O29:Q29"/>
-    <mergeCell ref="D2:Q2"/>
-    <mergeCell ref="D3:Q3"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="L24:Q24"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="L23:Q23"/>
-    <mergeCell ref="A63:Q63"/>
-    <mergeCell ref="A11:Q11"/>
-    <mergeCell ref="A12:Q12"/>
-    <mergeCell ref="O39:Q39"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="L21:Q21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="L25:Q25"/>
-    <mergeCell ref="L26:Q26"/>
-    <mergeCell ref="L22:N22"/>
-    <mergeCell ref="O22:Q22"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="D21:G21"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.39370078740157483" top="0.78740157480314965" bottom="0" header="0" footer="0"/>
@@ -4661,10 +4148,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="158" t="s">
+      <c r="A2" s="184" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="158"/>
+      <c r="B2" s="184"/>
       <c r="C2" s="5" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
fix(cbr): ajustar exportacion, footer y template ASTM
</commit_message>
<xml_diff>
--- a/app/templates/Temp_CBR_ASTM.xlsx
+++ b/app/templates/Temp_CBR_ASTM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{125A63E1-FFBC-475F-B49D-22BDB4BA5FA7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F28A87B-B48B-4603-8C74-0F2E8B7E76D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="103">
   <si>
     <t>FC</t>
   </si>
@@ -362,126 +362,6 @@
     <t>Versión: 02 (11-11-2024)</t>
   </si>
   <si>
-    <t>C.H. SIN SATURAR</t>
-  </si>
-  <si>
-    <t>C.H. SATURADO</t>
-  </si>
-  <si>
-    <t>CODIGOS</t>
-  </si>
-  <si>
-    <t>INS-173</t>
-  </si>
-  <si>
-    <t>INS-174</t>
-  </si>
-  <si>
-    <t>INS-175</t>
-  </si>
-  <si>
-    <t>INS-030</t>
-  </si>
-  <si>
-    <t>INS-031</t>
-  </si>
-  <si>
-    <t>INS-032</t>
-  </si>
-  <si>
-    <t>INS-027</t>
-  </si>
-  <si>
-    <t>INS-028</t>
-  </si>
-  <si>
-    <t>INS-029</t>
-  </si>
-  <si>
-    <t>INS-033</t>
-  </si>
-  <si>
-    <t>INS-034</t>
-  </si>
-  <si>
-    <t>INS-035</t>
-  </si>
-  <si>
-    <t>INS-200</t>
-  </si>
-  <si>
-    <t>INS-201</t>
-  </si>
-  <si>
-    <t>INS-202</t>
-  </si>
-  <si>
-    <t>INS-203</t>
-  </si>
-  <si>
-    <t>INS-204</t>
-  </si>
-  <si>
-    <t>INS-205</t>
-  </si>
-  <si>
-    <t>EQUIPOS UTILIZADOS</t>
-  </si>
-  <si>
-    <t>MOLDE 11</t>
-  </si>
-  <si>
-    <t>MOLDE 12</t>
-  </si>
-  <si>
-    <t>MOLDE 13</t>
-  </si>
-  <si>
-    <t>MOLDE 1</t>
-  </si>
-  <si>
-    <t>MOLDE 2</t>
-  </si>
-  <si>
-    <t>MOLDE 3</t>
-  </si>
-  <si>
-    <t>MOLDE 4</t>
-  </si>
-  <si>
-    <t>MOLDE 5</t>
-  </si>
-  <si>
-    <t>MOLDE 6</t>
-  </si>
-  <si>
-    <t>MOLDE 7</t>
-  </si>
-  <si>
-    <t>MOLDE 8</t>
-  </si>
-  <si>
-    <t>MOLDE 9</t>
-  </si>
-  <si>
-    <t>MOLDE A</t>
-  </si>
-  <si>
-    <t>MOLDE B</t>
-  </si>
-  <si>
-    <t>MOLDE C</t>
-  </si>
-  <si>
-    <t>MOLDE E</t>
-  </si>
-  <si>
-    <t>MOLDE H</t>
-  </si>
-  <si>
-    <t>MOLDE L</t>
-  </si>
-  <si>
     <t>EQP-0026</t>
   </si>
   <si>
@@ -531,17 +411,10 @@
     <numFmt numFmtId="166" formatCode="&quot;FORMATO F-LEM-P-SU-11.01&quot;"/>
     <numFmt numFmtId="167" formatCode="0.000"/>
   </numFmts>
-  <fonts count="20" x14ac:knownFonts="1">
+  <fonts count="19" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
     <font>
       <sz val="10"/>
@@ -651,7 +524,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -670,14 +543,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="8" tint="0.39997558519241921"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="17">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -854,638 +721,609 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF000000"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF000000"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF000000"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="top"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="195">
+  <cellXfs count="190">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="2" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="10" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="10" fontId="5" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="16" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="9" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="16" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="9" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="7" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="17" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="8" fillId="2" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="3" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="4" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="17" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="1" fontId="12" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="13" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="1" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="1" fontId="14" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="right" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyProtection="1">
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="4" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="7" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="6" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="4" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="8" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="11" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="20" fontId="11" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="7" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="10" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="20" fontId="10" fillId="3" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="4" borderId="16" xfId="5" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="8" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="8" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="16" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2408,43 +2246,43 @@
       <c r="A2" s="81"/>
       <c r="B2" s="82"/>
       <c r="C2" s="83"/>
-      <c r="D2" s="170" t="s">
+      <c r="D2" s="123" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="171"/>
-      <c r="F2" s="171"/>
-      <c r="G2" s="171"/>
-      <c r="H2" s="171"/>
-      <c r="I2" s="171"/>
-      <c r="J2" s="171"/>
-      <c r="K2" s="171"/>
-      <c r="L2" s="171"/>
-      <c r="M2" s="171"/>
-      <c r="N2" s="171"/>
-      <c r="O2" s="171"/>
-      <c r="P2" s="171"/>
-      <c r="Q2" s="172"/>
+      <c r="E2" s="124"/>
+      <c r="F2" s="124"/>
+      <c r="G2" s="124"/>
+      <c r="H2" s="124"/>
+      <c r="I2" s="124"/>
+      <c r="J2" s="124"/>
+      <c r="K2" s="124"/>
+      <c r="L2" s="124"/>
+      <c r="M2" s="124"/>
+      <c r="N2" s="124"/>
+      <c r="O2" s="124"/>
+      <c r="P2" s="124"/>
+      <c r="Q2" s="125"/>
     </row>
     <row r="3" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="81"/>
       <c r="B3" s="82"/>
       <c r="C3" s="83"/>
-      <c r="D3" s="173" t="s">
+      <c r="D3" s="126" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="174"/>
-      <c r="F3" s="174"/>
-      <c r="G3" s="174"/>
-      <c r="H3" s="174"/>
-      <c r="I3" s="174"/>
-      <c r="J3" s="174"/>
-      <c r="K3" s="174"/>
-      <c r="L3" s="174"/>
-      <c r="M3" s="174"/>
-      <c r="N3" s="174"/>
-      <c r="O3" s="174"/>
-      <c r="P3" s="174"/>
-      <c r="Q3" s="175"/>
+      <c r="E3" s="127"/>
+      <c r="F3" s="127"/>
+      <c r="G3" s="127"/>
+      <c r="H3" s="127"/>
+      <c r="I3" s="127"/>
+      <c r="J3" s="127"/>
+      <c r="K3" s="127"/>
+      <c r="L3" s="127"/>
+      <c r="M3" s="127"/>
+      <c r="N3" s="127"/>
+      <c r="O3" s="127"/>
+      <c r="P3" s="127"/>
+      <c r="Q3" s="128"/>
     </row>
     <row r="4" spans="1:17" ht="3" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="81"/>
@@ -2523,23 +2361,23 @@
     <row r="8" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="32"/>
       <c r="C8" s="32"/>
-      <c r="D8" s="190" t="s">
-        <v>139</v>
-      </c>
-      <c r="E8" s="191"/>
-      <c r="F8" s="189" t="s">
-        <v>140</v>
-      </c>
-      <c r="G8" s="185"/>
-      <c r="H8" s="186" t="s">
-        <v>141</v>
-      </c>
-      <c r="I8" s="187"/>
-      <c r="J8" s="185"/>
-      <c r="K8" s="186" t="s">
-        <v>142</v>
-      </c>
-      <c r="L8" s="188"/>
+      <c r="D8" s="121" t="s">
+        <v>99</v>
+      </c>
+      <c r="E8" s="122"/>
+      <c r="F8" s="117" t="s">
+        <v>100</v>
+      </c>
+      <c r="G8" s="113"/>
+      <c r="H8" s="114" t="s">
+        <v>101</v>
+      </c>
+      <c r="I8" s="115"/>
+      <c r="J8" s="113"/>
+      <c r="K8" s="114" t="s">
+        <v>102</v>
+      </c>
+      <c r="L8" s="116"/>
       <c r="M8" s="60"/>
       <c r="N8" s="15"/>
       <c r="O8" s="15"/>
@@ -2548,16 +2386,16 @@
       <c r="A9" s="32"/>
       <c r="B9" s="32"/>
       <c r="C9" s="32"/>
-      <c r="D9" s="185"/>
-      <c r="E9" s="187"/>
-      <c r="F9" s="192"/>
-      <c r="G9" s="185"/>
-      <c r="H9" s="193"/>
-      <c r="I9" s="187"/>
-      <c r="J9" s="185"/>
+      <c r="D9" s="113"/>
+      <c r="E9" s="115"/>
+      <c r="F9" s="118"/>
+      <c r="G9" s="113"/>
+      <c r="H9" s="119"/>
+      <c r="I9" s="115"/>
+      <c r="J9" s="113"/>
       <c r="K9" s="59"/>
       <c r="L9" s="59"/>
-      <c r="M9" s="194"/>
+      <c r="M9" s="120"/>
       <c r="N9" s="14"/>
       <c r="O9" s="14"/>
     </row>
@@ -2579,46 +2417,46 @@
       <c r="O10" s="35"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="177" t="s">
+      <c r="A11" s="132" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="178"/>
-      <c r="C11" s="178"/>
-      <c r="D11" s="178"/>
-      <c r="E11" s="178"/>
-      <c r="F11" s="178"/>
-      <c r="G11" s="178"/>
-      <c r="H11" s="178"/>
-      <c r="I11" s="178"/>
-      <c r="J11" s="178"/>
-      <c r="K11" s="178"/>
-      <c r="L11" s="178"/>
-      <c r="M11" s="178"/>
-      <c r="N11" s="178"/>
-      <c r="O11" s="178"/>
-      <c r="P11" s="178"/>
-      <c r="Q11" s="179"/>
+      <c r="B11" s="133"/>
+      <c r="C11" s="133"/>
+      <c r="D11" s="133"/>
+      <c r="E11" s="133"/>
+      <c r="F11" s="133"/>
+      <c r="G11" s="133"/>
+      <c r="H11" s="133"/>
+      <c r="I11" s="133"/>
+      <c r="J11" s="133"/>
+      <c r="K11" s="133"/>
+      <c r="L11" s="133"/>
+      <c r="M11" s="133"/>
+      <c r="N11" s="133"/>
+      <c r="O11" s="133"/>
+      <c r="P11" s="133"/>
+      <c r="Q11" s="134"/>
     </row>
     <row r="12" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="180" t="s">
+      <c r="A12" s="135" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="181"/>
-      <c r="C12" s="181"/>
-      <c r="D12" s="181"/>
-      <c r="E12" s="181"/>
-      <c r="F12" s="181"/>
-      <c r="G12" s="181"/>
-      <c r="H12" s="181"/>
-      <c r="I12" s="181"/>
-      <c r="J12" s="181"/>
-      <c r="K12" s="181"/>
-      <c r="L12" s="181"/>
-      <c r="M12" s="181"/>
-      <c r="N12" s="181"/>
-      <c r="O12" s="181"/>
-      <c r="P12" s="181"/>
-      <c r="Q12" s="182"/>
+      <c r="B12" s="136"/>
+      <c r="C12" s="136"/>
+      <c r="D12" s="136"/>
+      <c r="E12" s="136"/>
+      <c r="F12" s="136"/>
+      <c r="G12" s="136"/>
+      <c r="H12" s="136"/>
+      <c r="I12" s="136"/>
+      <c r="J12" s="136"/>
+      <c r="K12" s="136"/>
+      <c r="L12" s="136"/>
+      <c r="M12" s="136"/>
+      <c r="N12" s="136"/>
+      <c r="O12" s="136"/>
+      <c r="P12" s="136"/>
+      <c r="Q12" s="137"/>
     </row>
     <row r="13" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="36"/>
@@ -2646,8 +2484,8 @@
       <c r="B14" s="14"/>
       <c r="C14" s="43"/>
       <c r="D14" s="14"/>
-      <c r="E14" s="124"/>
-      <c r="F14" s="124"/>
+      <c r="E14" s="183"/>
+      <c r="F14" s="183"/>
       <c r="G14" s="87" t="s">
         <v>23</v>
       </c>
@@ -2657,8 +2495,8 @@
       <c r="N14" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="O14" s="122"/>
-      <c r="P14" s="123"/>
+      <c r="O14" s="181"/>
+      <c r="P14" s="182"/>
       <c r="Q14" s="27"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2668,8 +2506,8 @@
       <c r="B15" s="14"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
-      <c r="E15" s="124"/>
-      <c r="F15" s="124"/>
+      <c r="E15" s="183"/>
+      <c r="F15" s="183"/>
       <c r="G15" s="87" t="s">
         <v>25</v>
       </c>
@@ -2679,8 +2517,8 @@
       <c r="N15" s="45" t="s">
         <v>68</v>
       </c>
-      <c r="O15" s="122"/>
-      <c r="P15" s="123"/>
+      <c r="O15" s="181"/>
+      <c r="P15" s="182"/>
       <c r="Q15" s="27"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2692,7 +2530,7 @@
       <c r="D16" s="43" t="s">
         <v>60</v>
       </c>
-      <c r="E16" s="116"/>
+      <c r="E16" s="112"/>
       <c r="G16" s="72"/>
       <c r="H16" s="14"/>
       <c r="K16" s="14"/>
@@ -2700,8 +2538,8 @@
       <c r="N16" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="O16" s="122"/>
-      <c r="P16" s="123"/>
+      <c r="O16" s="181"/>
+      <c r="P16" s="182"/>
       <c r="Q16" s="27"/>
     </row>
     <row r="17" spans="1:20" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
@@ -2711,7 +2549,7 @@
       <c r="D17" s="88" t="s">
         <v>61</v>
       </c>
-      <c r="E17" s="106"/>
+      <c r="E17" s="105"/>
       <c r="F17" s="14"/>
       <c r="H17" s="14"/>
       <c r="K17" s="14"/>
@@ -2719,8 +2557,8 @@
       <c r="N17" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="O17" s="122"/>
-      <c r="P17" s="123"/>
+      <c r="O17" s="181"/>
+      <c r="P17" s="182"/>
       <c r="Q17" s="27"/>
     </row>
     <row r="18" spans="1:20" ht="6" customHeight="1" x14ac:dyDescent="0.2">
@@ -2751,8 +2589,8 @@
       <c r="D19" s="90"/>
       <c r="E19" s="98"/>
       <c r="F19" s="98"/>
-      <c r="G19" s="137"/>
-      <c r="H19" s="137"/>
+      <c r="G19" s="187"/>
+      <c r="H19" s="187"/>
       <c r="I19" s="91"/>
       <c r="J19" s="91"/>
       <c r="K19" s="90"/>
@@ -2770,404 +2608,385 @@
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
       <c r="D20" s="48"/>
-      <c r="E20" s="158" t="s">
+      <c r="E20" s="154" t="s">
         <v>36</v>
       </c>
-      <c r="F20" s="158"/>
-      <c r="G20" s="158"/>
-      <c r="H20" s="158"/>
-      <c r="I20" s="158"/>
-      <c r="J20" s="158"/>
-      <c r="K20" s="158"/>
-      <c r="L20" s="158"/>
-      <c r="M20" s="158"/>
-      <c r="N20" s="158"/>
-      <c r="O20" s="158"/>
-      <c r="P20" s="158"/>
-      <c r="Q20" s="159"/>
+      <c r="F20" s="154"/>
+      <c r="G20" s="154"/>
+      <c r="H20" s="154"/>
+      <c r="I20" s="154"/>
+      <c r="J20" s="154"/>
+      <c r="K20" s="154"/>
+      <c r="L20" s="154"/>
+      <c r="M20" s="154"/>
+      <c r="N20" s="154"/>
+      <c r="O20" s="154"/>
+      <c r="P20" s="154"/>
+      <c r="Q20" s="155"/>
     </row>
     <row r="21" spans="1:20" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="183" t="s">
+      <c r="A21" s="141" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="183"/>
-      <c r="C21" s="183"/>
-      <c r="D21" s="183" t="s">
+      <c r="B21" s="141"/>
+      <c r="C21" s="141"/>
+      <c r="D21" s="141" t="s">
         <v>27</v>
       </c>
-      <c r="E21" s="183"/>
-      <c r="F21" s="183"/>
-      <c r="G21" s="183"/>
-      <c r="H21" s="183" t="s">
+      <c r="E21" s="141"/>
+      <c r="F21" s="141"/>
+      <c r="G21" s="141"/>
+      <c r="H21" s="141" t="s">
         <v>28</v>
       </c>
-      <c r="I21" s="183"/>
-      <c r="J21" s="183"/>
-      <c r="K21" s="183"/>
-      <c r="L21" s="183" t="s">
+      <c r="I21" s="141"/>
+      <c r="J21" s="141"/>
+      <c r="K21" s="141"/>
+      <c r="L21" s="141" t="s">
         <v>29</v>
       </c>
-      <c r="M21" s="183"/>
-      <c r="N21" s="183"/>
-      <c r="O21" s="183"/>
-      <c r="P21" s="183"/>
-      <c r="Q21" s="183"/>
+      <c r="M21" s="141"/>
+      <c r="N21" s="141"/>
+      <c r="O21" s="141"/>
+      <c r="P21" s="141"/>
+      <c r="Q21" s="141"/>
       <c r="R21" s="13"/>
     </row>
     <row r="22" spans="1:20" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="183" t="s">
+      <c r="A22" s="141" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="183"/>
-      <c r="C22" s="183"/>
-      <c r="D22" s="183" t="s">
+      <c r="B22" s="141"/>
+      <c r="C22" s="141"/>
+      <c r="D22" s="141" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="183"/>
-      <c r="F22" s="183" t="s">
+      <c r="E22" s="141"/>
+      <c r="F22" s="141" t="s">
         <v>32</v>
       </c>
-      <c r="G22" s="183"/>
-      <c r="H22" s="183" t="s">
+      <c r="G22" s="141"/>
+      <c r="H22" s="141" t="s">
         <v>31</v>
       </c>
-      <c r="I22" s="183"/>
-      <c r="J22" s="183" t="s">
+      <c r="I22" s="141"/>
+      <c r="J22" s="141" t="s">
         <v>32</v>
       </c>
-      <c r="K22" s="183"/>
-      <c r="L22" s="183" t="s">
+      <c r="K22" s="141"/>
+      <c r="L22" s="141" t="s">
         <v>31</v>
       </c>
-      <c r="M22" s="183"/>
-      <c r="N22" s="183"/>
-      <c r="O22" s="183" t="s">
+      <c r="M22" s="141"/>
+      <c r="N22" s="141"/>
+      <c r="O22" s="141" t="s">
         <v>32</v>
       </c>
-      <c r="P22" s="183"/>
-      <c r="Q22" s="183"/>
+      <c r="P22" s="141"/>
+      <c r="Q22" s="141"/>
       <c r="R22" s="13"/>
     </row>
     <row r="23" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="151" t="s">
+      <c r="A23" s="145" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="151"/>
-      <c r="C23" s="151"/>
-      <c r="D23" s="167" t="s">
-        <v>137</v>
-      </c>
-      <c r="E23" s="167"/>
-      <c r="F23" s="167"/>
-      <c r="G23" s="167"/>
-      <c r="H23" s="144">
+      <c r="B23" s="145"/>
+      <c r="C23" s="145"/>
+      <c r="D23" s="129" t="s">
+        <v>97</v>
+      </c>
+      <c r="E23" s="129"/>
+      <c r="F23" s="129"/>
+      <c r="G23" s="129"/>
+      <c r="H23" s="130">
         <v>25</v>
       </c>
-      <c r="I23" s="144"/>
-      <c r="J23" s="144"/>
-      <c r="K23" s="144"/>
-      <c r="L23" s="144">
+      <c r="I23" s="130"/>
+      <c r="J23" s="130"/>
+      <c r="K23" s="130"/>
+      <c r="L23" s="130">
         <v>10</v>
       </c>
-      <c r="M23" s="144"/>
-      <c r="N23" s="144"/>
-      <c r="O23" s="144"/>
-      <c r="P23" s="144"/>
-      <c r="Q23" s="144"/>
+      <c r="M23" s="130"/>
+      <c r="N23" s="130"/>
+      <c r="O23" s="130"/>
+      <c r="P23" s="130"/>
+      <c r="Q23" s="130"/>
     </row>
     <row r="24" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="151" t="s">
+      <c r="A24" s="145" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="151"/>
-      <c r="C24" s="151"/>
-      <c r="D24" s="167" t="s">
-        <v>138</v>
-      </c>
-      <c r="E24" s="167"/>
-      <c r="F24" s="167"/>
-      <c r="G24" s="167"/>
-      <c r="H24" s="167" t="s">
-        <v>138</v>
-      </c>
-      <c r="I24" s="167"/>
-      <c r="J24" s="167"/>
-      <c r="K24" s="167"/>
-      <c r="L24" s="144" t="s">
-        <v>138</v>
-      </c>
-      <c r="M24" s="144"/>
-      <c r="N24" s="144"/>
-      <c r="O24" s="144"/>
-      <c r="P24" s="144"/>
-      <c r="Q24" s="144"/>
+      <c r="B24" s="145"/>
+      <c r="C24" s="145"/>
+      <c r="D24" s="129" t="s">
+        <v>98</v>
+      </c>
+      <c r="E24" s="129"/>
+      <c r="F24" s="129"/>
+      <c r="G24" s="129"/>
+      <c r="H24" s="129" t="s">
+        <v>98</v>
+      </c>
+      <c r="I24" s="129"/>
+      <c r="J24" s="129"/>
+      <c r="K24" s="129"/>
+      <c r="L24" s="130" t="s">
+        <v>98</v>
+      </c>
+      <c r="M24" s="130"/>
+      <c r="N24" s="130"/>
+      <c r="O24" s="130"/>
+      <c r="P24" s="130"/>
+      <c r="Q24" s="130"/>
     </row>
     <row r="25" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="160" t="s">
+      <c r="A25" s="156" t="s">
         <v>69</v>
       </c>
-      <c r="B25" s="161"/>
-      <c r="C25" s="162"/>
-      <c r="D25" s="145"/>
-      <c r="E25" s="147"/>
-      <c r="F25" s="147"/>
-      <c r="G25" s="146"/>
-      <c r="H25" s="145"/>
-      <c r="I25" s="147"/>
-      <c r="J25" s="147"/>
-      <c r="K25" s="146"/>
-      <c r="L25" s="141"/>
-      <c r="M25" s="142"/>
-      <c r="N25" s="142"/>
-      <c r="O25" s="142"/>
-      <c r="P25" s="142"/>
-      <c r="Q25" s="143"/>
-    </row>
-    <row r="26" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="160" t="s">
+      <c r="B25" s="157"/>
+      <c r="C25" s="158"/>
+      <c r="D25" s="148"/>
+      <c r="E25" s="149"/>
+      <c r="F25" s="149"/>
+      <c r="G25" s="150"/>
+      <c r="H25" s="148"/>
+      <c r="I25" s="149"/>
+      <c r="J25" s="149"/>
+      <c r="K25" s="150"/>
+      <c r="L25" s="142"/>
+      <c r="M25" s="143"/>
+      <c r="N25" s="143"/>
+      <c r="O25" s="143"/>
+      <c r="P25" s="143"/>
+      <c r="Q25" s="144"/>
+    </row>
+    <row r="26" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A26" s="156" t="s">
         <v>47</v>
       </c>
-      <c r="B26" s="161"/>
-      <c r="C26" s="162"/>
-      <c r="D26" s="145"/>
-      <c r="E26" s="147"/>
-      <c r="F26" s="147"/>
-      <c r="G26" s="146"/>
-      <c r="H26" s="145"/>
-      <c r="I26" s="147"/>
-      <c r="J26" s="147"/>
-      <c r="K26" s="146"/>
-      <c r="L26" s="141"/>
-      <c r="M26" s="142"/>
-      <c r="N26" s="142"/>
-      <c r="O26" s="142"/>
-      <c r="P26" s="142"/>
-      <c r="Q26" s="143"/>
-    </row>
-    <row r="27" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="151" t="s">
+      <c r="B26" s="157"/>
+      <c r="C26" s="158"/>
+      <c r="D26" s="148"/>
+      <c r="E26" s="149"/>
+      <c r="F26" s="149"/>
+      <c r="G26" s="150"/>
+      <c r="H26" s="148"/>
+      <c r="I26" s="149"/>
+      <c r="J26" s="149"/>
+      <c r="K26" s="150"/>
+      <c r="L26" s="142"/>
+      <c r="M26" s="143"/>
+      <c r="N26" s="143"/>
+      <c r="O26" s="143"/>
+      <c r="P26" s="143"/>
+      <c r="Q26" s="144"/>
+      <c r="S26"/>
+      <c r="T26"/>
+    </row>
+    <row r="27" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A27" s="145" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="151"/>
-      <c r="C27" s="151"/>
-      <c r="D27" s="140"/>
-      <c r="E27" s="140"/>
-      <c r="F27" s="144"/>
-      <c r="G27" s="144"/>
-      <c r="H27" s="145"/>
-      <c r="I27" s="146"/>
-      <c r="J27" s="144"/>
-      <c r="K27" s="144"/>
-      <c r="L27" s="144"/>
-      <c r="M27" s="144"/>
-      <c r="N27" s="144"/>
-      <c r="O27" s="144"/>
-      <c r="P27" s="144"/>
-      <c r="Q27" s="144"/>
-    </row>
-    <row r="28" spans="1:20" ht="11.4" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="163" t="s">
+      <c r="B27" s="145"/>
+      <c r="C27" s="145"/>
+      <c r="D27" s="151"/>
+      <c r="E27" s="151"/>
+      <c r="F27" s="130"/>
+      <c r="G27" s="130"/>
+      <c r="H27" s="148"/>
+      <c r="I27" s="150"/>
+      <c r="J27" s="130"/>
+      <c r="K27" s="130"/>
+      <c r="L27" s="130"/>
+      <c r="M27" s="130"/>
+      <c r="N27" s="130"/>
+      <c r="O27" s="130"/>
+      <c r="P27" s="130"/>
+      <c r="Q27" s="130"/>
+      <c r="S27"/>
+      <c r="T27"/>
+    </row>
+    <row r="28" spans="1:20" ht="11.4" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A28" s="159" t="s">
         <v>40</v>
       </c>
-      <c r="B28" s="164"/>
-      <c r="C28" s="164"/>
-      <c r="D28" s="164"/>
-      <c r="E28" s="164"/>
-      <c r="F28" s="164"/>
-      <c r="G28" s="164"/>
-      <c r="H28" s="164"/>
-      <c r="I28" s="164"/>
-      <c r="J28" s="164"/>
-      <c r="K28" s="164"/>
-      <c r="L28" s="164"/>
-      <c r="M28" s="164"/>
-      <c r="N28" s="164"/>
-      <c r="O28" s="164"/>
-      <c r="P28" s="164"/>
-      <c r="Q28" s="165"/>
-    </row>
-    <row r="29" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A29" s="151" t="s">
+      <c r="B28" s="160"/>
+      <c r="C28" s="160"/>
+      <c r="D28" s="160"/>
+      <c r="E28" s="160"/>
+      <c r="F28" s="160"/>
+      <c r="G28" s="160"/>
+      <c r="H28" s="160"/>
+      <c r="I28" s="160"/>
+      <c r="J28" s="160"/>
+      <c r="K28" s="160"/>
+      <c r="L28" s="160"/>
+      <c r="M28" s="160"/>
+      <c r="N28" s="160"/>
+      <c r="O28" s="160"/>
+      <c r="P28" s="160"/>
+      <c r="Q28" s="161"/>
+      <c r="S28"/>
+      <c r="T28"/>
+    </row>
+    <row r="29" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A29" s="145" t="s">
         <v>48</v>
       </c>
-      <c r="B29" s="151"/>
-      <c r="C29" s="151"/>
-      <c r="D29" s="140"/>
-      <c r="E29" s="140"/>
-      <c r="F29" s="144"/>
-      <c r="G29" s="144"/>
-      <c r="H29" s="145"/>
-      <c r="I29" s="146"/>
-      <c r="J29" s="144"/>
-      <c r="K29" s="144"/>
-      <c r="L29" s="145"/>
-      <c r="M29" s="147"/>
-      <c r="N29" s="146"/>
-      <c r="O29" s="145"/>
-      <c r="P29" s="147"/>
-      <c r="Q29" s="146"/>
-      <c r="S29" s="113" t="s">
-        <v>90</v>
-      </c>
-      <c r="T29" s="73">
-        <v>2500</v>
-      </c>
-    </row>
-    <row r="30" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A30" s="151" t="s">
+      <c r="B29" s="145"/>
+      <c r="C29" s="145"/>
+      <c r="D29" s="151"/>
+      <c r="E29" s="151"/>
+      <c r="F29" s="130"/>
+      <c r="G29" s="130"/>
+      <c r="H29" s="148"/>
+      <c r="I29" s="150"/>
+      <c r="J29" s="130"/>
+      <c r="K29" s="130"/>
+      <c r="L29" s="148"/>
+      <c r="M29" s="149"/>
+      <c r="N29" s="150"/>
+      <c r="O29" s="148"/>
+      <c r="P29" s="149"/>
+      <c r="Q29" s="150"/>
+      <c r="S29"/>
+      <c r="T29"/>
+    </row>
+    <row r="30" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A30" s="145" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="151"/>
-      <c r="C30" s="151"/>
-      <c r="D30" s="140"/>
-      <c r="E30" s="140"/>
-      <c r="F30" s="144"/>
-      <c r="G30" s="144"/>
-      <c r="H30" s="145"/>
-      <c r="I30" s="146"/>
-      <c r="J30" s="144"/>
-      <c r="K30" s="144"/>
-      <c r="L30" s="145"/>
-      <c r="M30" s="147"/>
-      <c r="N30" s="146"/>
-      <c r="O30" s="145"/>
-      <c r="P30" s="147"/>
-      <c r="Q30" s="146"/>
-      <c r="S30" s="103" t="e">
-        <f>+(D32-(D34-D30))/(D34-D30)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T30" s="73" t="str">
-        <f>+IF(D32&gt;T29,"Cumple","No Cumple")</f>
-        <v>No Cumple</v>
-      </c>
-    </row>
-    <row r="31" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A31" s="151" t="s">
+      <c r="B30" s="145"/>
+      <c r="C30" s="145"/>
+      <c r="D30" s="151"/>
+      <c r="E30" s="151"/>
+      <c r="F30" s="130"/>
+      <c r="G30" s="130"/>
+      <c r="H30" s="148"/>
+      <c r="I30" s="150"/>
+      <c r="J30" s="130"/>
+      <c r="K30" s="130"/>
+      <c r="L30" s="148"/>
+      <c r="M30" s="149"/>
+      <c r="N30" s="150"/>
+      <c r="O30" s="148"/>
+      <c r="P30" s="149"/>
+      <c r="Q30" s="150"/>
+      <c r="S30"/>
+      <c r="T30"/>
+    </row>
+    <row r="31" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="145" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="151"/>
-      <c r="C31" s="151"/>
-      <c r="D31" s="140"/>
-      <c r="E31" s="140"/>
-      <c r="F31" s="144"/>
-      <c r="G31" s="144"/>
-      <c r="H31" s="145"/>
-      <c r="I31" s="146"/>
-      <c r="J31" s="144"/>
-      <c r="K31" s="144"/>
-      <c r="L31" s="145"/>
-      <c r="M31" s="147"/>
-      <c r="N31" s="146"/>
-      <c r="O31" s="145"/>
-      <c r="P31" s="147"/>
-      <c r="Q31" s="146"/>
-      <c r="S31" s="103" t="e">
-        <f>+(H32-(H34-H30))/(H34-H30)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T31" s="73" t="str">
-        <f>+IF(H32&gt;T29,"Cumple","No Cumple")</f>
-        <v>No Cumple</v>
-      </c>
-    </row>
-    <row r="32" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A32" s="166" t="s">
+      <c r="B31" s="145"/>
+      <c r="C31" s="145"/>
+      <c r="D31" s="151"/>
+      <c r="E31" s="151"/>
+      <c r="F31" s="130"/>
+      <c r="G31" s="130"/>
+      <c r="H31" s="148"/>
+      <c r="I31" s="150"/>
+      <c r="J31" s="130"/>
+      <c r="K31" s="130"/>
+      <c r="L31" s="148"/>
+      <c r="M31" s="149"/>
+      <c r="N31" s="150"/>
+      <c r="O31" s="148"/>
+      <c r="P31" s="149"/>
+      <c r="Q31" s="150"/>
+      <c r="S31"/>
+      <c r="T31"/>
+    </row>
+    <row r="32" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A32" s="162" t="s">
         <v>86</v>
       </c>
-      <c r="B32" s="166"/>
-      <c r="C32" s="166"/>
-      <c r="D32" s="140">
+      <c r="B32" s="162"/>
+      <c r="C32" s="162"/>
+      <c r="D32" s="151">
         <f>+D31-D30</f>
         <v>0</v>
       </c>
-      <c r="E32" s="140"/>
-      <c r="F32" s="140">
+      <c r="E32" s="151"/>
+      <c r="F32" s="151">
         <f>+F31-F30</f>
         <v>0</v>
       </c>
-      <c r="G32" s="140"/>
-      <c r="H32" s="140">
+      <c r="G32" s="151"/>
+      <c r="H32" s="151">
         <f>+H31-H30</f>
         <v>0</v>
       </c>
-      <c r="I32" s="140"/>
-      <c r="J32" s="140">
+      <c r="I32" s="151"/>
+      <c r="J32" s="151">
         <f>+J31-J30</f>
         <v>0</v>
       </c>
-      <c r="K32" s="140"/>
-      <c r="L32" s="141">
+      <c r="K32" s="151"/>
+      <c r="L32" s="142">
         <f>+L31-L30</f>
         <v>0</v>
       </c>
-      <c r="M32" s="142"/>
-      <c r="N32" s="143"/>
-      <c r="O32" s="141">
+      <c r="M32" s="143"/>
+      <c r="N32" s="144"/>
+      <c r="O32" s="142">
         <f>+O31-O30</f>
         <v>0</v>
       </c>
-      <c r="P32" s="142"/>
-      <c r="Q32" s="143"/>
-      <c r="S32" s="103" t="e">
-        <f>+(L32-(L34-L30))/(L34-L30)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-      <c r="T32" s="73" t="str">
-        <f>+IF(L32&gt;T29,"Cumple","No Cumple")</f>
-        <v>No Cumple</v>
-      </c>
-    </row>
-    <row r="33" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="151" t="s">
+      <c r="P32" s="143"/>
+      <c r="Q32" s="144"/>
+      <c r="S32"/>
+      <c r="T32"/>
+    </row>
+    <row r="33" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A33" s="145" t="s">
         <v>51</v>
       </c>
-      <c r="B33" s="151"/>
-      <c r="C33" s="151"/>
-      <c r="D33" s="140"/>
-      <c r="E33" s="140"/>
-      <c r="F33" s="144"/>
-      <c r="G33" s="144"/>
-      <c r="H33" s="145"/>
-      <c r="I33" s="146"/>
-      <c r="J33" s="144"/>
-      <c r="K33" s="144"/>
-      <c r="L33" s="145"/>
-      <c r="M33" s="147"/>
-      <c r="N33" s="146"/>
-      <c r="O33" s="145"/>
-      <c r="P33" s="147"/>
-      <c r="Q33" s="146"/>
-      <c r="S33" s="73" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="34" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="151" t="s">
+      <c r="B33" s="145"/>
+      <c r="C33" s="145"/>
+      <c r="D33" s="151"/>
+      <c r="E33" s="151"/>
+      <c r="F33" s="130"/>
+      <c r="G33" s="130"/>
+      <c r="H33" s="148"/>
+      <c r="I33" s="150"/>
+      <c r="J33" s="130"/>
+      <c r="K33" s="130"/>
+      <c r="L33" s="148"/>
+      <c r="M33" s="149"/>
+      <c r="N33" s="150"/>
+      <c r="O33" s="148"/>
+      <c r="P33" s="149"/>
+      <c r="Q33" s="150"/>
+      <c r="S33"/>
+      <c r="T33"/>
+    </row>
+    <row r="34" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A34" s="145" t="s">
         <v>52</v>
       </c>
-      <c r="B34" s="151"/>
-      <c r="C34" s="151"/>
-      <c r="D34" s="140"/>
-      <c r="E34" s="140"/>
-      <c r="F34" s="144"/>
-      <c r="G34" s="144"/>
-      <c r="H34" s="145"/>
-      <c r="I34" s="146"/>
-      <c r="J34" s="144"/>
-      <c r="K34" s="144"/>
-      <c r="L34" s="145"/>
-      <c r="M34" s="147"/>
-      <c r="N34" s="146"/>
-      <c r="O34" s="145"/>
-      <c r="P34" s="147"/>
-      <c r="Q34" s="146"/>
-      <c r="S34" s="103" t="e">
-        <f>+(F32-(F34-F30))/(F34-F30)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="35" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B34" s="145"/>
+      <c r="C34" s="145"/>
+      <c r="D34" s="151"/>
+      <c r="E34" s="151"/>
+      <c r="F34" s="130"/>
+      <c r="G34" s="130"/>
+      <c r="H34" s="148"/>
+      <c r="I34" s="150"/>
+      <c r="J34" s="130"/>
+      <c r="K34" s="130"/>
+      <c r="L34" s="148"/>
+      <c r="M34" s="149"/>
+      <c r="N34" s="150"/>
+      <c r="O34" s="148"/>
+      <c r="P34" s="149"/>
+      <c r="Q34" s="150"/>
+      <c r="S34"/>
+      <c r="T34"/>
+    </row>
+    <row r="35" spans="1:20" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="99" t="s">
         <v>87</v>
       </c>
@@ -3187,12 +3006,10 @@
       <c r="O35" s="95"/>
       <c r="P35" s="95"/>
       <c r="Q35" s="96"/>
-      <c r="S35" s="103" t="e">
-        <f>+(J32-(J34-J30))/(J34-J30)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="36" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S35"/>
+      <c r="T35"/>
+    </row>
+    <row r="36" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="17" t="s">
         <v>41</v>
       </c>
@@ -3212,69 +3029,69 @@
       <c r="O36" s="26"/>
       <c r="P36" s="26"/>
       <c r="Q36" s="27"/>
-      <c r="S36" s="103" t="e">
-        <f>+(O32-(O34-O30))/(O34-O30)*100</f>
-        <v>#DIV/0!</v>
-      </c>
-    </row>
-    <row r="37" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A37" s="152" t="s">
+      <c r="S36"/>
+      <c r="T36"/>
+    </row>
+    <row r="37" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="165" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="118" t="s">
+      <c r="B37" s="138" t="s">
         <v>17</v>
       </c>
-      <c r="C37" s="119"/>
+      <c r="C37" s="140"/>
       <c r="D37" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E37" s="118" t="s">
+      <c r="E37" s="138" t="s">
         <v>45</v>
       </c>
-      <c r="F37" s="157"/>
-      <c r="G37" s="157"/>
-      <c r="H37" s="157"/>
-      <c r="I37" s="157"/>
-      <c r="J37" s="119"/>
+      <c r="F37" s="139"/>
+      <c r="G37" s="139"/>
+      <c r="H37" s="139"/>
+      <c r="I37" s="139"/>
+      <c r="J37" s="140"/>
       <c r="K37" s="49"/>
-      <c r="L37" s="138" t="s">
+      <c r="L37" s="188" t="s">
         <v>83</v>
       </c>
-      <c r="M37" s="138"/>
-      <c r="N37" s="138"/>
-      <c r="O37" s="138"/>
-      <c r="P37" s="138"/>
-      <c r="Q37" s="138"/>
-    </row>
-    <row r="38" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="153"/>
-      <c r="B38" s="155" t="s">
+      <c r="M37" s="188"/>
+      <c r="N37" s="188"/>
+      <c r="O37" s="188"/>
+      <c r="P37" s="188"/>
+      <c r="Q37" s="188"/>
+      <c r="S37"/>
+      <c r="T37"/>
+    </row>
+    <row r="38" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="166"/>
+      <c r="B38" s="168" t="s">
         <v>70</v>
       </c>
-      <c r="C38" s="155" t="s">
+      <c r="C38" s="168" t="s">
         <v>71</v>
       </c>
       <c r="D38" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E38" s="133" t="s">
+      <c r="E38" s="170" t="s">
         <v>44</v>
       </c>
-      <c r="F38" s="134"/>
-      <c r="G38" s="133" t="s">
+      <c r="F38" s="171"/>
+      <c r="G38" s="170" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="134"/>
-      <c r="I38" s="133" t="s">
+      <c r="H38" s="171"/>
+      <c r="I38" s="170" t="s">
         <v>44</v>
       </c>
-      <c r="J38" s="134"/>
+      <c r="J38" s="171"/>
       <c r="K38" s="49"/>
-      <c r="L38" s="133" t="s">
+      <c r="L38" s="170" t="s">
         <v>19</v>
       </c>
-      <c r="M38" s="134"/>
-      <c r="N38" s="168" t="s">
+      <c r="M38" s="171"/>
+      <c r="N38" s="152" t="s">
         <v>34</v>
       </c>
       <c r="O38" s="73" t="s">
@@ -3286,42 +3103,34 @@
       <c r="Q38" s="73" t="s">
         <v>56</v>
       </c>
-      <c r="S38" s="115" t="s">
-        <v>92</v>
-      </c>
-      <c r="T38" s="115" t="s">
-        <v>111</v>
-      </c>
+      <c r="S38"/>
+      <c r="T38"/>
     </row>
     <row r="39" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="154"/>
-      <c r="B39" s="156"/>
-      <c r="C39" s="156"/>
+      <c r="A39" s="167"/>
+      <c r="B39" s="169"/>
+      <c r="C39" s="169"/>
       <c r="D39" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="E39" s="135"/>
-      <c r="F39" s="136"/>
-      <c r="G39" s="135"/>
-      <c r="H39" s="136"/>
-      <c r="I39" s="135"/>
-      <c r="J39" s="136"/>
+      <c r="E39" s="172"/>
+      <c r="F39" s="173"/>
+      <c r="G39" s="172"/>
+      <c r="H39" s="173"/>
+      <c r="I39" s="172"/>
+      <c r="J39" s="173"/>
       <c r="K39" s="49"/>
-      <c r="L39" s="135"/>
-      <c r="M39" s="136"/>
-      <c r="N39" s="169"/>
-      <c r="O39" s="118" t="s">
+      <c r="L39" s="172"/>
+      <c r="M39" s="173"/>
+      <c r="N39" s="153"/>
+      <c r="O39" s="138" t="s">
         <v>73</v>
       </c>
-      <c r="P39" s="157"/>
-      <c r="Q39" s="119"/>
+      <c r="P39" s="139"/>
+      <c r="Q39" s="140"/>
       <c r="R39" s="50"/>
-      <c r="S39" s="117" t="s">
-        <v>93</v>
-      </c>
-      <c r="T39" s="114" t="s">
-        <v>112</v>
-      </c>
+      <c r="S39"/>
+      <c r="T39"/>
     </row>
     <row r="40" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="24" t="s">
@@ -3334,28 +3143,24 @@
         <v>0</v>
       </c>
       <c r="D40" s="23"/>
-      <c r="E40" s="118"/>
-      <c r="F40" s="119"/>
-      <c r="G40" s="118"/>
-      <c r="H40" s="119"/>
-      <c r="I40" s="118"/>
-      <c r="J40" s="119"/>
+      <c r="E40" s="138"/>
+      <c r="F40" s="140"/>
+      <c r="G40" s="138"/>
+      <c r="H40" s="140"/>
+      <c r="I40" s="138"/>
+      <c r="J40" s="140"/>
       <c r="K40" s="49"/>
-      <c r="L40" s="148"/>
-      <c r="M40" s="149"/>
+      <c r="L40" s="146"/>
+      <c r="M40" s="147"/>
       <c r="N40" s="69"/>
       <c r="O40" s="102"/>
       <c r="P40" s="102"/>
       <c r="Q40" s="70"/>
       <c r="R40" s="50"/>
-      <c r="S40" s="117" t="s">
-        <v>94</v>
-      </c>
-      <c r="T40" s="114" t="s">
-        <v>113</v>
-      </c>
-    </row>
-    <row r="41" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S40"/>
+      <c r="T40"/>
+    </row>
+    <row r="41" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="24" t="s">
         <v>18</v>
       </c>
@@ -3366,28 +3171,24 @@
         <v>0.64</v>
       </c>
       <c r="D41" s="23"/>
-      <c r="E41" s="118"/>
-      <c r="F41" s="119"/>
-      <c r="G41" s="118"/>
-      <c r="H41" s="119"/>
-      <c r="I41" s="118"/>
-      <c r="J41" s="119"/>
+      <c r="E41" s="138"/>
+      <c r="F41" s="140"/>
+      <c r="G41" s="138"/>
+      <c r="H41" s="140"/>
+      <c r="I41" s="138"/>
+      <c r="J41" s="140"/>
       <c r="K41" s="51"/>
-      <c r="L41" s="148"/>
-      <c r="M41" s="149"/>
+      <c r="L41" s="146"/>
+      <c r="M41" s="147"/>
       <c r="N41" s="69"/>
       <c r="O41" s="19"/>
       <c r="P41" s="19"/>
       <c r="Q41" s="19"/>
       <c r="R41" s="52"/>
-      <c r="S41" s="117" t="s">
-        <v>95</v>
-      </c>
-      <c r="T41" s="114" t="s">
-        <v>114</v>
-      </c>
-    </row>
-    <row r="42" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S41"/>
+      <c r="T41"/>
+    </row>
+    <row r="42" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="24" t="s">
         <v>20</v>
       </c>
@@ -3398,28 +3199,24 @@
         <v>1.3</v>
       </c>
       <c r="D42" s="23"/>
-      <c r="E42" s="118"/>
-      <c r="F42" s="119"/>
-      <c r="G42" s="118"/>
-      <c r="H42" s="119"/>
-      <c r="I42" s="118"/>
-      <c r="J42" s="119"/>
+      <c r="E42" s="138"/>
+      <c r="F42" s="140"/>
+      <c r="G42" s="138"/>
+      <c r="H42" s="140"/>
+      <c r="I42" s="138"/>
+      <c r="J42" s="140"/>
       <c r="K42" s="51"/>
-      <c r="L42" s="148"/>
-      <c r="M42" s="149"/>
+      <c r="L42" s="146"/>
+      <c r="M42" s="147"/>
       <c r="N42" s="69"/>
       <c r="O42" s="19"/>
       <c r="P42" s="19"/>
       <c r="Q42" s="19"/>
       <c r="R42" s="52"/>
-      <c r="S42" s="117" t="s">
-        <v>96</v>
-      </c>
-      <c r="T42" s="114" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="43" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S42"/>
+      <c r="T42"/>
+    </row>
+    <row r="43" spans="1:20" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="24" t="s">
         <v>21</v>
       </c>
@@ -3430,78 +3227,70 @@
         <v>1.9</v>
       </c>
       <c r="D43" s="23"/>
-      <c r="E43" s="118"/>
-      <c r="F43" s="119"/>
-      <c r="G43" s="118"/>
-      <c r="H43" s="119"/>
-      <c r="I43" s="118"/>
-      <c r="J43" s="119"/>
+      <c r="E43" s="138"/>
+      <c r="F43" s="140"/>
+      <c r="G43" s="138"/>
+      <c r="H43" s="140"/>
+      <c r="I43" s="138"/>
+      <c r="J43" s="140"/>
       <c r="K43" s="51"/>
-      <c r="L43" s="148"/>
-      <c r="M43" s="149"/>
+      <c r="L43" s="146"/>
+      <c r="M43" s="147"/>
       <c r="N43" s="69"/>
       <c r="O43" s="19"/>
       <c r="P43" s="19"/>
       <c r="Q43" s="19"/>
       <c r="R43" s="52"/>
-      <c r="S43" s="117" t="s">
-        <v>97</v>
-      </c>
-      <c r="T43" s="114" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="44" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A44" s="108" t="s">
+      <c r="S43"/>
+      <c r="T43"/>
+    </row>
+    <row r="44" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A44" s="107" t="s">
         <v>22</v>
       </c>
-      <c r="B44" s="109">
+      <c r="B44" s="108">
         <v>0.1</v>
       </c>
-      <c r="C44" s="110">
+      <c r="C44" s="109">
         <v>2.5</v>
       </c>
-      <c r="D44" s="111">
+      <c r="D44" s="110">
         <v>1000</v>
       </c>
-      <c r="E44" s="131"/>
-      <c r="F44" s="132"/>
-      <c r="G44" s="131"/>
-      <c r="H44" s="132"/>
-      <c r="I44" s="131"/>
-      <c r="J44" s="132"/>
+      <c r="E44" s="163"/>
+      <c r="F44" s="164"/>
+      <c r="G44" s="163"/>
+      <c r="H44" s="164"/>
+      <c r="I44" s="163"/>
+      <c r="J44" s="164"/>
       <c r="K44" s="51"/>
-      <c r="L44" s="148"/>
-      <c r="M44" s="149"/>
+      <c r="L44" s="146"/>
+      <c r="M44" s="147"/>
       <c r="N44" s="69"/>
       <c r="O44" s="19"/>
       <c r="P44" s="19"/>
       <c r="Q44" s="19"/>
       <c r="R44" s="52"/>
-      <c r="S44" s="117" t="s">
-        <v>98</v>
-      </c>
-      <c r="T44" s="114" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="45" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A45" s="107">
+      <c r="S44"/>
+      <c r="T44"/>
+    </row>
+    <row r="45" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A45" s="106">
         <v>0.10416666666666667</v>
       </c>
-      <c r="B45" s="104">
+      <c r="B45" s="103">
         <v>0.125</v>
       </c>
-      <c r="C45" s="105">
+      <c r="C45" s="104">
         <v>3.18</v>
       </c>
-      <c r="D45" s="106"/>
-      <c r="E45" s="131"/>
-      <c r="F45" s="132"/>
-      <c r="G45" s="131"/>
-      <c r="H45" s="132"/>
-      <c r="I45" s="131"/>
-      <c r="J45" s="132"/>
+      <c r="D45" s="105"/>
+      <c r="E45" s="163"/>
+      <c r="F45" s="164"/>
+      <c r="G45" s="163"/>
+      <c r="H45" s="164"/>
+      <c r="I45" s="163"/>
+      <c r="J45" s="164"/>
       <c r="K45" s="51"/>
       <c r="L45" s="40"/>
       <c r="M45" s="40"/>
@@ -3510,124 +3299,108 @@
       <c r="P45" s="40"/>
       <c r="Q45" s="41"/>
       <c r="R45" s="52"/>
-      <c r="S45" s="117" t="s">
-        <v>99</v>
-      </c>
-      <c r="T45" s="114" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="46" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A46" s="107">
+      <c r="S45"/>
+      <c r="T45"/>
+    </row>
+    <row r="46" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A46" s="106">
         <v>0.125</v>
       </c>
-      <c r="B46" s="104">
+      <c r="B46" s="103">
         <v>0.15</v>
       </c>
-      <c r="C46" s="105">
+      <c r="C46" s="104">
         <v>3.8</v>
       </c>
-      <c r="D46" s="106"/>
-      <c r="E46" s="131"/>
-      <c r="F46" s="132"/>
-      <c r="G46" s="131"/>
-      <c r="H46" s="132"/>
-      <c r="I46" s="131"/>
-      <c r="J46" s="132"/>
+      <c r="D46" s="105"/>
+      <c r="E46" s="163"/>
+      <c r="F46" s="164"/>
+      <c r="G46" s="163"/>
+      <c r="H46" s="164"/>
+      <c r="I46" s="163"/>
+      <c r="J46" s="164"/>
       <c r="K46" s="51"/>
-      <c r="L46" s="125" t="s">
+      <c r="L46" s="184" t="s">
         <v>75</v>
       </c>
-      <c r="M46" s="126"/>
-      <c r="N46" s="127"/>
-      <c r="O46" s="150" t="s">
+      <c r="M46" s="185"/>
+      <c r="N46" s="186"/>
+      <c r="O46" s="178" t="s">
         <v>76</v>
       </c>
-      <c r="P46" s="150"/>
-      <c r="Q46" s="150"/>
+      <c r="P46" s="178"/>
+      <c r="Q46" s="178"/>
       <c r="R46" s="52"/>
-      <c r="S46" s="117" t="s">
-        <v>100</v>
-      </c>
-      <c r="T46" s="114" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="47" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A47" s="107">
+      <c r="S46"/>
+      <c r="T46"/>
+    </row>
+    <row r="47" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A47" s="106">
         <v>0.14583333333333334</v>
       </c>
-      <c r="B47" s="104">
+      <c r="B47" s="103">
         <v>0.17499999999999999</v>
       </c>
-      <c r="C47" s="105">
+      <c r="C47" s="104">
         <v>4.45</v>
       </c>
-      <c r="D47" s="106"/>
-      <c r="E47" s="131"/>
-      <c r="F47" s="132"/>
-      <c r="G47" s="131"/>
-      <c r="H47" s="132"/>
-      <c r="I47" s="131"/>
-      <c r="J47" s="132"/>
+      <c r="D47" s="105"/>
+      <c r="E47" s="163"/>
+      <c r="F47" s="164"/>
+      <c r="G47" s="163"/>
+      <c r="H47" s="164"/>
+      <c r="I47" s="163"/>
+      <c r="J47" s="164"/>
       <c r="K47" s="51"/>
-      <c r="L47" s="128" t="s">
+      <c r="L47" s="175" t="s">
         <v>80</v>
       </c>
-      <c r="M47" s="129"/>
-      <c r="N47" s="130"/>
-      <c r="O47" s="139" t="s">
-        <v>130</v>
-      </c>
-      <c r="P47" s="139"/>
-      <c r="Q47" s="139"/>
+      <c r="M47" s="176"/>
+      <c r="N47" s="177"/>
+      <c r="O47" s="174" t="s">
+        <v>90</v>
+      </c>
+      <c r="P47" s="174"/>
+      <c r="Q47" s="174"/>
       <c r="R47" s="52"/>
-      <c r="S47" s="117" t="s">
-        <v>101</v>
-      </c>
-      <c r="T47" s="114" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="48" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A48" s="112">
+      <c r="S47"/>
+      <c r="T47"/>
+    </row>
+    <row r="48" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A48" s="111">
         <v>0.16666666666666666</v>
       </c>
-      <c r="B48" s="109">
+      <c r="B48" s="108">
         <v>0.2</v>
       </c>
-      <c r="C48" s="110">
+      <c r="C48" s="109">
         <v>5.0999999999999996</v>
       </c>
-      <c r="D48" s="111">
+      <c r="D48" s="110">
         <v>1500</v>
       </c>
-      <c r="E48" s="131"/>
-      <c r="F48" s="132"/>
-      <c r="G48" s="131"/>
-      <c r="H48" s="132"/>
-      <c r="I48" s="131"/>
-      <c r="J48" s="132"/>
+      <c r="E48" s="163"/>
+      <c r="F48" s="164"/>
+      <c r="G48" s="163"/>
+      <c r="H48" s="164"/>
+      <c r="I48" s="163"/>
+      <c r="J48" s="164"/>
       <c r="K48" s="51"/>
-      <c r="L48" s="128" t="s">
+      <c r="L48" s="175" t="s">
         <v>81</v>
       </c>
-      <c r="M48" s="129"/>
-      <c r="N48" s="130"/>
-      <c r="O48" s="139" t="s">
-        <v>131</v>
-      </c>
-      <c r="P48" s="139"/>
-      <c r="Q48" s="139"/>
+      <c r="M48" s="176"/>
+      <c r="N48" s="177"/>
+      <c r="O48" s="174" t="s">
+        <v>91</v>
+      </c>
+      <c r="P48" s="174"/>
+      <c r="Q48" s="174"/>
       <c r="R48" s="52"/>
-      <c r="S48" s="117" t="s">
-        <v>102</v>
-      </c>
-      <c r="T48" s="114" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="49" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S48"/>
+      <c r="T48"/>
+    </row>
+    <row r="49" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="25">
         <v>0.25</v>
       </c>
@@ -3638,32 +3411,28 @@
         <v>7.6</v>
       </c>
       <c r="D49" s="23"/>
-      <c r="E49" s="118"/>
-      <c r="F49" s="119"/>
-      <c r="G49" s="118"/>
-      <c r="H49" s="119"/>
-      <c r="I49" s="118"/>
-      <c r="J49" s="119"/>
+      <c r="E49" s="138"/>
+      <c r="F49" s="140"/>
+      <c r="G49" s="138"/>
+      <c r="H49" s="140"/>
+      <c r="I49" s="138"/>
+      <c r="J49" s="140"/>
       <c r="K49" s="53"/>
-      <c r="L49" s="128" t="s">
+      <c r="L49" s="175" t="s">
         <v>82</v>
       </c>
-      <c r="M49" s="129"/>
-      <c r="N49" s="130"/>
-      <c r="O49" s="139" t="s">
-        <v>132</v>
-      </c>
-      <c r="P49" s="139"/>
-      <c r="Q49" s="139"/>
+      <c r="M49" s="176"/>
+      <c r="N49" s="177"/>
+      <c r="O49" s="174" t="s">
+        <v>92</v>
+      </c>
+      <c r="P49" s="174"/>
+      <c r="Q49" s="174"/>
       <c r="R49" s="52"/>
-      <c r="S49" s="117" t="s">
-        <v>103</v>
-      </c>
-      <c r="T49" s="114" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="50" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S49"/>
+      <c r="T49"/>
+    </row>
+    <row r="50" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="25">
         <v>0.33333333333333331</v>
       </c>
@@ -3674,32 +3443,28 @@
         <v>10</v>
       </c>
       <c r="D50" s="23"/>
-      <c r="E50" s="118"/>
-      <c r="F50" s="119"/>
-      <c r="G50" s="118"/>
-      <c r="H50" s="119"/>
-      <c r="I50" s="118"/>
-      <c r="J50" s="119"/>
+      <c r="E50" s="138"/>
+      <c r="F50" s="140"/>
+      <c r="G50" s="138"/>
+      <c r="H50" s="140"/>
+      <c r="I50" s="138"/>
+      <c r="J50" s="140"/>
       <c r="K50" s="53"/>
       <c r="L50" s="74" t="s">
         <v>78</v>
       </c>
       <c r="M50" s="75"/>
       <c r="N50" s="76"/>
-      <c r="O50" s="139" t="s">
-        <v>133</v>
-      </c>
-      <c r="P50" s="139"/>
-      <c r="Q50" s="139"/>
+      <c r="O50" s="174" t="s">
+        <v>93</v>
+      </c>
+      <c r="P50" s="174"/>
+      <c r="Q50" s="174"/>
       <c r="R50" s="52"/>
-      <c r="S50" s="117" t="s">
-        <v>104</v>
-      </c>
-      <c r="T50" s="114" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="51" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S50"/>
+      <c r="T50"/>
+    </row>
+    <row r="51" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="25">
         <v>0.41666666666666669</v>
       </c>
@@ -3710,32 +3475,28 @@
         <v>13</v>
       </c>
       <c r="D51" s="23"/>
-      <c r="E51" s="118"/>
-      <c r="F51" s="119"/>
-      <c r="G51" s="118"/>
-      <c r="H51" s="119"/>
-      <c r="I51" s="118"/>
-      <c r="J51" s="119"/>
+      <c r="E51" s="138"/>
+      <c r="F51" s="140"/>
+      <c r="G51" s="138"/>
+      <c r="H51" s="140"/>
+      <c r="I51" s="138"/>
+      <c r="J51" s="140"/>
       <c r="K51" s="54"/>
       <c r="L51" s="74" t="s">
         <v>79</v>
       </c>
       <c r="M51" s="75"/>
       <c r="N51" s="76"/>
-      <c r="O51" s="139" t="s">
-        <v>134</v>
-      </c>
-      <c r="P51" s="139"/>
-      <c r="Q51" s="139"/>
+      <c r="O51" s="174" t="s">
+        <v>94</v>
+      </c>
+      <c r="P51" s="174"/>
+      <c r="Q51" s="174"/>
       <c r="R51" s="52"/>
-      <c r="S51" s="117" t="s">
-        <v>105</v>
-      </c>
-      <c r="T51" s="114" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="52" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S51"/>
+      <c r="T51"/>
+    </row>
+    <row r="52" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="55"/>
       <c r="B52" s="28"/>
       <c r="C52" s="28"/>
@@ -3747,55 +3508,47 @@
       <c r="I52" s="57"/>
       <c r="J52" s="28"/>
       <c r="K52" s="14"/>
-      <c r="L52" s="128" t="s">
+      <c r="L52" s="175" t="s">
         <v>77</v>
       </c>
-      <c r="M52" s="129"/>
-      <c r="N52" s="130"/>
-      <c r="O52" s="139" t="s">
-        <v>135</v>
-      </c>
-      <c r="P52" s="139"/>
-      <c r="Q52" s="139"/>
-      <c r="S52" s="117" t="s">
-        <v>106</v>
-      </c>
-      <c r="T52" s="114" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="53" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M52" s="176"/>
+      <c r="N52" s="177"/>
+      <c r="O52" s="174" t="s">
+        <v>95</v>
+      </c>
+      <c r="P52" s="174"/>
+      <c r="Q52" s="174"/>
+      <c r="S52"/>
+      <c r="T52"/>
+    </row>
+    <row r="53" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="58" t="s">
         <v>37</v>
       </c>
       <c r="B53" s="59"/>
       <c r="C53" s="59"/>
       <c r="D53" s="60"/>
-      <c r="E53" s="118"/>
-      <c r="F53" s="119"/>
-      <c r="G53" s="118"/>
-      <c r="H53" s="119"/>
-      <c r="I53" s="120"/>
-      <c r="J53" s="121"/>
+      <c r="E53" s="138"/>
+      <c r="F53" s="140"/>
+      <c r="G53" s="138"/>
+      <c r="H53" s="140"/>
+      <c r="I53" s="179"/>
+      <c r="J53" s="180"/>
       <c r="K53" s="61"/>
-      <c r="L53" s="128" t="s">
+      <c r="L53" s="175" t="s">
         <v>84</v>
       </c>
-      <c r="M53" s="129"/>
-      <c r="N53" s="130"/>
-      <c r="O53" s="139" t="s">
-        <v>136</v>
-      </c>
-      <c r="P53" s="139"/>
-      <c r="Q53" s="139"/>
-      <c r="S53" s="117" t="s">
-        <v>107</v>
-      </c>
-      <c r="T53" s="114" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="54" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="M53" s="176"/>
+      <c r="N53" s="177"/>
+      <c r="O53" s="174" t="s">
+        <v>96</v>
+      </c>
+      <c r="P53" s="174"/>
+      <c r="Q53" s="174"/>
+      <c r="S53"/>
+      <c r="T53"/>
+    </row>
+    <row r="54" spans="1:20" ht="16.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="14"/>
       <c r="B54" s="14"/>
       <c r="C54" s="14"/>
@@ -3813,14 +3566,10 @@
       <c r="O54" s="14"/>
       <c r="P54" s="14"/>
       <c r="Q54" s="14"/>
-      <c r="S54" s="117" t="s">
-        <v>108</v>
-      </c>
-      <c r="T54" s="114" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="55" spans="1:20" ht="15.6" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S54"/>
+      <c r="T54"/>
+    </row>
+    <row r="55" spans="1:20" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="55"/>
       <c r="B55" s="28"/>
       <c r="C55" s="28"/>
@@ -3838,14 +3587,10 @@
       <c r="O55" s="28"/>
       <c r="P55" s="28"/>
       <c r="Q55" s="29"/>
-      <c r="S55" s="117" t="s">
-        <v>109</v>
-      </c>
-      <c r="T55" s="114" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="56" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S55"/>
+      <c r="T55"/>
+    </row>
+    <row r="56" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="62" t="s">
         <v>24</v>
       </c>
@@ -3865,14 +3610,10 @@
       <c r="O56" s="63"/>
       <c r="P56" s="63"/>
       <c r="Q56" s="66"/>
-      <c r="S56" s="117" t="s">
-        <v>110</v>
-      </c>
-      <c r="T56" s="114" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="57" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="S56"/>
+      <c r="T56"/>
+    </row>
+    <row r="57" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="77"/>
       <c r="B57" s="28"/>
       <c r="C57" s="28"/>
@@ -3890,6 +3631,8 @@
       <c r="O57" s="28"/>
       <c r="P57" s="28"/>
       <c r="Q57" s="29"/>
+      <c r="S57"/>
+      <c r="T57"/>
     </row>
     <row r="58" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="59" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3934,25 +3677,25 @@
     </row>
     <row r="62" spans="1:20" ht="7.2" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="63" spans="1:20" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="176" t="s">
+      <c r="A63" s="131" t="s">
         <v>85</v>
       </c>
-      <c r="B63" s="176"/>
-      <c r="C63" s="176"/>
-      <c r="D63" s="176"/>
-      <c r="E63" s="176"/>
-      <c r="F63" s="176"/>
-      <c r="G63" s="176"/>
-      <c r="H63" s="176"/>
-      <c r="I63" s="176"/>
-      <c r="J63" s="176"/>
-      <c r="K63" s="176"/>
-      <c r="L63" s="176"/>
-      <c r="M63" s="176"/>
-      <c r="N63" s="176"/>
-      <c r="O63" s="176"/>
-      <c r="P63" s="176"/>
-      <c r="Q63" s="176"/>
+      <c r="B63" s="131"/>
+      <c r="C63" s="131"/>
+      <c r="D63" s="131"/>
+      <c r="E63" s="131"/>
+      <c r="F63" s="131"/>
+      <c r="G63" s="131"/>
+      <c r="H63" s="131"/>
+      <c r="I63" s="131"/>
+      <c r="J63" s="131"/>
+      <c r="K63" s="131"/>
+      <c r="L63" s="131"/>
+      <c r="M63" s="131"/>
+      <c r="N63" s="131"/>
+      <c r="O63" s="131"/>
+      <c r="P63" s="131"/>
+      <c r="Q63" s="131"/>
     </row>
     <row r="64" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="65" ht="15.9" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3962,6 +3705,143 @@
     <protectedRange sqref="C8:C9" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="161">
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="L46:N46"/>
+    <mergeCell ref="L47:N47"/>
+    <mergeCell ref="L48:N48"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="L38:M39"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="L37:Q37"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="O50:Q50"/>
+    <mergeCell ref="L53:N53"/>
+    <mergeCell ref="O53:Q53"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="O47:Q47"/>
+    <mergeCell ref="O48:Q48"/>
+    <mergeCell ref="O49:Q49"/>
+    <mergeCell ref="O52:Q52"/>
+    <mergeCell ref="O51:Q51"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="O46:Q46"/>
+    <mergeCell ref="G48:H48"/>
+    <mergeCell ref="E53:F53"/>
+    <mergeCell ref="G53:H53"/>
+    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="L49:N49"/>
+    <mergeCell ref="L52:N52"/>
+    <mergeCell ref="L32:N32"/>
+    <mergeCell ref="O32:Q32"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="O34:Q34"/>
+    <mergeCell ref="I38:J39"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="G49:H49"/>
+    <mergeCell ref="G50:H50"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="A37:A39"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="E37:J37"/>
+    <mergeCell ref="E38:F39"/>
+    <mergeCell ref="G38:H39"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="O29:Q29"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="E20:Q20"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="O31:Q31"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="L44:M44"/>
+    <mergeCell ref="O30:Q30"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="H26:K26"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="O33:Q33"/>
+    <mergeCell ref="N38:N39"/>
+    <mergeCell ref="O27:Q27"/>
     <mergeCell ref="D8:E8"/>
     <mergeCell ref="D2:Q2"/>
     <mergeCell ref="D3:Q3"/>
@@ -3986,143 +3866,6 @@
     <mergeCell ref="L22:N22"/>
     <mergeCell ref="O22:Q22"/>
     <mergeCell ref="A21:C21"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="L44:M44"/>
-    <mergeCell ref="O30:Q30"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="H25:K25"/>
-    <mergeCell ref="H26:K26"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="O33:Q33"/>
-    <mergeCell ref="N38:N39"/>
-    <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="O29:Q29"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="E20:Q20"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="A28:Q28"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="G49:H49"/>
-    <mergeCell ref="G50:H50"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="A37:A39"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="E37:J37"/>
-    <mergeCell ref="E38:F39"/>
-    <mergeCell ref="G38:H39"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="L32:N32"/>
-    <mergeCell ref="O32:Q32"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="L34:N34"/>
-    <mergeCell ref="O34:Q34"/>
-    <mergeCell ref="I38:J39"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="L41:M41"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="L43:M43"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="O50:Q50"/>
-    <mergeCell ref="L53:N53"/>
-    <mergeCell ref="O53:Q53"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="O47:Q47"/>
-    <mergeCell ref="O48:Q48"/>
-    <mergeCell ref="O49:Q49"/>
-    <mergeCell ref="O52:Q52"/>
-    <mergeCell ref="O51:Q51"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="O46:Q46"/>
-    <mergeCell ref="G48:H48"/>
-    <mergeCell ref="E53:F53"/>
-    <mergeCell ref="G53:H53"/>
-    <mergeCell ref="I53:J53"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="L46:N46"/>
-    <mergeCell ref="L47:N47"/>
-    <mergeCell ref="L48:N48"/>
-    <mergeCell ref="L49:N49"/>
-    <mergeCell ref="L52:N52"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="L38:M39"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="L37:Q37"/>
-    <mergeCell ref="E48:F48"/>
-    <mergeCell ref="E49:F49"/>
-    <mergeCell ref="E50:F50"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="E44:F44"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.39370078740157483" top="0.78740157480314965" bottom="0" header="0" footer="0"/>
@@ -4148,10 +3891,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="184" t="s">
+      <c r="A2" s="189" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="184"/>
+      <c r="B2" s="189"/>
       <c r="C2" s="5" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
chore(cbr): actualizar template con encabezados fusionados
</commit_message>
<xml_diff>
--- a/app/templates/Temp_CBR_ASTM.xlsx
+++ b/app/templates/Temp_CBR_ASTM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F28A87B-B48B-4603-8C74-0F2E8B7E76D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8715C8F-9907-45E4-ACB1-FDE61825F565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -733,7 +733,7 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="17" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="190">
+  <cellXfs count="186">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1075,29 +1075,174 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1125,12 +1270,6 @@
     <xf numFmtId="166" fontId="15" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1159,171 +1298,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2246,43 +2234,43 @@
       <c r="A2" s="81"/>
       <c r="B2" s="82"/>
       <c r="C2" s="83"/>
-      <c r="D2" s="123" t="s">
+      <c r="D2" s="168" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="124"/>
-      <c r="F2" s="124"/>
-      <c r="G2" s="124"/>
-      <c r="H2" s="124"/>
-      <c r="I2" s="124"/>
-      <c r="J2" s="124"/>
-      <c r="K2" s="124"/>
-      <c r="L2" s="124"/>
-      <c r="M2" s="124"/>
-      <c r="N2" s="124"/>
-      <c r="O2" s="124"/>
-      <c r="P2" s="124"/>
-      <c r="Q2" s="125"/>
+      <c r="E2" s="169"/>
+      <c r="F2" s="169"/>
+      <c r="G2" s="169"/>
+      <c r="H2" s="169"/>
+      <c r="I2" s="169"/>
+      <c r="J2" s="169"/>
+      <c r="K2" s="169"/>
+      <c r="L2" s="169"/>
+      <c r="M2" s="169"/>
+      <c r="N2" s="169"/>
+      <c r="O2" s="169"/>
+      <c r="P2" s="169"/>
+      <c r="Q2" s="170"/>
     </row>
     <row r="3" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="81"/>
       <c r="B3" s="82"/>
       <c r="C3" s="83"/>
-      <c r="D3" s="126" t="s">
+      <c r="D3" s="171" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="127"/>
-      <c r="F3" s="127"/>
-      <c r="G3" s="127"/>
-      <c r="H3" s="127"/>
-      <c r="I3" s="127"/>
-      <c r="J3" s="127"/>
-      <c r="K3" s="127"/>
-      <c r="L3" s="127"/>
-      <c r="M3" s="127"/>
-      <c r="N3" s="127"/>
-      <c r="O3" s="127"/>
-      <c r="P3" s="127"/>
-      <c r="Q3" s="128"/>
+      <c r="E3" s="172"/>
+      <c r="F3" s="172"/>
+      <c r="G3" s="172"/>
+      <c r="H3" s="172"/>
+      <c r="I3" s="172"/>
+      <c r="J3" s="172"/>
+      <c r="K3" s="172"/>
+      <c r="L3" s="172"/>
+      <c r="M3" s="172"/>
+      <c r="N3" s="172"/>
+      <c r="O3" s="172"/>
+      <c r="P3" s="172"/>
+      <c r="Q3" s="173"/>
     </row>
     <row r="4" spans="1:17" ht="3" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="81"/>
@@ -2361,43 +2349,41 @@
     <row r="8" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="32"/>
       <c r="C8" s="32"/>
-      <c r="D8" s="121" t="s">
+      <c r="D8" s="166" t="s">
         <v>99</v>
       </c>
-      <c r="E8" s="122"/>
-      <c r="F8" s="117" t="s">
+      <c r="E8" s="167"/>
+      <c r="F8" s="166" t="s">
         <v>100</v>
       </c>
-      <c r="G8" s="113"/>
-      <c r="H8" s="114" t="s">
+      <c r="G8" s="167"/>
+      <c r="H8" s="166" t="s">
         <v>101</v>
       </c>
-      <c r="I8" s="115"/>
-      <c r="J8" s="113"/>
-      <c r="K8" s="114" t="s">
+      <c r="I8" s="185"/>
+      <c r="J8" s="167"/>
+      <c r="K8" s="166" t="s">
         <v>102</v>
       </c>
-      <c r="L8" s="116"/>
-      <c r="M8" s="60"/>
-      <c r="N8" s="15"/>
-      <c r="O8" s="15"/>
+      <c r="L8" s="185"/>
+      <c r="M8" s="185"/>
+      <c r="N8" s="167"/>
     </row>
     <row r="9" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="32"/>
       <c r="B9" s="32"/>
       <c r="C9" s="32"/>
-      <c r="D9" s="113"/>
-      <c r="E9" s="115"/>
-      <c r="F9" s="118"/>
-      <c r="G9" s="113"/>
-      <c r="H9" s="119"/>
-      <c r="I9" s="115"/>
-      <c r="J9" s="113"/>
-      <c r="K9" s="59"/>
-      <c r="L9" s="59"/>
-      <c r="M9" s="120"/>
-      <c r="N9" s="14"/>
-      <c r="O9" s="14"/>
+      <c r="D9" s="182"/>
+      <c r="E9" s="184"/>
+      <c r="F9" s="182"/>
+      <c r="G9" s="184"/>
+      <c r="H9" s="182"/>
+      <c r="I9" s="183"/>
+      <c r="J9" s="184"/>
+      <c r="K9" s="182"/>
+      <c r="L9" s="183"/>
+      <c r="M9" s="183"/>
+      <c r="N9" s="184"/>
     </row>
     <row r="10" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="32"/>
@@ -2417,46 +2403,46 @@
       <c r="O10" s="35"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="132" t="s">
+      <c r="A11" s="175" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="133"/>
-      <c r="C11" s="133"/>
-      <c r="D11" s="133"/>
-      <c r="E11" s="133"/>
-      <c r="F11" s="133"/>
-      <c r="G11" s="133"/>
-      <c r="H11" s="133"/>
-      <c r="I11" s="133"/>
-      <c r="J11" s="133"/>
-      <c r="K11" s="133"/>
-      <c r="L11" s="133"/>
-      <c r="M11" s="133"/>
-      <c r="N11" s="133"/>
-      <c r="O11" s="133"/>
-      <c r="P11" s="133"/>
-      <c r="Q11" s="134"/>
+      <c r="B11" s="176"/>
+      <c r="C11" s="176"/>
+      <c r="D11" s="176"/>
+      <c r="E11" s="176"/>
+      <c r="F11" s="176"/>
+      <c r="G11" s="176"/>
+      <c r="H11" s="176"/>
+      <c r="I11" s="176"/>
+      <c r="J11" s="176"/>
+      <c r="K11" s="176"/>
+      <c r="L11" s="176"/>
+      <c r="M11" s="176"/>
+      <c r="N11" s="176"/>
+      <c r="O11" s="176"/>
+      <c r="P11" s="176"/>
+      <c r="Q11" s="177"/>
     </row>
     <row r="12" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="135" t="s">
+      <c r="A12" s="178" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="136"/>
-      <c r="C12" s="136"/>
-      <c r="D12" s="136"/>
-      <c r="E12" s="136"/>
-      <c r="F12" s="136"/>
-      <c r="G12" s="136"/>
-      <c r="H12" s="136"/>
-      <c r="I12" s="136"/>
-      <c r="J12" s="136"/>
-      <c r="K12" s="136"/>
-      <c r="L12" s="136"/>
-      <c r="M12" s="136"/>
-      <c r="N12" s="136"/>
-      <c r="O12" s="136"/>
-      <c r="P12" s="136"/>
-      <c r="Q12" s="137"/>
+      <c r="B12" s="179"/>
+      <c r="C12" s="179"/>
+      <c r="D12" s="179"/>
+      <c r="E12" s="179"/>
+      <c r="F12" s="179"/>
+      <c r="G12" s="179"/>
+      <c r="H12" s="179"/>
+      <c r="I12" s="179"/>
+      <c r="J12" s="179"/>
+      <c r="K12" s="179"/>
+      <c r="L12" s="179"/>
+      <c r="M12" s="179"/>
+      <c r="N12" s="179"/>
+      <c r="O12" s="179"/>
+      <c r="P12" s="179"/>
+      <c r="Q12" s="180"/>
     </row>
     <row r="13" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="36"/>
@@ -2484,8 +2470,8 @@
       <c r="B14" s="14"/>
       <c r="C14" s="43"/>
       <c r="D14" s="14"/>
-      <c r="E14" s="183"/>
-      <c r="F14" s="183"/>
+      <c r="E14" s="119"/>
+      <c r="F14" s="119"/>
       <c r="G14" s="87" t="s">
         <v>23</v>
       </c>
@@ -2495,8 +2481,8 @@
       <c r="N14" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="O14" s="181"/>
-      <c r="P14" s="182"/>
+      <c r="O14" s="117"/>
+      <c r="P14" s="118"/>
       <c r="Q14" s="27"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2506,8 +2492,8 @@
       <c r="B15" s="14"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
-      <c r="E15" s="183"/>
-      <c r="F15" s="183"/>
+      <c r="E15" s="119"/>
+      <c r="F15" s="119"/>
       <c r="G15" s="87" t="s">
         <v>25</v>
       </c>
@@ -2517,8 +2503,8 @@
       <c r="N15" s="45" t="s">
         <v>68</v>
       </c>
-      <c r="O15" s="181"/>
-      <c r="P15" s="182"/>
+      <c r="O15" s="117"/>
+      <c r="P15" s="118"/>
       <c r="Q15" s="27"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2538,8 +2524,8 @@
       <c r="N16" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="O16" s="181"/>
-      <c r="P16" s="182"/>
+      <c r="O16" s="117"/>
+      <c r="P16" s="118"/>
       <c r="Q16" s="27"/>
     </row>
     <row r="17" spans="1:20" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
@@ -2557,8 +2543,8 @@
       <c r="N17" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="O17" s="181"/>
-      <c r="P17" s="182"/>
+      <c r="O17" s="117"/>
+      <c r="P17" s="118"/>
       <c r="Q17" s="27"/>
     </row>
     <row r="18" spans="1:20" ht="6" customHeight="1" x14ac:dyDescent="0.2">
@@ -2589,8 +2575,8 @@
       <c r="D19" s="90"/>
       <c r="E19" s="98"/>
       <c r="F19" s="98"/>
-      <c r="G19" s="187"/>
-      <c r="H19" s="187"/>
+      <c r="G19" s="130"/>
+      <c r="H19" s="130"/>
       <c r="I19" s="91"/>
       <c r="J19" s="91"/>
       <c r="K19" s="90"/>
@@ -2608,381 +2594,381 @@
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
       <c r="D20" s="48"/>
-      <c r="E20" s="154" t="s">
+      <c r="E20" s="153" t="s">
         <v>36</v>
       </c>
-      <c r="F20" s="154"/>
-      <c r="G20" s="154"/>
-      <c r="H20" s="154"/>
-      <c r="I20" s="154"/>
-      <c r="J20" s="154"/>
-      <c r="K20" s="154"/>
-      <c r="L20" s="154"/>
-      <c r="M20" s="154"/>
-      <c r="N20" s="154"/>
-      <c r="O20" s="154"/>
-      <c r="P20" s="154"/>
-      <c r="Q20" s="155"/>
+      <c r="F20" s="153"/>
+      <c r="G20" s="153"/>
+      <c r="H20" s="153"/>
+      <c r="I20" s="153"/>
+      <c r="J20" s="153"/>
+      <c r="K20" s="153"/>
+      <c r="L20" s="153"/>
+      <c r="M20" s="153"/>
+      <c r="N20" s="153"/>
+      <c r="O20" s="153"/>
+      <c r="P20" s="153"/>
+      <c r="Q20" s="154"/>
     </row>
     <row r="21" spans="1:20" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="141" t="s">
+      <c r="A21" s="162" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="141"/>
-      <c r="C21" s="141"/>
-      <c r="D21" s="141" t="s">
+      <c r="B21" s="162"/>
+      <c r="C21" s="162"/>
+      <c r="D21" s="162" t="s">
         <v>27</v>
       </c>
-      <c r="E21" s="141"/>
-      <c r="F21" s="141"/>
-      <c r="G21" s="141"/>
-      <c r="H21" s="141" t="s">
+      <c r="E21" s="162"/>
+      <c r="F21" s="162"/>
+      <c r="G21" s="162"/>
+      <c r="H21" s="162" t="s">
         <v>28</v>
       </c>
-      <c r="I21" s="141"/>
-      <c r="J21" s="141"/>
-      <c r="K21" s="141"/>
-      <c r="L21" s="141" t="s">
+      <c r="I21" s="162"/>
+      <c r="J21" s="162"/>
+      <c r="K21" s="162"/>
+      <c r="L21" s="162" t="s">
         <v>29</v>
       </c>
-      <c r="M21" s="141"/>
-      <c r="N21" s="141"/>
-      <c r="O21" s="141"/>
-      <c r="P21" s="141"/>
-      <c r="Q21" s="141"/>
+      <c r="M21" s="162"/>
+      <c r="N21" s="162"/>
+      <c r="O21" s="162"/>
+      <c r="P21" s="162"/>
+      <c r="Q21" s="162"/>
       <c r="R21" s="13"/>
     </row>
     <row r="22" spans="1:20" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="141" t="s">
+      <c r="A22" s="162" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="141"/>
-      <c r="C22" s="141"/>
-      <c r="D22" s="141" t="s">
+      <c r="B22" s="162"/>
+      <c r="C22" s="162"/>
+      <c r="D22" s="162" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="141"/>
-      <c r="F22" s="141" t="s">
+      <c r="E22" s="162"/>
+      <c r="F22" s="162" t="s">
         <v>32</v>
       </c>
-      <c r="G22" s="141"/>
-      <c r="H22" s="141" t="s">
+      <c r="G22" s="162"/>
+      <c r="H22" s="162" t="s">
         <v>31</v>
       </c>
-      <c r="I22" s="141"/>
-      <c r="J22" s="141" t="s">
+      <c r="I22" s="162"/>
+      <c r="J22" s="162" t="s">
         <v>32</v>
       </c>
-      <c r="K22" s="141"/>
-      <c r="L22" s="141" t="s">
+      <c r="K22" s="162"/>
+      <c r="L22" s="162" t="s">
         <v>31</v>
       </c>
-      <c r="M22" s="141"/>
-      <c r="N22" s="141"/>
-      <c r="O22" s="141" t="s">
+      <c r="M22" s="162"/>
+      <c r="N22" s="162"/>
+      <c r="O22" s="162" t="s">
         <v>32</v>
       </c>
-      <c r="P22" s="141"/>
-      <c r="Q22" s="141"/>
+      <c r="P22" s="162"/>
+      <c r="Q22" s="162"/>
       <c r="R22" s="13"/>
     </row>
     <row r="23" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="145" t="s">
+      <c r="A23" s="146" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="145"/>
-      <c r="C23" s="145"/>
-      <c r="D23" s="129" t="s">
+      <c r="B23" s="146"/>
+      <c r="C23" s="146"/>
+      <c r="D23" s="163" t="s">
         <v>97</v>
       </c>
-      <c r="E23" s="129"/>
-      <c r="F23" s="129"/>
-      <c r="G23" s="129"/>
-      <c r="H23" s="130">
+      <c r="E23" s="163"/>
+      <c r="F23" s="163"/>
+      <c r="G23" s="163"/>
+      <c r="H23" s="139">
         <v>25</v>
       </c>
-      <c r="I23" s="130"/>
-      <c r="J23" s="130"/>
-      <c r="K23" s="130"/>
-      <c r="L23" s="130">
+      <c r="I23" s="139"/>
+      <c r="J23" s="139"/>
+      <c r="K23" s="139"/>
+      <c r="L23" s="139">
         <v>10</v>
       </c>
-      <c r="M23" s="130"/>
-      <c r="N23" s="130"/>
-      <c r="O23" s="130"/>
-      <c r="P23" s="130"/>
-      <c r="Q23" s="130"/>
+      <c r="M23" s="139"/>
+      <c r="N23" s="139"/>
+      <c r="O23" s="139"/>
+      <c r="P23" s="139"/>
+      <c r="Q23" s="139"/>
     </row>
     <row r="24" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="145" t="s">
+      <c r="A24" s="146" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="145"/>
-      <c r="C24" s="145"/>
-      <c r="D24" s="129" t="s">
+      <c r="B24" s="146"/>
+      <c r="C24" s="146"/>
+      <c r="D24" s="163" t="s">
         <v>98</v>
       </c>
-      <c r="E24" s="129"/>
-      <c r="F24" s="129"/>
-      <c r="G24" s="129"/>
-      <c r="H24" s="129" t="s">
+      <c r="E24" s="163"/>
+      <c r="F24" s="163"/>
+      <c r="G24" s="163"/>
+      <c r="H24" s="163" t="s">
         <v>98</v>
       </c>
-      <c r="I24" s="129"/>
-      <c r="J24" s="129"/>
-      <c r="K24" s="129"/>
-      <c r="L24" s="130" t="s">
+      <c r="I24" s="163"/>
+      <c r="J24" s="163"/>
+      <c r="K24" s="163"/>
+      <c r="L24" s="139" t="s">
         <v>98</v>
       </c>
-      <c r="M24" s="130"/>
-      <c r="N24" s="130"/>
-      <c r="O24" s="130"/>
-      <c r="P24" s="130"/>
-      <c r="Q24" s="130"/>
+      <c r="M24" s="139"/>
+      <c r="N24" s="139"/>
+      <c r="O24" s="139"/>
+      <c r="P24" s="139"/>
+      <c r="Q24" s="139"/>
     </row>
     <row r="25" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="156" t="s">
+      <c r="A25" s="155" t="s">
         <v>69</v>
       </c>
-      <c r="B25" s="157"/>
-      <c r="C25" s="158"/>
-      <c r="D25" s="148"/>
-      <c r="E25" s="149"/>
-      <c r="F25" s="149"/>
-      <c r="G25" s="150"/>
-      <c r="H25" s="148"/>
-      <c r="I25" s="149"/>
-      <c r="J25" s="149"/>
-      <c r="K25" s="150"/>
-      <c r="L25" s="142"/>
-      <c r="M25" s="143"/>
-      <c r="N25" s="143"/>
-      <c r="O25" s="143"/>
-      <c r="P25" s="143"/>
-      <c r="Q25" s="144"/>
+      <c r="B25" s="156"/>
+      <c r="C25" s="157"/>
+      <c r="D25" s="140"/>
+      <c r="E25" s="142"/>
+      <c r="F25" s="142"/>
+      <c r="G25" s="141"/>
+      <c r="H25" s="140"/>
+      <c r="I25" s="142"/>
+      <c r="J25" s="142"/>
+      <c r="K25" s="141"/>
+      <c r="L25" s="136"/>
+      <c r="M25" s="137"/>
+      <c r="N25" s="137"/>
+      <c r="O25" s="137"/>
+      <c r="P25" s="137"/>
+      <c r="Q25" s="138"/>
     </row>
     <row r="26" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="156" t="s">
+      <c r="A26" s="155" t="s">
         <v>47</v>
       </c>
-      <c r="B26" s="157"/>
-      <c r="C26" s="158"/>
-      <c r="D26" s="148"/>
-      <c r="E26" s="149"/>
-      <c r="F26" s="149"/>
-      <c r="G26" s="150"/>
-      <c r="H26" s="148"/>
-      <c r="I26" s="149"/>
-      <c r="J26" s="149"/>
-      <c r="K26" s="150"/>
-      <c r="L26" s="142"/>
-      <c r="M26" s="143"/>
-      <c r="N26" s="143"/>
-      <c r="O26" s="143"/>
-      <c r="P26" s="143"/>
-      <c r="Q26" s="144"/>
+      <c r="B26" s="156"/>
+      <c r="C26" s="157"/>
+      <c r="D26" s="140"/>
+      <c r="E26" s="142"/>
+      <c r="F26" s="142"/>
+      <c r="G26" s="141"/>
+      <c r="H26" s="140"/>
+      <c r="I26" s="142"/>
+      <c r="J26" s="142"/>
+      <c r="K26" s="141"/>
+      <c r="L26" s="136"/>
+      <c r="M26" s="137"/>
+      <c r="N26" s="137"/>
+      <c r="O26" s="137"/>
+      <c r="P26" s="137"/>
+      <c r="Q26" s="138"/>
       <c r="S26"/>
       <c r="T26"/>
     </row>
     <row r="27" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="145" t="s">
+      <c r="A27" s="146" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="145"/>
-      <c r="C27" s="145"/>
-      <c r="D27" s="151"/>
-      <c r="E27" s="151"/>
-      <c r="F27" s="130"/>
-      <c r="G27" s="130"/>
-      <c r="H27" s="148"/>
-      <c r="I27" s="150"/>
-      <c r="J27" s="130"/>
-      <c r="K27" s="130"/>
-      <c r="L27" s="130"/>
-      <c r="M27" s="130"/>
-      <c r="N27" s="130"/>
-      <c r="O27" s="130"/>
-      <c r="P27" s="130"/>
-      <c r="Q27" s="130"/>
+      <c r="B27" s="146"/>
+      <c r="C27" s="146"/>
+      <c r="D27" s="145"/>
+      <c r="E27" s="145"/>
+      <c r="F27" s="139"/>
+      <c r="G27" s="139"/>
+      <c r="H27" s="140"/>
+      <c r="I27" s="141"/>
+      <c r="J27" s="139"/>
+      <c r="K27" s="139"/>
+      <c r="L27" s="139"/>
+      <c r="M27" s="139"/>
+      <c r="N27" s="139"/>
+      <c r="O27" s="139"/>
+      <c r="P27" s="139"/>
+      <c r="Q27" s="139"/>
       <c r="S27"/>
       <c r="T27"/>
     </row>
     <row r="28" spans="1:20" ht="11.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="159" t="s">
+      <c r="A28" s="158" t="s">
         <v>40</v>
       </c>
-      <c r="B28" s="160"/>
-      <c r="C28" s="160"/>
-      <c r="D28" s="160"/>
-      <c r="E28" s="160"/>
-      <c r="F28" s="160"/>
-      <c r="G28" s="160"/>
-      <c r="H28" s="160"/>
-      <c r="I28" s="160"/>
-      <c r="J28" s="160"/>
-      <c r="K28" s="160"/>
-      <c r="L28" s="160"/>
-      <c r="M28" s="160"/>
-      <c r="N28" s="160"/>
-      <c r="O28" s="160"/>
-      <c r="P28" s="160"/>
-      <c r="Q28" s="161"/>
+      <c r="B28" s="159"/>
+      <c r="C28" s="159"/>
+      <c r="D28" s="159"/>
+      <c r="E28" s="159"/>
+      <c r="F28" s="159"/>
+      <c r="G28" s="159"/>
+      <c r="H28" s="159"/>
+      <c r="I28" s="159"/>
+      <c r="J28" s="159"/>
+      <c r="K28" s="159"/>
+      <c r="L28" s="159"/>
+      <c r="M28" s="159"/>
+      <c r="N28" s="159"/>
+      <c r="O28" s="159"/>
+      <c r="P28" s="159"/>
+      <c r="Q28" s="160"/>
       <c r="S28"/>
       <c r="T28"/>
     </row>
     <row r="29" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="145" t="s">
+      <c r="A29" s="146" t="s">
         <v>48</v>
       </c>
-      <c r="B29" s="145"/>
-      <c r="C29" s="145"/>
-      <c r="D29" s="151"/>
-      <c r="E29" s="151"/>
-      <c r="F29" s="130"/>
-      <c r="G29" s="130"/>
-      <c r="H29" s="148"/>
-      <c r="I29" s="150"/>
-      <c r="J29" s="130"/>
-      <c r="K29" s="130"/>
-      <c r="L29" s="148"/>
-      <c r="M29" s="149"/>
-      <c r="N29" s="150"/>
-      <c r="O29" s="148"/>
-      <c r="P29" s="149"/>
-      <c r="Q29" s="150"/>
+      <c r="B29" s="146"/>
+      <c r="C29" s="146"/>
+      <c r="D29" s="145"/>
+      <c r="E29" s="145"/>
+      <c r="F29" s="139"/>
+      <c r="G29" s="139"/>
+      <c r="H29" s="140"/>
+      <c r="I29" s="141"/>
+      <c r="J29" s="139"/>
+      <c r="K29" s="139"/>
+      <c r="L29" s="140"/>
+      <c r="M29" s="142"/>
+      <c r="N29" s="141"/>
+      <c r="O29" s="140"/>
+      <c r="P29" s="142"/>
+      <c r="Q29" s="141"/>
       <c r="S29"/>
       <c r="T29"/>
     </row>
     <row r="30" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="145" t="s">
+      <c r="A30" s="146" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="145"/>
-      <c r="C30" s="145"/>
-      <c r="D30" s="151"/>
-      <c r="E30" s="151"/>
-      <c r="F30" s="130"/>
-      <c r="G30" s="130"/>
-      <c r="H30" s="148"/>
-      <c r="I30" s="150"/>
-      <c r="J30" s="130"/>
-      <c r="K30" s="130"/>
-      <c r="L30" s="148"/>
-      <c r="M30" s="149"/>
-      <c r="N30" s="150"/>
-      <c r="O30" s="148"/>
-      <c r="P30" s="149"/>
-      <c r="Q30" s="150"/>
+      <c r="B30" s="146"/>
+      <c r="C30" s="146"/>
+      <c r="D30" s="145"/>
+      <c r="E30" s="145"/>
+      <c r="F30" s="139"/>
+      <c r="G30" s="139"/>
+      <c r="H30" s="140"/>
+      <c r="I30" s="141"/>
+      <c r="J30" s="139"/>
+      <c r="K30" s="139"/>
+      <c r="L30" s="140"/>
+      <c r="M30" s="142"/>
+      <c r="N30" s="141"/>
+      <c r="O30" s="140"/>
+      <c r="P30" s="142"/>
+      <c r="Q30" s="141"/>
       <c r="S30"/>
       <c r="T30"/>
     </row>
     <row r="31" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="145" t="s">
+      <c r="A31" s="146" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="145"/>
-      <c r="C31" s="145"/>
-      <c r="D31" s="151"/>
-      <c r="E31" s="151"/>
-      <c r="F31" s="130"/>
-      <c r="G31" s="130"/>
-      <c r="H31" s="148"/>
-      <c r="I31" s="150"/>
-      <c r="J31" s="130"/>
-      <c r="K31" s="130"/>
-      <c r="L31" s="148"/>
-      <c r="M31" s="149"/>
-      <c r="N31" s="150"/>
-      <c r="O31" s="148"/>
-      <c r="P31" s="149"/>
-      <c r="Q31" s="150"/>
+      <c r="B31" s="146"/>
+      <c r="C31" s="146"/>
+      <c r="D31" s="145"/>
+      <c r="E31" s="145"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="140"/>
+      <c r="I31" s="141"/>
+      <c r="J31" s="139"/>
+      <c r="K31" s="139"/>
+      <c r="L31" s="140"/>
+      <c r="M31" s="142"/>
+      <c r="N31" s="141"/>
+      <c r="O31" s="140"/>
+      <c r="P31" s="142"/>
+      <c r="Q31" s="141"/>
       <c r="S31"/>
       <c r="T31"/>
     </row>
     <row r="32" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="162" t="s">
+      <c r="A32" s="161" t="s">
         <v>86</v>
       </c>
-      <c r="B32" s="162"/>
-      <c r="C32" s="162"/>
-      <c r="D32" s="151">
+      <c r="B32" s="161"/>
+      <c r="C32" s="161"/>
+      <c r="D32" s="145">
         <f>+D31-D30</f>
         <v>0</v>
       </c>
-      <c r="E32" s="151"/>
-      <c r="F32" s="151">
+      <c r="E32" s="145"/>
+      <c r="F32" s="145">
         <f>+F31-F30</f>
         <v>0</v>
       </c>
-      <c r="G32" s="151"/>
-      <c r="H32" s="151">
+      <c r="G32" s="145"/>
+      <c r="H32" s="145">
         <f>+H31-H30</f>
         <v>0</v>
       </c>
-      <c r="I32" s="151"/>
-      <c r="J32" s="151">
+      <c r="I32" s="145"/>
+      <c r="J32" s="145">
         <f>+J31-J30</f>
         <v>0</v>
       </c>
-      <c r="K32" s="151"/>
-      <c r="L32" s="142">
+      <c r="K32" s="145"/>
+      <c r="L32" s="136">
         <f>+L31-L30</f>
         <v>0</v>
       </c>
-      <c r="M32" s="143"/>
-      <c r="N32" s="144"/>
-      <c r="O32" s="142">
+      <c r="M32" s="137"/>
+      <c r="N32" s="138"/>
+      <c r="O32" s="136">
         <f>+O31-O30</f>
         <v>0</v>
       </c>
-      <c r="P32" s="143"/>
-      <c r="Q32" s="144"/>
+      <c r="P32" s="137"/>
+      <c r="Q32" s="138"/>
       <c r="S32"/>
       <c r="T32"/>
     </row>
     <row r="33" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="145" t="s">
+      <c r="A33" s="146" t="s">
         <v>51</v>
       </c>
-      <c r="B33" s="145"/>
-      <c r="C33" s="145"/>
-      <c r="D33" s="151"/>
-      <c r="E33" s="151"/>
-      <c r="F33" s="130"/>
-      <c r="G33" s="130"/>
-      <c r="H33" s="148"/>
-      <c r="I33" s="150"/>
-      <c r="J33" s="130"/>
-      <c r="K33" s="130"/>
-      <c r="L33" s="148"/>
-      <c r="M33" s="149"/>
-      <c r="N33" s="150"/>
-      <c r="O33" s="148"/>
-      <c r="P33" s="149"/>
-      <c r="Q33" s="150"/>
+      <c r="B33" s="146"/>
+      <c r="C33" s="146"/>
+      <c r="D33" s="145"/>
+      <c r="E33" s="145"/>
+      <c r="F33" s="139"/>
+      <c r="G33" s="139"/>
+      <c r="H33" s="140"/>
+      <c r="I33" s="141"/>
+      <c r="J33" s="139"/>
+      <c r="K33" s="139"/>
+      <c r="L33" s="140"/>
+      <c r="M33" s="142"/>
+      <c r="N33" s="141"/>
+      <c r="O33" s="140"/>
+      <c r="P33" s="142"/>
+      <c r="Q33" s="141"/>
       <c r="S33"/>
       <c r="T33"/>
     </row>
     <row r="34" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="145" t="s">
+      <c r="A34" s="146" t="s">
         <v>52</v>
       </c>
-      <c r="B34" s="145"/>
-      <c r="C34" s="145"/>
-      <c r="D34" s="151"/>
-      <c r="E34" s="151"/>
-      <c r="F34" s="130"/>
-      <c r="G34" s="130"/>
-      <c r="H34" s="148"/>
-      <c r="I34" s="150"/>
-      <c r="J34" s="130"/>
-      <c r="K34" s="130"/>
-      <c r="L34" s="148"/>
-      <c r="M34" s="149"/>
-      <c r="N34" s="150"/>
-      <c r="O34" s="148"/>
-      <c r="P34" s="149"/>
-      <c r="Q34" s="150"/>
+      <c r="B34" s="146"/>
+      <c r="C34" s="146"/>
+      <c r="D34" s="145"/>
+      <c r="E34" s="145"/>
+      <c r="F34" s="139"/>
+      <c r="G34" s="139"/>
+      <c r="H34" s="140"/>
+      <c r="I34" s="141"/>
+      <c r="J34" s="139"/>
+      <c r="K34" s="139"/>
+      <c r="L34" s="140"/>
+      <c r="M34" s="142"/>
+      <c r="N34" s="141"/>
+      <c r="O34" s="140"/>
+      <c r="P34" s="142"/>
+      <c r="Q34" s="141"/>
       <c r="S34"/>
       <c r="T34"/>
     </row>
@@ -3033,65 +3019,65 @@
       <c r="T36"/>
     </row>
     <row r="37" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="165" t="s">
+      <c r="A37" s="147" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="138" t="s">
+      <c r="B37" s="113" t="s">
         <v>17</v>
       </c>
-      <c r="C37" s="140"/>
+      <c r="C37" s="114"/>
       <c r="D37" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E37" s="138" t="s">
+      <c r="E37" s="113" t="s">
         <v>45</v>
       </c>
-      <c r="F37" s="139"/>
-      <c r="G37" s="139"/>
-      <c r="H37" s="139"/>
-      <c r="I37" s="139"/>
-      <c r="J37" s="140"/>
+      <c r="F37" s="152"/>
+      <c r="G37" s="152"/>
+      <c r="H37" s="152"/>
+      <c r="I37" s="152"/>
+      <c r="J37" s="114"/>
       <c r="K37" s="49"/>
-      <c r="L37" s="188" t="s">
+      <c r="L37" s="131" t="s">
         <v>83</v>
       </c>
-      <c r="M37" s="188"/>
-      <c r="N37" s="188"/>
-      <c r="O37" s="188"/>
-      <c r="P37" s="188"/>
-      <c r="Q37" s="188"/>
+      <c r="M37" s="131"/>
+      <c r="N37" s="131"/>
+      <c r="O37" s="131"/>
+      <c r="P37" s="131"/>
+      <c r="Q37" s="131"/>
       <c r="S37"/>
       <c r="T37"/>
     </row>
     <row r="38" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="166"/>
-      <c r="B38" s="168" t="s">
+      <c r="A38" s="148"/>
+      <c r="B38" s="150" t="s">
         <v>70</v>
       </c>
-      <c r="C38" s="168" t="s">
+      <c r="C38" s="150" t="s">
         <v>71</v>
       </c>
       <c r="D38" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E38" s="170" t="s">
+      <c r="E38" s="126" t="s">
         <v>44</v>
       </c>
-      <c r="F38" s="171"/>
-      <c r="G38" s="170" t="s">
+      <c r="F38" s="127"/>
+      <c r="G38" s="126" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="171"/>
-      <c r="I38" s="170" t="s">
+      <c r="H38" s="127"/>
+      <c r="I38" s="126" t="s">
         <v>44</v>
       </c>
-      <c r="J38" s="171"/>
+      <c r="J38" s="127"/>
       <c r="K38" s="49"/>
-      <c r="L38" s="170" t="s">
+      <c r="L38" s="126" t="s">
         <v>19</v>
       </c>
-      <c r="M38" s="171"/>
-      <c r="N38" s="152" t="s">
+      <c r="M38" s="127"/>
+      <c r="N38" s="164" t="s">
         <v>34</v>
       </c>
       <c r="O38" s="73" t="s">
@@ -3107,27 +3093,27 @@
       <c r="T38"/>
     </row>
     <row r="39" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="167"/>
-      <c r="B39" s="169"/>
-      <c r="C39" s="169"/>
+      <c r="A39" s="149"/>
+      <c r="B39" s="151"/>
+      <c r="C39" s="151"/>
       <c r="D39" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="E39" s="172"/>
-      <c r="F39" s="173"/>
-      <c r="G39" s="172"/>
-      <c r="H39" s="173"/>
-      <c r="I39" s="172"/>
-      <c r="J39" s="173"/>
+      <c r="E39" s="128"/>
+      <c r="F39" s="129"/>
+      <c r="G39" s="128"/>
+      <c r="H39" s="129"/>
+      <c r="I39" s="128"/>
+      <c r="J39" s="129"/>
       <c r="K39" s="49"/>
-      <c r="L39" s="172"/>
-      <c r="M39" s="173"/>
-      <c r="N39" s="153"/>
-      <c r="O39" s="138" t="s">
+      <c r="L39" s="128"/>
+      <c r="M39" s="129"/>
+      <c r="N39" s="165"/>
+      <c r="O39" s="113" t="s">
         <v>73</v>
       </c>
-      <c r="P39" s="139"/>
-      <c r="Q39" s="140"/>
+      <c r="P39" s="152"/>
+      <c r="Q39" s="114"/>
       <c r="R39" s="50"/>
       <c r="S39"/>
       <c r="T39"/>
@@ -3143,15 +3129,15 @@
         <v>0</v>
       </c>
       <c r="D40" s="23"/>
-      <c r="E40" s="138"/>
-      <c r="F40" s="140"/>
-      <c r="G40" s="138"/>
-      <c r="H40" s="140"/>
-      <c r="I40" s="138"/>
-      <c r="J40" s="140"/>
+      <c r="E40" s="113"/>
+      <c r="F40" s="114"/>
+      <c r="G40" s="113"/>
+      <c r="H40" s="114"/>
+      <c r="I40" s="113"/>
+      <c r="J40" s="114"/>
       <c r="K40" s="49"/>
-      <c r="L40" s="146"/>
-      <c r="M40" s="147"/>
+      <c r="L40" s="143"/>
+      <c r="M40" s="144"/>
       <c r="N40" s="69"/>
       <c r="O40" s="102"/>
       <c r="P40" s="102"/>
@@ -3171,15 +3157,15 @@
         <v>0.64</v>
       </c>
       <c r="D41" s="23"/>
-      <c r="E41" s="138"/>
-      <c r="F41" s="140"/>
-      <c r="G41" s="138"/>
-      <c r="H41" s="140"/>
-      <c r="I41" s="138"/>
-      <c r="J41" s="140"/>
+      <c r="E41" s="113"/>
+      <c r="F41" s="114"/>
+      <c r="G41" s="113"/>
+      <c r="H41" s="114"/>
+      <c r="I41" s="113"/>
+      <c r="J41" s="114"/>
       <c r="K41" s="51"/>
-      <c r="L41" s="146"/>
-      <c r="M41" s="147"/>
+      <c r="L41" s="143"/>
+      <c r="M41" s="144"/>
       <c r="N41" s="69"/>
       <c r="O41" s="19"/>
       <c r="P41" s="19"/>
@@ -3199,15 +3185,15 @@
         <v>1.3</v>
       </c>
       <c r="D42" s="23"/>
-      <c r="E42" s="138"/>
-      <c r="F42" s="140"/>
-      <c r="G42" s="138"/>
-      <c r="H42" s="140"/>
-      <c r="I42" s="138"/>
-      <c r="J42" s="140"/>
+      <c r="E42" s="113"/>
+      <c r="F42" s="114"/>
+      <c r="G42" s="113"/>
+      <c r="H42" s="114"/>
+      <c r="I42" s="113"/>
+      <c r="J42" s="114"/>
       <c r="K42" s="51"/>
-      <c r="L42" s="146"/>
-      <c r="M42" s="147"/>
+      <c r="L42" s="143"/>
+      <c r="M42" s="144"/>
       <c r="N42" s="69"/>
       <c r="O42" s="19"/>
       <c r="P42" s="19"/>
@@ -3227,15 +3213,15 @@
         <v>1.9</v>
       </c>
       <c r="D43" s="23"/>
-      <c r="E43" s="138"/>
-      <c r="F43" s="140"/>
-      <c r="G43" s="138"/>
-      <c r="H43" s="140"/>
-      <c r="I43" s="138"/>
-      <c r="J43" s="140"/>
+      <c r="E43" s="113"/>
+      <c r="F43" s="114"/>
+      <c r="G43" s="113"/>
+      <c r="H43" s="114"/>
+      <c r="I43" s="113"/>
+      <c r="J43" s="114"/>
       <c r="K43" s="51"/>
-      <c r="L43" s="146"/>
-      <c r="M43" s="147"/>
+      <c r="L43" s="143"/>
+      <c r="M43" s="144"/>
       <c r="N43" s="69"/>
       <c r="O43" s="19"/>
       <c r="P43" s="19"/>
@@ -3257,15 +3243,15 @@
       <c r="D44" s="110">
         <v>1000</v>
       </c>
-      <c r="E44" s="163"/>
-      <c r="F44" s="164"/>
-      <c r="G44" s="163"/>
-      <c r="H44" s="164"/>
-      <c r="I44" s="163"/>
-      <c r="J44" s="164"/>
+      <c r="E44" s="115"/>
+      <c r="F44" s="116"/>
+      <c r="G44" s="115"/>
+      <c r="H44" s="116"/>
+      <c r="I44" s="115"/>
+      <c r="J44" s="116"/>
       <c r="K44" s="51"/>
-      <c r="L44" s="146"/>
-      <c r="M44" s="147"/>
+      <c r="L44" s="143"/>
+      <c r="M44" s="144"/>
       <c r="N44" s="69"/>
       <c r="O44" s="19"/>
       <c r="P44" s="19"/>
@@ -3285,12 +3271,12 @@
         <v>3.18</v>
       </c>
       <c r="D45" s="105"/>
-      <c r="E45" s="163"/>
-      <c r="F45" s="164"/>
-      <c r="G45" s="163"/>
-      <c r="H45" s="164"/>
-      <c r="I45" s="163"/>
-      <c r="J45" s="164"/>
+      <c r="E45" s="115"/>
+      <c r="F45" s="116"/>
+      <c r="G45" s="115"/>
+      <c r="H45" s="116"/>
+      <c r="I45" s="115"/>
+      <c r="J45" s="116"/>
       <c r="K45" s="51"/>
       <c r="L45" s="40"/>
       <c r="M45" s="40"/>
@@ -3313,23 +3299,23 @@
         <v>3.8</v>
       </c>
       <c r="D46" s="105"/>
-      <c r="E46" s="163"/>
-      <c r="F46" s="164"/>
-      <c r="G46" s="163"/>
-      <c r="H46" s="164"/>
-      <c r="I46" s="163"/>
-      <c r="J46" s="164"/>
+      <c r="E46" s="115"/>
+      <c r="F46" s="116"/>
+      <c r="G46" s="115"/>
+      <c r="H46" s="116"/>
+      <c r="I46" s="115"/>
+      <c r="J46" s="116"/>
       <c r="K46" s="51"/>
-      <c r="L46" s="184" t="s">
+      <c r="L46" s="120" t="s">
         <v>75</v>
       </c>
-      <c r="M46" s="185"/>
-      <c r="N46" s="186"/>
-      <c r="O46" s="178" t="s">
+      <c r="M46" s="121"/>
+      <c r="N46" s="122"/>
+      <c r="O46" s="133" t="s">
         <v>76</v>
       </c>
-      <c r="P46" s="178"/>
-      <c r="Q46" s="178"/>
+      <c r="P46" s="133"/>
+      <c r="Q46" s="133"/>
       <c r="R46" s="52"/>
       <c r="S46"/>
       <c r="T46"/>
@@ -3345,23 +3331,23 @@
         <v>4.45</v>
       </c>
       <c r="D47" s="105"/>
-      <c r="E47" s="163"/>
-      <c r="F47" s="164"/>
-      <c r="G47" s="163"/>
-      <c r="H47" s="164"/>
-      <c r="I47" s="163"/>
-      <c r="J47" s="164"/>
+      <c r="E47" s="115"/>
+      <c r="F47" s="116"/>
+      <c r="G47" s="115"/>
+      <c r="H47" s="116"/>
+      <c r="I47" s="115"/>
+      <c r="J47" s="116"/>
       <c r="K47" s="51"/>
-      <c r="L47" s="175" t="s">
+      <c r="L47" s="123" t="s">
         <v>80</v>
       </c>
-      <c r="M47" s="176"/>
-      <c r="N47" s="177"/>
-      <c r="O47" s="174" t="s">
+      <c r="M47" s="124"/>
+      <c r="N47" s="125"/>
+      <c r="O47" s="132" t="s">
         <v>90</v>
       </c>
-      <c r="P47" s="174"/>
-      <c r="Q47" s="174"/>
+      <c r="P47" s="132"/>
+      <c r="Q47" s="132"/>
       <c r="R47" s="52"/>
       <c r="S47"/>
       <c r="T47"/>
@@ -3379,23 +3365,23 @@
       <c r="D48" s="110">
         <v>1500</v>
       </c>
-      <c r="E48" s="163"/>
-      <c r="F48" s="164"/>
-      <c r="G48" s="163"/>
-      <c r="H48" s="164"/>
-      <c r="I48" s="163"/>
-      <c r="J48" s="164"/>
+      <c r="E48" s="115"/>
+      <c r="F48" s="116"/>
+      <c r="G48" s="115"/>
+      <c r="H48" s="116"/>
+      <c r="I48" s="115"/>
+      <c r="J48" s="116"/>
       <c r="K48" s="51"/>
-      <c r="L48" s="175" t="s">
+      <c r="L48" s="123" t="s">
         <v>81</v>
       </c>
-      <c r="M48" s="176"/>
-      <c r="N48" s="177"/>
-      <c r="O48" s="174" t="s">
+      <c r="M48" s="124"/>
+      <c r="N48" s="125"/>
+      <c r="O48" s="132" t="s">
         <v>91</v>
       </c>
-      <c r="P48" s="174"/>
-      <c r="Q48" s="174"/>
+      <c r="P48" s="132"/>
+      <c r="Q48" s="132"/>
       <c r="R48" s="52"/>
       <c r="S48"/>
       <c r="T48"/>
@@ -3411,23 +3397,23 @@
         <v>7.6</v>
       </c>
       <c r="D49" s="23"/>
-      <c r="E49" s="138"/>
-      <c r="F49" s="140"/>
-      <c r="G49" s="138"/>
-      <c r="H49" s="140"/>
-      <c r="I49" s="138"/>
-      <c r="J49" s="140"/>
+      <c r="E49" s="113"/>
+      <c r="F49" s="114"/>
+      <c r="G49" s="113"/>
+      <c r="H49" s="114"/>
+      <c r="I49" s="113"/>
+      <c r="J49" s="114"/>
       <c r="K49" s="53"/>
-      <c r="L49" s="175" t="s">
+      <c r="L49" s="123" t="s">
         <v>82</v>
       </c>
-      <c r="M49" s="176"/>
-      <c r="N49" s="177"/>
-      <c r="O49" s="174" t="s">
+      <c r="M49" s="124"/>
+      <c r="N49" s="125"/>
+      <c r="O49" s="132" t="s">
         <v>92</v>
       </c>
-      <c r="P49" s="174"/>
-      <c r="Q49" s="174"/>
+      <c r="P49" s="132"/>
+      <c r="Q49" s="132"/>
       <c r="R49" s="52"/>
       <c r="S49"/>
       <c r="T49"/>
@@ -3443,23 +3429,23 @@
         <v>10</v>
       </c>
       <c r="D50" s="23"/>
-      <c r="E50" s="138"/>
-      <c r="F50" s="140"/>
-      <c r="G50" s="138"/>
-      <c r="H50" s="140"/>
-      <c r="I50" s="138"/>
-      <c r="J50" s="140"/>
+      <c r="E50" s="113"/>
+      <c r="F50" s="114"/>
+      <c r="G50" s="113"/>
+      <c r="H50" s="114"/>
+      <c r="I50" s="113"/>
+      <c r="J50" s="114"/>
       <c r="K50" s="53"/>
       <c r="L50" s="74" t="s">
         <v>78</v>
       </c>
       <c r="M50" s="75"/>
       <c r="N50" s="76"/>
-      <c r="O50" s="174" t="s">
+      <c r="O50" s="132" t="s">
         <v>93</v>
       </c>
-      <c r="P50" s="174"/>
-      <c r="Q50" s="174"/>
+      <c r="P50" s="132"/>
+      <c r="Q50" s="132"/>
       <c r="R50" s="52"/>
       <c r="S50"/>
       <c r="T50"/>
@@ -3475,23 +3461,23 @@
         <v>13</v>
       </c>
       <c r="D51" s="23"/>
-      <c r="E51" s="138"/>
-      <c r="F51" s="140"/>
-      <c r="G51" s="138"/>
-      <c r="H51" s="140"/>
-      <c r="I51" s="138"/>
-      <c r="J51" s="140"/>
+      <c r="E51" s="113"/>
+      <c r="F51" s="114"/>
+      <c r="G51" s="113"/>
+      <c r="H51" s="114"/>
+      <c r="I51" s="113"/>
+      <c r="J51" s="114"/>
       <c r="K51" s="54"/>
       <c r="L51" s="74" t="s">
         <v>79</v>
       </c>
       <c r="M51" s="75"/>
       <c r="N51" s="76"/>
-      <c r="O51" s="174" t="s">
+      <c r="O51" s="132" t="s">
         <v>94</v>
       </c>
-      <c r="P51" s="174"/>
-      <c r="Q51" s="174"/>
+      <c r="P51" s="132"/>
+      <c r="Q51" s="132"/>
       <c r="R51" s="52"/>
       <c r="S51"/>
       <c r="T51"/>
@@ -3508,16 +3494,16 @@
       <c r="I52" s="57"/>
       <c r="J52" s="28"/>
       <c r="K52" s="14"/>
-      <c r="L52" s="175" t="s">
+      <c r="L52" s="123" t="s">
         <v>77</v>
       </c>
-      <c r="M52" s="176"/>
-      <c r="N52" s="177"/>
-      <c r="O52" s="174" t="s">
+      <c r="M52" s="124"/>
+      <c r="N52" s="125"/>
+      <c r="O52" s="132" t="s">
         <v>95</v>
       </c>
-      <c r="P52" s="174"/>
-      <c r="Q52" s="174"/>
+      <c r="P52" s="132"/>
+      <c r="Q52" s="132"/>
       <c r="S52"/>
       <c r="T52"/>
     </row>
@@ -3528,23 +3514,23 @@
       <c r="B53" s="59"/>
       <c r="C53" s="59"/>
       <c r="D53" s="60"/>
-      <c r="E53" s="138"/>
-      <c r="F53" s="140"/>
-      <c r="G53" s="138"/>
-      <c r="H53" s="140"/>
-      <c r="I53" s="179"/>
-      <c r="J53" s="180"/>
+      <c r="E53" s="113"/>
+      <c r="F53" s="114"/>
+      <c r="G53" s="113"/>
+      <c r="H53" s="114"/>
+      <c r="I53" s="134"/>
+      <c r="J53" s="135"/>
       <c r="K53" s="61"/>
-      <c r="L53" s="175" t="s">
+      <c r="L53" s="123" t="s">
         <v>84</v>
       </c>
-      <c r="M53" s="176"/>
-      <c r="N53" s="177"/>
-      <c r="O53" s="174" t="s">
+      <c r="M53" s="124"/>
+      <c r="N53" s="125"/>
+      <c r="O53" s="132" t="s">
         <v>96</v>
       </c>
-      <c r="P53" s="174"/>
-      <c r="Q53" s="174"/>
+      <c r="P53" s="132"/>
+      <c r="Q53" s="132"/>
       <c r="S53"/>
       <c r="T53"/>
     </row>
@@ -3677,25 +3663,25 @@
     </row>
     <row r="62" spans="1:20" ht="7.2" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="63" spans="1:20" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="131" t="s">
+      <c r="A63" s="174" t="s">
         <v>85</v>
       </c>
-      <c r="B63" s="131"/>
-      <c r="C63" s="131"/>
-      <c r="D63" s="131"/>
-      <c r="E63" s="131"/>
-      <c r="F63" s="131"/>
-      <c r="G63" s="131"/>
-      <c r="H63" s="131"/>
-      <c r="I63" s="131"/>
-      <c r="J63" s="131"/>
-      <c r="K63" s="131"/>
-      <c r="L63" s="131"/>
-      <c r="M63" s="131"/>
-      <c r="N63" s="131"/>
-      <c r="O63" s="131"/>
-      <c r="P63" s="131"/>
-      <c r="Q63" s="131"/>
+      <c r="B63" s="174"/>
+      <c r="C63" s="174"/>
+      <c r="D63" s="174"/>
+      <c r="E63" s="174"/>
+      <c r="F63" s="174"/>
+      <c r="G63" s="174"/>
+      <c r="H63" s="174"/>
+      <c r="I63" s="174"/>
+      <c r="J63" s="174"/>
+      <c r="K63" s="174"/>
+      <c r="L63" s="174"/>
+      <c r="M63" s="174"/>
+      <c r="N63" s="174"/>
+      <c r="O63" s="174"/>
+      <c r="P63" s="174"/>
+      <c r="Q63" s="174"/>
     </row>
     <row r="64" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="65" ht="15.9" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3704,26 +3690,127 @@
     <protectedRange sqref="C10 C13" name="Rango3_3_1_1_1_1_1_1_1_1"/>
     <protectedRange sqref="C8:C9" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
-  <mergeCells count="161">
-    <mergeCell ref="E49:F49"/>
-    <mergeCell ref="E50:F50"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="L46:N46"/>
-    <mergeCell ref="L47:N47"/>
-    <mergeCell ref="L48:N48"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="L38:M39"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="L37:Q37"/>
-    <mergeCell ref="E48:F48"/>
+  <mergeCells count="168">
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D2:Q2"/>
+    <mergeCell ref="D3:Q3"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="L24:Q24"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="L23:Q23"/>
+    <mergeCell ref="A63:Q63"/>
+    <mergeCell ref="A11:Q11"/>
+    <mergeCell ref="A12:Q12"/>
+    <mergeCell ref="O39:Q39"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="L21:Q21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="L25:Q25"/>
+    <mergeCell ref="L26:Q26"/>
+    <mergeCell ref="L22:N22"/>
+    <mergeCell ref="O22:Q22"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="L44:M44"/>
+    <mergeCell ref="O30:Q30"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="H26:K26"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="O33:Q33"/>
+    <mergeCell ref="N38:N39"/>
+    <mergeCell ref="O27:Q27"/>
+    <mergeCell ref="O29:Q29"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="J27:K27"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="E20:Q20"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="O31:Q31"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="A37:A39"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="E37:J37"/>
+    <mergeCell ref="E38:F39"/>
+    <mergeCell ref="G38:H39"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="G49:H49"/>
+    <mergeCell ref="G50:H50"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="O34:Q34"/>
+    <mergeCell ref="I38:J39"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="L43:M43"/>
     <mergeCell ref="E51:F51"/>
     <mergeCell ref="G40:H40"/>
     <mergeCell ref="O50:Q50"/>
@@ -3748,124 +3835,30 @@
     <mergeCell ref="I53:J53"/>
     <mergeCell ref="L49:N49"/>
     <mergeCell ref="L52:N52"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="L46:N46"/>
+    <mergeCell ref="L47:N47"/>
+    <mergeCell ref="L48:N48"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="L38:M39"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="L37:Q37"/>
+    <mergeCell ref="E48:F48"/>
     <mergeCell ref="L32:N32"/>
     <mergeCell ref="O32:Q32"/>
     <mergeCell ref="I40:J40"/>
     <mergeCell ref="G44:H44"/>
     <mergeCell ref="G45:H45"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="L34:N34"/>
-    <mergeCell ref="O34:Q34"/>
-    <mergeCell ref="I38:J39"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="L41:M41"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="L43:M43"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="G49:H49"/>
-    <mergeCell ref="G50:H50"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="A37:A39"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="E37:J37"/>
-    <mergeCell ref="E38:F39"/>
-    <mergeCell ref="G38:H39"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="O29:Q29"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="E20:Q20"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="A28:Q28"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="L44:M44"/>
-    <mergeCell ref="O30:Q30"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="H25:K25"/>
-    <mergeCell ref="H26:K26"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="O33:Q33"/>
-    <mergeCell ref="N38:N39"/>
-    <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D2:Q2"/>
-    <mergeCell ref="D3:Q3"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="L24:Q24"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="L23:Q23"/>
-    <mergeCell ref="A63:Q63"/>
-    <mergeCell ref="A11:Q11"/>
-    <mergeCell ref="A12:Q12"/>
-    <mergeCell ref="O39:Q39"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="L21:Q21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="L25:Q25"/>
-    <mergeCell ref="L26:Q26"/>
-    <mergeCell ref="L22:N22"/>
-    <mergeCell ref="O22:Q22"/>
-    <mergeCell ref="A21:C21"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.39370078740157483" top="0.78740157480314965" bottom="0" header="0" footer="0"/>
@@ -3891,10 +3884,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="189" t="s">
+      <c r="A2" s="181" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="189"/>
+      <c r="B2" s="181"/>
       <c r="C2" s="5" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
fix: update Excel footer template
</commit_message>
<xml_diff>
--- a/app/templates/Temp_CBR_ASTM.xlsx
+++ b/app/templates/Temp_CBR_ASTM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8715C8F-9907-45E4-ACB1-FDE61825F565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280D318E-027D-4178-AB49-43739CC68D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -359,9 +359,6 @@
 (visual) (in):</t>
   </si>
   <si>
-    <t>Versión: 02 (11-11-2024)</t>
-  </si>
-  <si>
     <t>EQP-0026</t>
   </si>
   <si>
@@ -399,6 +396,9 @@
   </si>
   <si>
     <t>REALIZADO</t>
+  </si>
+  <si>
+    <t>Versión: 02 (11-11-2026)</t>
   </si>
 </sst>
 </file>
@@ -1075,16 +1075,212 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="15" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="7" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1108,210 +1304,14 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="15" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2234,43 +2234,43 @@
       <c r="A2" s="81"/>
       <c r="B2" s="82"/>
       <c r="C2" s="83"/>
-      <c r="D2" s="168" t="s">
+      <c r="D2" s="119" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="169"/>
-      <c r="F2" s="169"/>
-      <c r="G2" s="169"/>
-      <c r="H2" s="169"/>
-      <c r="I2" s="169"/>
-      <c r="J2" s="169"/>
-      <c r="K2" s="169"/>
-      <c r="L2" s="169"/>
-      <c r="M2" s="169"/>
-      <c r="N2" s="169"/>
-      <c r="O2" s="169"/>
-      <c r="P2" s="169"/>
-      <c r="Q2" s="170"/>
+      <c r="E2" s="120"/>
+      <c r="F2" s="120"/>
+      <c r="G2" s="120"/>
+      <c r="H2" s="120"/>
+      <c r="I2" s="120"/>
+      <c r="J2" s="120"/>
+      <c r="K2" s="120"/>
+      <c r="L2" s="120"/>
+      <c r="M2" s="120"/>
+      <c r="N2" s="120"/>
+      <c r="O2" s="120"/>
+      <c r="P2" s="120"/>
+      <c r="Q2" s="121"/>
     </row>
     <row r="3" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="81"/>
       <c r="B3" s="82"/>
       <c r="C3" s="83"/>
-      <c r="D3" s="171" t="s">
+      <c r="D3" s="122" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="172"/>
-      <c r="F3" s="172"/>
-      <c r="G3" s="172"/>
-      <c r="H3" s="172"/>
-      <c r="I3" s="172"/>
-      <c r="J3" s="172"/>
-      <c r="K3" s="172"/>
-      <c r="L3" s="172"/>
-      <c r="M3" s="172"/>
-      <c r="N3" s="172"/>
-      <c r="O3" s="172"/>
-      <c r="P3" s="172"/>
-      <c r="Q3" s="173"/>
+      <c r="E3" s="123"/>
+      <c r="F3" s="123"/>
+      <c r="G3" s="123"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
+      <c r="L3" s="123"/>
+      <c r="M3" s="123"/>
+      <c r="N3" s="123"/>
+      <c r="O3" s="123"/>
+      <c r="P3" s="123"/>
+      <c r="Q3" s="124"/>
     </row>
     <row r="4" spans="1:17" ht="3" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="81"/>
@@ -2349,41 +2349,41 @@
     <row r="8" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="32"/>
       <c r="C8" s="32"/>
-      <c r="D8" s="166" t="s">
+      <c r="D8" s="113" t="s">
+        <v>98</v>
+      </c>
+      <c r="E8" s="114"/>
+      <c r="F8" s="113" t="s">
         <v>99</v>
       </c>
-      <c r="E8" s="167"/>
-      <c r="F8" s="166" t="s">
+      <c r="G8" s="114"/>
+      <c r="H8" s="113" t="s">
         <v>100</v>
       </c>
-      <c r="G8" s="167"/>
-      <c r="H8" s="166" t="s">
+      <c r="I8" s="118"/>
+      <c r="J8" s="114"/>
+      <c r="K8" s="113" t="s">
         <v>101</v>
       </c>
-      <c r="I8" s="185"/>
-      <c r="J8" s="167"/>
-      <c r="K8" s="166" t="s">
-        <v>102</v>
-      </c>
-      <c r="L8" s="185"/>
-      <c r="M8" s="185"/>
-      <c r="N8" s="167"/>
+      <c r="L8" s="118"/>
+      <c r="M8" s="118"/>
+      <c r="N8" s="114"/>
     </row>
     <row r="9" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="32"/>
       <c r="B9" s="32"/>
       <c r="C9" s="32"/>
-      <c r="D9" s="182"/>
-      <c r="E9" s="184"/>
-      <c r="F9" s="182"/>
-      <c r="G9" s="184"/>
-      <c r="H9" s="182"/>
-      <c r="I9" s="183"/>
-      <c r="J9" s="184"/>
-      <c r="K9" s="182"/>
-      <c r="L9" s="183"/>
-      <c r="M9" s="183"/>
-      <c r="N9" s="184"/>
+      <c r="D9" s="115"/>
+      <c r="E9" s="116"/>
+      <c r="F9" s="115"/>
+      <c r="G9" s="116"/>
+      <c r="H9" s="115"/>
+      <c r="I9" s="117"/>
+      <c r="J9" s="116"/>
+      <c r="K9" s="115"/>
+      <c r="L9" s="117"/>
+      <c r="M9" s="117"/>
+      <c r="N9" s="116"/>
     </row>
     <row r="10" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="32"/>
@@ -2403,46 +2403,46 @@
       <c r="O10" s="35"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="175" t="s">
+      <c r="A11" s="128" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="176"/>
-      <c r="C11" s="176"/>
-      <c r="D11" s="176"/>
-      <c r="E11" s="176"/>
-      <c r="F11" s="176"/>
-      <c r="G11" s="176"/>
-      <c r="H11" s="176"/>
-      <c r="I11" s="176"/>
-      <c r="J11" s="176"/>
-      <c r="K11" s="176"/>
-      <c r="L11" s="176"/>
-      <c r="M11" s="176"/>
-      <c r="N11" s="176"/>
-      <c r="O11" s="176"/>
-      <c r="P11" s="176"/>
-      <c r="Q11" s="177"/>
+      <c r="B11" s="129"/>
+      <c r="C11" s="129"/>
+      <c r="D11" s="129"/>
+      <c r="E11" s="129"/>
+      <c r="F11" s="129"/>
+      <c r="G11" s="129"/>
+      <c r="H11" s="129"/>
+      <c r="I11" s="129"/>
+      <c r="J11" s="129"/>
+      <c r="K11" s="129"/>
+      <c r="L11" s="129"/>
+      <c r="M11" s="129"/>
+      <c r="N11" s="129"/>
+      <c r="O11" s="129"/>
+      <c r="P11" s="129"/>
+      <c r="Q11" s="130"/>
     </row>
     <row r="12" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="178" t="s">
+      <c r="A12" s="131" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="179"/>
-      <c r="C12" s="179"/>
-      <c r="D12" s="179"/>
-      <c r="E12" s="179"/>
-      <c r="F12" s="179"/>
-      <c r="G12" s="179"/>
-      <c r="H12" s="179"/>
-      <c r="I12" s="179"/>
-      <c r="J12" s="179"/>
-      <c r="K12" s="179"/>
-      <c r="L12" s="179"/>
-      <c r="M12" s="179"/>
-      <c r="N12" s="179"/>
-      <c r="O12" s="179"/>
-      <c r="P12" s="179"/>
-      <c r="Q12" s="180"/>
+      <c r="B12" s="132"/>
+      <c r="C12" s="132"/>
+      <c r="D12" s="132"/>
+      <c r="E12" s="132"/>
+      <c r="F12" s="132"/>
+      <c r="G12" s="132"/>
+      <c r="H12" s="132"/>
+      <c r="I12" s="132"/>
+      <c r="J12" s="132"/>
+      <c r="K12" s="132"/>
+      <c r="L12" s="132"/>
+      <c r="M12" s="132"/>
+      <c r="N12" s="132"/>
+      <c r="O12" s="132"/>
+      <c r="P12" s="132"/>
+      <c r="Q12" s="133"/>
     </row>
     <row r="13" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="36"/>
@@ -2470,8 +2470,8 @@
       <c r="B14" s="14"/>
       <c r="C14" s="43"/>
       <c r="D14" s="14"/>
-      <c r="E14" s="119"/>
-      <c r="F14" s="119"/>
+      <c r="E14" s="179"/>
+      <c r="F14" s="179"/>
       <c r="G14" s="87" t="s">
         <v>23</v>
       </c>
@@ -2481,8 +2481,8 @@
       <c r="N14" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="O14" s="117"/>
-      <c r="P14" s="118"/>
+      <c r="O14" s="177"/>
+      <c r="P14" s="178"/>
       <c r="Q14" s="27"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2492,8 +2492,8 @@
       <c r="B15" s="14"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
-      <c r="E15" s="119"/>
-      <c r="F15" s="119"/>
+      <c r="E15" s="179"/>
+      <c r="F15" s="179"/>
       <c r="G15" s="87" t="s">
         <v>25</v>
       </c>
@@ -2503,8 +2503,8 @@
       <c r="N15" s="45" t="s">
         <v>68</v>
       </c>
-      <c r="O15" s="117"/>
-      <c r="P15" s="118"/>
+      <c r="O15" s="177"/>
+      <c r="P15" s="178"/>
       <c r="Q15" s="27"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2524,8 +2524,8 @@
       <c r="N16" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="O16" s="117"/>
-      <c r="P16" s="118"/>
+      <c r="O16" s="177"/>
+      <c r="P16" s="178"/>
       <c r="Q16" s="27"/>
     </row>
     <row r="17" spans="1:20" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
@@ -2543,8 +2543,8 @@
       <c r="N17" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="O17" s="117"/>
-      <c r="P17" s="118"/>
+      <c r="O17" s="177"/>
+      <c r="P17" s="178"/>
       <c r="Q17" s="27"/>
     </row>
     <row r="18" spans="1:20" ht="6" customHeight="1" x14ac:dyDescent="0.2">
@@ -2575,8 +2575,8 @@
       <c r="D19" s="90"/>
       <c r="E19" s="98"/>
       <c r="F19" s="98"/>
-      <c r="G19" s="130"/>
-      <c r="H19" s="130"/>
+      <c r="G19" s="183"/>
+      <c r="H19" s="183"/>
       <c r="I19" s="91"/>
       <c r="J19" s="91"/>
       <c r="K19" s="90"/>
@@ -2594,381 +2594,381 @@
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
       <c r="D20" s="48"/>
-      <c r="E20" s="153" t="s">
+      <c r="E20" s="150" t="s">
         <v>36</v>
       </c>
-      <c r="F20" s="153"/>
-      <c r="G20" s="153"/>
-      <c r="H20" s="153"/>
-      <c r="I20" s="153"/>
-      <c r="J20" s="153"/>
-      <c r="K20" s="153"/>
-      <c r="L20" s="153"/>
-      <c r="M20" s="153"/>
-      <c r="N20" s="153"/>
-      <c r="O20" s="153"/>
-      <c r="P20" s="153"/>
-      <c r="Q20" s="154"/>
+      <c r="F20" s="150"/>
+      <c r="G20" s="150"/>
+      <c r="H20" s="150"/>
+      <c r="I20" s="150"/>
+      <c r="J20" s="150"/>
+      <c r="K20" s="150"/>
+      <c r="L20" s="150"/>
+      <c r="M20" s="150"/>
+      <c r="N20" s="150"/>
+      <c r="O20" s="150"/>
+      <c r="P20" s="150"/>
+      <c r="Q20" s="151"/>
     </row>
     <row r="21" spans="1:20" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="162" t="s">
+      <c r="A21" s="137" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="162"/>
-      <c r="C21" s="162"/>
-      <c r="D21" s="162" t="s">
+      <c r="B21" s="137"/>
+      <c r="C21" s="137"/>
+      <c r="D21" s="137" t="s">
         <v>27</v>
       </c>
-      <c r="E21" s="162"/>
-      <c r="F21" s="162"/>
-      <c r="G21" s="162"/>
-      <c r="H21" s="162" t="s">
+      <c r="E21" s="137"/>
+      <c r="F21" s="137"/>
+      <c r="G21" s="137"/>
+      <c r="H21" s="137" t="s">
         <v>28</v>
       </c>
-      <c r="I21" s="162"/>
-      <c r="J21" s="162"/>
-      <c r="K21" s="162"/>
-      <c r="L21" s="162" t="s">
+      <c r="I21" s="137"/>
+      <c r="J21" s="137"/>
+      <c r="K21" s="137"/>
+      <c r="L21" s="137" t="s">
         <v>29</v>
       </c>
-      <c r="M21" s="162"/>
-      <c r="N21" s="162"/>
-      <c r="O21" s="162"/>
-      <c r="P21" s="162"/>
-      <c r="Q21" s="162"/>
+      <c r="M21" s="137"/>
+      <c r="N21" s="137"/>
+      <c r="O21" s="137"/>
+      <c r="P21" s="137"/>
+      <c r="Q21" s="137"/>
       <c r="R21" s="13"/>
     </row>
     <row r="22" spans="1:20" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="162" t="s">
+      <c r="A22" s="137" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="162"/>
-      <c r="C22" s="162"/>
-      <c r="D22" s="162" t="s">
+      <c r="B22" s="137"/>
+      <c r="C22" s="137"/>
+      <c r="D22" s="137" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="162"/>
-      <c r="F22" s="162" t="s">
+      <c r="E22" s="137"/>
+      <c r="F22" s="137" t="s">
         <v>32</v>
       </c>
-      <c r="G22" s="162"/>
-      <c r="H22" s="162" t="s">
+      <c r="G22" s="137"/>
+      <c r="H22" s="137" t="s">
         <v>31</v>
       </c>
-      <c r="I22" s="162"/>
-      <c r="J22" s="162" t="s">
+      <c r="I22" s="137"/>
+      <c r="J22" s="137" t="s">
         <v>32</v>
       </c>
-      <c r="K22" s="162"/>
-      <c r="L22" s="162" t="s">
+      <c r="K22" s="137"/>
+      <c r="L22" s="137" t="s">
         <v>31</v>
       </c>
-      <c r="M22" s="162"/>
-      <c r="N22" s="162"/>
-      <c r="O22" s="162" t="s">
+      <c r="M22" s="137"/>
+      <c r="N22" s="137"/>
+      <c r="O22" s="137" t="s">
         <v>32</v>
       </c>
-      <c r="P22" s="162"/>
-      <c r="Q22" s="162"/>
+      <c r="P22" s="137"/>
+      <c r="Q22" s="137"/>
       <c r="R22" s="13"/>
     </row>
     <row r="23" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="146" t="s">
+      <c r="A23" s="141" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="146"/>
-      <c r="C23" s="146"/>
-      <c r="D23" s="163" t="s">
+      <c r="B23" s="141"/>
+      <c r="C23" s="141"/>
+      <c r="D23" s="125" t="s">
+        <v>96</v>
+      </c>
+      <c r="E23" s="125"/>
+      <c r="F23" s="125"/>
+      <c r="G23" s="125"/>
+      <c r="H23" s="126">
+        <v>25</v>
+      </c>
+      <c r="I23" s="126"/>
+      <c r="J23" s="126"/>
+      <c r="K23" s="126"/>
+      <c r="L23" s="126">
+        <v>10</v>
+      </c>
+      <c r="M23" s="126"/>
+      <c r="N23" s="126"/>
+      <c r="O23" s="126"/>
+      <c r="P23" s="126"/>
+      <c r="Q23" s="126"/>
+    </row>
+    <row r="24" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A24" s="141" t="s">
+        <v>33</v>
+      </c>
+      <c r="B24" s="141"/>
+      <c r="C24" s="141"/>
+      <c r="D24" s="125" t="s">
         <v>97</v>
       </c>
-      <c r="E23" s="163"/>
-      <c r="F23" s="163"/>
-      <c r="G23" s="163"/>
-      <c r="H23" s="139">
-        <v>25</v>
-      </c>
-      <c r="I23" s="139"/>
-      <c r="J23" s="139"/>
-      <c r="K23" s="139"/>
-      <c r="L23" s="139">
-        <v>10</v>
-      </c>
-      <c r="M23" s="139"/>
-      <c r="N23" s="139"/>
-      <c r="O23" s="139"/>
-      <c r="P23" s="139"/>
-      <c r="Q23" s="139"/>
-    </row>
-    <row r="24" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="146" t="s">
-        <v>33</v>
-      </c>
-      <c r="B24" s="146"/>
-      <c r="C24" s="146"/>
-      <c r="D24" s="163" t="s">
-        <v>98</v>
-      </c>
-      <c r="E24" s="163"/>
-      <c r="F24" s="163"/>
-      <c r="G24" s="163"/>
-      <c r="H24" s="163" t="s">
-        <v>98</v>
-      </c>
-      <c r="I24" s="163"/>
-      <c r="J24" s="163"/>
-      <c r="K24" s="163"/>
-      <c r="L24" s="139" t="s">
-        <v>98</v>
-      </c>
-      <c r="M24" s="139"/>
-      <c r="N24" s="139"/>
-      <c r="O24" s="139"/>
-      <c r="P24" s="139"/>
-      <c r="Q24" s="139"/>
+      <c r="E24" s="125"/>
+      <c r="F24" s="125"/>
+      <c r="G24" s="125"/>
+      <c r="H24" s="125" t="s">
+        <v>97</v>
+      </c>
+      <c r="I24" s="125"/>
+      <c r="J24" s="125"/>
+      <c r="K24" s="125"/>
+      <c r="L24" s="126" t="s">
+        <v>97</v>
+      </c>
+      <c r="M24" s="126"/>
+      <c r="N24" s="126"/>
+      <c r="O24" s="126"/>
+      <c r="P24" s="126"/>
+      <c r="Q24" s="126"/>
     </row>
     <row r="25" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="155" t="s">
+      <c r="A25" s="152" t="s">
         <v>69</v>
       </c>
-      <c r="B25" s="156"/>
-      <c r="C25" s="157"/>
-      <c r="D25" s="140"/>
-      <c r="E25" s="142"/>
-      <c r="F25" s="142"/>
-      <c r="G25" s="141"/>
-      <c r="H25" s="140"/>
-      <c r="I25" s="142"/>
-      <c r="J25" s="142"/>
-      <c r="K25" s="141"/>
-      <c r="L25" s="136"/>
-      <c r="M25" s="137"/>
-      <c r="N25" s="137"/>
-      <c r="O25" s="137"/>
-      <c r="P25" s="137"/>
-      <c r="Q25" s="138"/>
+      <c r="B25" s="153"/>
+      <c r="C25" s="154"/>
+      <c r="D25" s="144"/>
+      <c r="E25" s="145"/>
+      <c r="F25" s="145"/>
+      <c r="G25" s="146"/>
+      <c r="H25" s="144"/>
+      <c r="I25" s="145"/>
+      <c r="J25" s="145"/>
+      <c r="K25" s="146"/>
+      <c r="L25" s="138"/>
+      <c r="M25" s="139"/>
+      <c r="N25" s="139"/>
+      <c r="O25" s="139"/>
+      <c r="P25" s="139"/>
+      <c r="Q25" s="140"/>
     </row>
     <row r="26" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="155" t="s">
+      <c r="A26" s="152" t="s">
         <v>47</v>
       </c>
-      <c r="B26" s="156"/>
-      <c r="C26" s="157"/>
-      <c r="D26" s="140"/>
-      <c r="E26" s="142"/>
-      <c r="F26" s="142"/>
-      <c r="G26" s="141"/>
-      <c r="H26" s="140"/>
-      <c r="I26" s="142"/>
-      <c r="J26" s="142"/>
-      <c r="K26" s="141"/>
-      <c r="L26" s="136"/>
-      <c r="M26" s="137"/>
-      <c r="N26" s="137"/>
-      <c r="O26" s="137"/>
-      <c r="P26" s="137"/>
-      <c r="Q26" s="138"/>
+      <c r="B26" s="153"/>
+      <c r="C26" s="154"/>
+      <c r="D26" s="144"/>
+      <c r="E26" s="145"/>
+      <c r="F26" s="145"/>
+      <c r="G26" s="146"/>
+      <c r="H26" s="144"/>
+      <c r="I26" s="145"/>
+      <c r="J26" s="145"/>
+      <c r="K26" s="146"/>
+      <c r="L26" s="138"/>
+      <c r="M26" s="139"/>
+      <c r="N26" s="139"/>
+      <c r="O26" s="139"/>
+      <c r="P26" s="139"/>
+      <c r="Q26" s="140"/>
       <c r="S26"/>
       <c r="T26"/>
     </row>
     <row r="27" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="146" t="s">
+      <c r="A27" s="141" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="146"/>
-      <c r="C27" s="146"/>
-      <c r="D27" s="145"/>
-      <c r="E27" s="145"/>
-      <c r="F27" s="139"/>
-      <c r="G27" s="139"/>
-      <c r="H27" s="140"/>
-      <c r="I27" s="141"/>
-      <c r="J27" s="139"/>
-      <c r="K27" s="139"/>
-      <c r="L27" s="139"/>
-      <c r="M27" s="139"/>
-      <c r="N27" s="139"/>
-      <c r="O27" s="139"/>
-      <c r="P27" s="139"/>
-      <c r="Q27" s="139"/>
+      <c r="B27" s="141"/>
+      <c r="C27" s="141"/>
+      <c r="D27" s="147"/>
+      <c r="E27" s="147"/>
+      <c r="F27" s="126"/>
+      <c r="G27" s="126"/>
+      <c r="H27" s="144"/>
+      <c r="I27" s="146"/>
+      <c r="J27" s="126"/>
+      <c r="K27" s="126"/>
+      <c r="L27" s="126"/>
+      <c r="M27" s="126"/>
+      <c r="N27" s="126"/>
+      <c r="O27" s="126"/>
+      <c r="P27" s="126"/>
+      <c r="Q27" s="126"/>
       <c r="S27"/>
       <c r="T27"/>
     </row>
     <row r="28" spans="1:20" ht="11.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="158" t="s">
+      <c r="A28" s="155" t="s">
         <v>40</v>
       </c>
-      <c r="B28" s="159"/>
-      <c r="C28" s="159"/>
-      <c r="D28" s="159"/>
-      <c r="E28" s="159"/>
-      <c r="F28" s="159"/>
-      <c r="G28" s="159"/>
-      <c r="H28" s="159"/>
-      <c r="I28" s="159"/>
-      <c r="J28" s="159"/>
-      <c r="K28" s="159"/>
-      <c r="L28" s="159"/>
-      <c r="M28" s="159"/>
-      <c r="N28" s="159"/>
-      <c r="O28" s="159"/>
-      <c r="P28" s="159"/>
-      <c r="Q28" s="160"/>
+      <c r="B28" s="156"/>
+      <c r="C28" s="156"/>
+      <c r="D28" s="156"/>
+      <c r="E28" s="156"/>
+      <c r="F28" s="156"/>
+      <c r="G28" s="156"/>
+      <c r="H28" s="156"/>
+      <c r="I28" s="156"/>
+      <c r="J28" s="156"/>
+      <c r="K28" s="156"/>
+      <c r="L28" s="156"/>
+      <c r="M28" s="156"/>
+      <c r="N28" s="156"/>
+      <c r="O28" s="156"/>
+      <c r="P28" s="156"/>
+      <c r="Q28" s="157"/>
       <c r="S28"/>
       <c r="T28"/>
     </row>
     <row r="29" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="146" t="s">
+      <c r="A29" s="141" t="s">
         <v>48</v>
       </c>
-      <c r="B29" s="146"/>
-      <c r="C29" s="146"/>
-      <c r="D29" s="145"/>
-      <c r="E29" s="145"/>
-      <c r="F29" s="139"/>
-      <c r="G29" s="139"/>
-      <c r="H29" s="140"/>
-      <c r="I29" s="141"/>
-      <c r="J29" s="139"/>
-      <c r="K29" s="139"/>
-      <c r="L29" s="140"/>
-      <c r="M29" s="142"/>
-      <c r="N29" s="141"/>
-      <c r="O29" s="140"/>
-      <c r="P29" s="142"/>
-      <c r="Q29" s="141"/>
+      <c r="B29" s="141"/>
+      <c r="C29" s="141"/>
+      <c r="D29" s="147"/>
+      <c r="E29" s="147"/>
+      <c r="F29" s="126"/>
+      <c r="G29" s="126"/>
+      <c r="H29" s="144"/>
+      <c r="I29" s="146"/>
+      <c r="J29" s="126"/>
+      <c r="K29" s="126"/>
+      <c r="L29" s="144"/>
+      <c r="M29" s="145"/>
+      <c r="N29" s="146"/>
+      <c r="O29" s="144"/>
+      <c r="P29" s="145"/>
+      <c r="Q29" s="146"/>
       <c r="S29"/>
       <c r="T29"/>
     </row>
     <row r="30" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="146" t="s">
+      <c r="A30" s="141" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="146"/>
-      <c r="C30" s="146"/>
-      <c r="D30" s="145"/>
-      <c r="E30" s="145"/>
-      <c r="F30" s="139"/>
-      <c r="G30" s="139"/>
-      <c r="H30" s="140"/>
-      <c r="I30" s="141"/>
-      <c r="J30" s="139"/>
-      <c r="K30" s="139"/>
-      <c r="L30" s="140"/>
-      <c r="M30" s="142"/>
-      <c r="N30" s="141"/>
-      <c r="O30" s="140"/>
-      <c r="P30" s="142"/>
-      <c r="Q30" s="141"/>
+      <c r="B30" s="141"/>
+      <c r="C30" s="141"/>
+      <c r="D30" s="147"/>
+      <c r="E30" s="147"/>
+      <c r="F30" s="126"/>
+      <c r="G30" s="126"/>
+      <c r="H30" s="144"/>
+      <c r="I30" s="146"/>
+      <c r="J30" s="126"/>
+      <c r="K30" s="126"/>
+      <c r="L30" s="144"/>
+      <c r="M30" s="145"/>
+      <c r="N30" s="146"/>
+      <c r="O30" s="144"/>
+      <c r="P30" s="145"/>
+      <c r="Q30" s="146"/>
       <c r="S30"/>
       <c r="T30"/>
     </row>
     <row r="31" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="146" t="s">
+      <c r="A31" s="141" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="146"/>
-      <c r="C31" s="146"/>
-      <c r="D31" s="145"/>
-      <c r="E31" s="145"/>
-      <c r="F31" s="139"/>
-      <c r="G31" s="139"/>
-      <c r="H31" s="140"/>
-      <c r="I31" s="141"/>
-      <c r="J31" s="139"/>
-      <c r="K31" s="139"/>
-      <c r="L31" s="140"/>
-      <c r="M31" s="142"/>
-      <c r="N31" s="141"/>
-      <c r="O31" s="140"/>
-      <c r="P31" s="142"/>
-      <c r="Q31" s="141"/>
+      <c r="B31" s="141"/>
+      <c r="C31" s="141"/>
+      <c r="D31" s="147"/>
+      <c r="E31" s="147"/>
+      <c r="F31" s="126"/>
+      <c r="G31" s="126"/>
+      <c r="H31" s="144"/>
+      <c r="I31" s="146"/>
+      <c r="J31" s="126"/>
+      <c r="K31" s="126"/>
+      <c r="L31" s="144"/>
+      <c r="M31" s="145"/>
+      <c r="N31" s="146"/>
+      <c r="O31" s="144"/>
+      <c r="P31" s="145"/>
+      <c r="Q31" s="146"/>
       <c r="S31"/>
       <c r="T31"/>
     </row>
     <row r="32" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="161" t="s">
+      <c r="A32" s="158" t="s">
         <v>86</v>
       </c>
-      <c r="B32" s="161"/>
-      <c r="C32" s="161"/>
-      <c r="D32" s="145">
+      <c r="B32" s="158"/>
+      <c r="C32" s="158"/>
+      <c r="D32" s="147">
         <f>+D31-D30</f>
         <v>0</v>
       </c>
-      <c r="E32" s="145"/>
-      <c r="F32" s="145">
+      <c r="E32" s="147"/>
+      <c r="F32" s="147">
         <f>+F31-F30</f>
         <v>0</v>
       </c>
-      <c r="G32" s="145"/>
-      <c r="H32" s="145">
+      <c r="G32" s="147"/>
+      <c r="H32" s="147">
         <f>+H31-H30</f>
         <v>0</v>
       </c>
-      <c r="I32" s="145"/>
-      <c r="J32" s="145">
+      <c r="I32" s="147"/>
+      <c r="J32" s="147">
         <f>+J31-J30</f>
         <v>0</v>
       </c>
-      <c r="K32" s="145"/>
-      <c r="L32" s="136">
+      <c r="K32" s="147"/>
+      <c r="L32" s="138">
         <f>+L31-L30</f>
         <v>0</v>
       </c>
-      <c r="M32" s="137"/>
-      <c r="N32" s="138"/>
-      <c r="O32" s="136">
+      <c r="M32" s="139"/>
+      <c r="N32" s="140"/>
+      <c r="O32" s="138">
         <f>+O31-O30</f>
         <v>0</v>
       </c>
-      <c r="P32" s="137"/>
-      <c r="Q32" s="138"/>
+      <c r="P32" s="139"/>
+      <c r="Q32" s="140"/>
       <c r="S32"/>
       <c r="T32"/>
     </row>
     <row r="33" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="146" t="s">
+      <c r="A33" s="141" t="s">
         <v>51</v>
       </c>
-      <c r="B33" s="146"/>
-      <c r="C33" s="146"/>
-      <c r="D33" s="145"/>
-      <c r="E33" s="145"/>
-      <c r="F33" s="139"/>
-      <c r="G33" s="139"/>
-      <c r="H33" s="140"/>
-      <c r="I33" s="141"/>
-      <c r="J33" s="139"/>
-      <c r="K33" s="139"/>
-      <c r="L33" s="140"/>
-      <c r="M33" s="142"/>
-      <c r="N33" s="141"/>
-      <c r="O33" s="140"/>
-      <c r="P33" s="142"/>
-      <c r="Q33" s="141"/>
+      <c r="B33" s="141"/>
+      <c r="C33" s="141"/>
+      <c r="D33" s="147"/>
+      <c r="E33" s="147"/>
+      <c r="F33" s="126"/>
+      <c r="G33" s="126"/>
+      <c r="H33" s="144"/>
+      <c r="I33" s="146"/>
+      <c r="J33" s="126"/>
+      <c r="K33" s="126"/>
+      <c r="L33" s="144"/>
+      <c r="M33" s="145"/>
+      <c r="N33" s="146"/>
+      <c r="O33" s="144"/>
+      <c r="P33" s="145"/>
+      <c r="Q33" s="146"/>
       <c r="S33"/>
       <c r="T33"/>
     </row>
     <row r="34" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="146" t="s">
+      <c r="A34" s="141" t="s">
         <v>52</v>
       </c>
-      <c r="B34" s="146"/>
-      <c r="C34" s="146"/>
-      <c r="D34" s="145"/>
-      <c r="E34" s="145"/>
-      <c r="F34" s="139"/>
-      <c r="G34" s="139"/>
-      <c r="H34" s="140"/>
-      <c r="I34" s="141"/>
-      <c r="J34" s="139"/>
-      <c r="K34" s="139"/>
-      <c r="L34" s="140"/>
-      <c r="M34" s="142"/>
-      <c r="N34" s="141"/>
-      <c r="O34" s="140"/>
-      <c r="P34" s="142"/>
-      <c r="Q34" s="141"/>
+      <c r="B34" s="141"/>
+      <c r="C34" s="141"/>
+      <c r="D34" s="147"/>
+      <c r="E34" s="147"/>
+      <c r="F34" s="126"/>
+      <c r="G34" s="126"/>
+      <c r="H34" s="144"/>
+      <c r="I34" s="146"/>
+      <c r="J34" s="126"/>
+      <c r="K34" s="126"/>
+      <c r="L34" s="144"/>
+      <c r="M34" s="145"/>
+      <c r="N34" s="146"/>
+      <c r="O34" s="144"/>
+      <c r="P34" s="145"/>
+      <c r="Q34" s="146"/>
       <c r="S34"/>
       <c r="T34"/>
     </row>
@@ -3019,65 +3019,65 @@
       <c r="T36"/>
     </row>
     <row r="37" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="147" t="s">
+      <c r="A37" s="161" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="113" t="s">
+      <c r="B37" s="134" t="s">
         <v>17</v>
       </c>
-      <c r="C37" s="114"/>
+      <c r="C37" s="136"/>
       <c r="D37" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E37" s="113" t="s">
+      <c r="E37" s="134" t="s">
         <v>45</v>
       </c>
-      <c r="F37" s="152"/>
-      <c r="G37" s="152"/>
-      <c r="H37" s="152"/>
-      <c r="I37" s="152"/>
-      <c r="J37" s="114"/>
+      <c r="F37" s="135"/>
+      <c r="G37" s="135"/>
+      <c r="H37" s="135"/>
+      <c r="I37" s="135"/>
+      <c r="J37" s="136"/>
       <c r="K37" s="49"/>
-      <c r="L37" s="131" t="s">
+      <c r="L37" s="184" t="s">
         <v>83</v>
       </c>
-      <c r="M37" s="131"/>
-      <c r="N37" s="131"/>
-      <c r="O37" s="131"/>
-      <c r="P37" s="131"/>
-      <c r="Q37" s="131"/>
+      <c r="M37" s="184"/>
+      <c r="N37" s="184"/>
+      <c r="O37" s="184"/>
+      <c r="P37" s="184"/>
+      <c r="Q37" s="184"/>
       <c r="S37"/>
       <c r="T37"/>
     </row>
     <row r="38" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="148"/>
-      <c r="B38" s="150" t="s">
+      <c r="A38" s="162"/>
+      <c r="B38" s="164" t="s">
         <v>70</v>
       </c>
-      <c r="C38" s="150" t="s">
+      <c r="C38" s="164" t="s">
         <v>71</v>
       </c>
       <c r="D38" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E38" s="126" t="s">
+      <c r="E38" s="166" t="s">
         <v>44</v>
       </c>
-      <c r="F38" s="127"/>
-      <c r="G38" s="126" t="s">
+      <c r="F38" s="167"/>
+      <c r="G38" s="166" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="127"/>
-      <c r="I38" s="126" t="s">
+      <c r="H38" s="167"/>
+      <c r="I38" s="166" t="s">
         <v>44</v>
       </c>
-      <c r="J38" s="127"/>
+      <c r="J38" s="167"/>
       <c r="K38" s="49"/>
-      <c r="L38" s="126" t="s">
+      <c r="L38" s="166" t="s">
         <v>19</v>
       </c>
-      <c r="M38" s="127"/>
-      <c r="N38" s="164" t="s">
+      <c r="M38" s="167"/>
+      <c r="N38" s="148" t="s">
         <v>34</v>
       </c>
       <c r="O38" s="73" t="s">
@@ -3093,27 +3093,27 @@
       <c r="T38"/>
     </row>
     <row r="39" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="149"/>
-      <c r="B39" s="151"/>
-      <c r="C39" s="151"/>
+      <c r="A39" s="163"/>
+      <c r="B39" s="165"/>
+      <c r="C39" s="165"/>
       <c r="D39" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="E39" s="128"/>
-      <c r="F39" s="129"/>
-      <c r="G39" s="128"/>
-      <c r="H39" s="129"/>
-      <c r="I39" s="128"/>
-      <c r="J39" s="129"/>
+      <c r="E39" s="168"/>
+      <c r="F39" s="169"/>
+      <c r="G39" s="168"/>
+      <c r="H39" s="169"/>
+      <c r="I39" s="168"/>
+      <c r="J39" s="169"/>
       <c r="K39" s="49"/>
-      <c r="L39" s="128"/>
-      <c r="M39" s="129"/>
-      <c r="N39" s="165"/>
-      <c r="O39" s="113" t="s">
+      <c r="L39" s="168"/>
+      <c r="M39" s="169"/>
+      <c r="N39" s="149"/>
+      <c r="O39" s="134" t="s">
         <v>73</v>
       </c>
-      <c r="P39" s="152"/>
-      <c r="Q39" s="114"/>
+      <c r="P39" s="135"/>
+      <c r="Q39" s="136"/>
       <c r="R39" s="50"/>
       <c r="S39"/>
       <c r="T39"/>
@@ -3129,15 +3129,15 @@
         <v>0</v>
       </c>
       <c r="D40" s="23"/>
-      <c r="E40" s="113"/>
-      <c r="F40" s="114"/>
-      <c r="G40" s="113"/>
-      <c r="H40" s="114"/>
-      <c r="I40" s="113"/>
-      <c r="J40" s="114"/>
+      <c r="E40" s="134"/>
+      <c r="F40" s="136"/>
+      <c r="G40" s="134"/>
+      <c r="H40" s="136"/>
+      <c r="I40" s="134"/>
+      <c r="J40" s="136"/>
       <c r="K40" s="49"/>
-      <c r="L40" s="143"/>
-      <c r="M40" s="144"/>
+      <c r="L40" s="142"/>
+      <c r="M40" s="143"/>
       <c r="N40" s="69"/>
       <c r="O40" s="102"/>
       <c r="P40" s="102"/>
@@ -3157,15 +3157,15 @@
         <v>0.64</v>
       </c>
       <c r="D41" s="23"/>
-      <c r="E41" s="113"/>
-      <c r="F41" s="114"/>
-      <c r="G41" s="113"/>
-      <c r="H41" s="114"/>
-      <c r="I41" s="113"/>
-      <c r="J41" s="114"/>
+      <c r="E41" s="134"/>
+      <c r="F41" s="136"/>
+      <c r="G41" s="134"/>
+      <c r="H41" s="136"/>
+      <c r="I41" s="134"/>
+      <c r="J41" s="136"/>
       <c r="K41" s="51"/>
-      <c r="L41" s="143"/>
-      <c r="M41" s="144"/>
+      <c r="L41" s="142"/>
+      <c r="M41" s="143"/>
       <c r="N41" s="69"/>
       <c r="O41" s="19"/>
       <c r="P41" s="19"/>
@@ -3185,15 +3185,15 @@
         <v>1.3</v>
       </c>
       <c r="D42" s="23"/>
-      <c r="E42" s="113"/>
-      <c r="F42" s="114"/>
-      <c r="G42" s="113"/>
-      <c r="H42" s="114"/>
-      <c r="I42" s="113"/>
-      <c r="J42" s="114"/>
+      <c r="E42" s="134"/>
+      <c r="F42" s="136"/>
+      <c r="G42" s="134"/>
+      <c r="H42" s="136"/>
+      <c r="I42" s="134"/>
+      <c r="J42" s="136"/>
       <c r="K42" s="51"/>
-      <c r="L42" s="143"/>
-      <c r="M42" s="144"/>
+      <c r="L42" s="142"/>
+      <c r="M42" s="143"/>
       <c r="N42" s="69"/>
       <c r="O42" s="19"/>
       <c r="P42" s="19"/>
@@ -3213,15 +3213,15 @@
         <v>1.9</v>
       </c>
       <c r="D43" s="23"/>
-      <c r="E43" s="113"/>
-      <c r="F43" s="114"/>
-      <c r="G43" s="113"/>
-      <c r="H43" s="114"/>
-      <c r="I43" s="113"/>
-      <c r="J43" s="114"/>
+      <c r="E43" s="134"/>
+      <c r="F43" s="136"/>
+      <c r="G43" s="134"/>
+      <c r="H43" s="136"/>
+      <c r="I43" s="134"/>
+      <c r="J43" s="136"/>
       <c r="K43" s="51"/>
-      <c r="L43" s="143"/>
-      <c r="M43" s="144"/>
+      <c r="L43" s="142"/>
+      <c r="M43" s="143"/>
       <c r="N43" s="69"/>
       <c r="O43" s="19"/>
       <c r="P43" s="19"/>
@@ -3243,15 +3243,15 @@
       <c r="D44" s="110">
         <v>1000</v>
       </c>
-      <c r="E44" s="115"/>
-      <c r="F44" s="116"/>
-      <c r="G44" s="115"/>
-      <c r="H44" s="116"/>
-      <c r="I44" s="115"/>
-      <c r="J44" s="116"/>
+      <c r="E44" s="159"/>
+      <c r="F44" s="160"/>
+      <c r="G44" s="159"/>
+      <c r="H44" s="160"/>
+      <c r="I44" s="159"/>
+      <c r="J44" s="160"/>
       <c r="K44" s="51"/>
-      <c r="L44" s="143"/>
-      <c r="M44" s="144"/>
+      <c r="L44" s="142"/>
+      <c r="M44" s="143"/>
       <c r="N44" s="69"/>
       <c r="O44" s="19"/>
       <c r="P44" s="19"/>
@@ -3271,12 +3271,12 @@
         <v>3.18</v>
       </c>
       <c r="D45" s="105"/>
-      <c r="E45" s="115"/>
-      <c r="F45" s="116"/>
-      <c r="G45" s="115"/>
-      <c r="H45" s="116"/>
-      <c r="I45" s="115"/>
-      <c r="J45" s="116"/>
+      <c r="E45" s="159"/>
+      <c r="F45" s="160"/>
+      <c r="G45" s="159"/>
+      <c r="H45" s="160"/>
+      <c r="I45" s="159"/>
+      <c r="J45" s="160"/>
       <c r="K45" s="51"/>
       <c r="L45" s="40"/>
       <c r="M45" s="40"/>
@@ -3299,23 +3299,23 @@
         <v>3.8</v>
       </c>
       <c r="D46" s="105"/>
-      <c r="E46" s="115"/>
-      <c r="F46" s="116"/>
-      <c r="G46" s="115"/>
-      <c r="H46" s="116"/>
-      <c r="I46" s="115"/>
-      <c r="J46" s="116"/>
+      <c r="E46" s="159"/>
+      <c r="F46" s="160"/>
+      <c r="G46" s="159"/>
+      <c r="H46" s="160"/>
+      <c r="I46" s="159"/>
+      <c r="J46" s="160"/>
       <c r="K46" s="51"/>
-      <c r="L46" s="120" t="s">
+      <c r="L46" s="180" t="s">
         <v>75</v>
       </c>
-      <c r="M46" s="121"/>
-      <c r="N46" s="122"/>
-      <c r="O46" s="133" t="s">
+      <c r="M46" s="181"/>
+      <c r="N46" s="182"/>
+      <c r="O46" s="174" t="s">
         <v>76</v>
       </c>
-      <c r="P46" s="133"/>
-      <c r="Q46" s="133"/>
+      <c r="P46" s="174"/>
+      <c r="Q46" s="174"/>
       <c r="R46" s="52"/>
       <c r="S46"/>
       <c r="T46"/>
@@ -3331,23 +3331,23 @@
         <v>4.45</v>
       </c>
       <c r="D47" s="105"/>
-      <c r="E47" s="115"/>
-      <c r="F47" s="116"/>
-      <c r="G47" s="115"/>
-      <c r="H47" s="116"/>
-      <c r="I47" s="115"/>
-      <c r="J47" s="116"/>
+      <c r="E47" s="159"/>
+      <c r="F47" s="160"/>
+      <c r="G47" s="159"/>
+      <c r="H47" s="160"/>
+      <c r="I47" s="159"/>
+      <c r="J47" s="160"/>
       <c r="K47" s="51"/>
-      <c r="L47" s="123" t="s">
+      <c r="L47" s="171" t="s">
         <v>80</v>
       </c>
-      <c r="M47" s="124"/>
-      <c r="N47" s="125"/>
-      <c r="O47" s="132" t="s">
-        <v>90</v>
-      </c>
-      <c r="P47" s="132"/>
-      <c r="Q47" s="132"/>
+      <c r="M47" s="172"/>
+      <c r="N47" s="173"/>
+      <c r="O47" s="170" t="s">
+        <v>89</v>
+      </c>
+      <c r="P47" s="170"/>
+      <c r="Q47" s="170"/>
       <c r="R47" s="52"/>
       <c r="S47"/>
       <c r="T47"/>
@@ -3365,23 +3365,23 @@
       <c r="D48" s="110">
         <v>1500</v>
       </c>
-      <c r="E48" s="115"/>
-      <c r="F48" s="116"/>
-      <c r="G48" s="115"/>
-      <c r="H48" s="116"/>
-      <c r="I48" s="115"/>
-      <c r="J48" s="116"/>
+      <c r="E48" s="159"/>
+      <c r="F48" s="160"/>
+      <c r="G48" s="159"/>
+      <c r="H48" s="160"/>
+      <c r="I48" s="159"/>
+      <c r="J48" s="160"/>
       <c r="K48" s="51"/>
-      <c r="L48" s="123" t="s">
+      <c r="L48" s="171" t="s">
         <v>81</v>
       </c>
-      <c r="M48" s="124"/>
-      <c r="N48" s="125"/>
-      <c r="O48" s="132" t="s">
-        <v>91</v>
-      </c>
-      <c r="P48" s="132"/>
-      <c r="Q48" s="132"/>
+      <c r="M48" s="172"/>
+      <c r="N48" s="173"/>
+      <c r="O48" s="170" t="s">
+        <v>90</v>
+      </c>
+      <c r="P48" s="170"/>
+      <c r="Q48" s="170"/>
       <c r="R48" s="52"/>
       <c r="S48"/>
       <c r="T48"/>
@@ -3397,23 +3397,23 @@
         <v>7.6</v>
       </c>
       <c r="D49" s="23"/>
-      <c r="E49" s="113"/>
-      <c r="F49" s="114"/>
-      <c r="G49" s="113"/>
-      <c r="H49" s="114"/>
-      <c r="I49" s="113"/>
-      <c r="J49" s="114"/>
+      <c r="E49" s="134"/>
+      <c r="F49" s="136"/>
+      <c r="G49" s="134"/>
+      <c r="H49" s="136"/>
+      <c r="I49" s="134"/>
+      <c r="J49" s="136"/>
       <c r="K49" s="53"/>
-      <c r="L49" s="123" t="s">
+      <c r="L49" s="171" t="s">
         <v>82</v>
       </c>
-      <c r="M49" s="124"/>
-      <c r="N49" s="125"/>
-      <c r="O49" s="132" t="s">
-        <v>92</v>
-      </c>
-      <c r="P49" s="132"/>
-      <c r="Q49" s="132"/>
+      <c r="M49" s="172"/>
+      <c r="N49" s="173"/>
+      <c r="O49" s="170" t="s">
+        <v>91</v>
+      </c>
+      <c r="P49" s="170"/>
+      <c r="Q49" s="170"/>
       <c r="R49" s="52"/>
       <c r="S49"/>
       <c r="T49"/>
@@ -3429,23 +3429,23 @@
         <v>10</v>
       </c>
       <c r="D50" s="23"/>
-      <c r="E50" s="113"/>
-      <c r="F50" s="114"/>
-      <c r="G50" s="113"/>
-      <c r="H50" s="114"/>
-      <c r="I50" s="113"/>
-      <c r="J50" s="114"/>
+      <c r="E50" s="134"/>
+      <c r="F50" s="136"/>
+      <c r="G50" s="134"/>
+      <c r="H50" s="136"/>
+      <c r="I50" s="134"/>
+      <c r="J50" s="136"/>
       <c r="K50" s="53"/>
       <c r="L50" s="74" t="s">
         <v>78</v>
       </c>
       <c r="M50" s="75"/>
       <c r="N50" s="76"/>
-      <c r="O50" s="132" t="s">
-        <v>93</v>
-      </c>
-      <c r="P50" s="132"/>
-      <c r="Q50" s="132"/>
+      <c r="O50" s="170" t="s">
+        <v>92</v>
+      </c>
+      <c r="P50" s="170"/>
+      <c r="Q50" s="170"/>
       <c r="R50" s="52"/>
       <c r="S50"/>
       <c r="T50"/>
@@ -3461,23 +3461,23 @@
         <v>13</v>
       </c>
       <c r="D51" s="23"/>
-      <c r="E51" s="113"/>
-      <c r="F51" s="114"/>
-      <c r="G51" s="113"/>
-      <c r="H51" s="114"/>
-      <c r="I51" s="113"/>
-      <c r="J51" s="114"/>
+      <c r="E51" s="134"/>
+      <c r="F51" s="136"/>
+      <c r="G51" s="134"/>
+      <c r="H51" s="136"/>
+      <c r="I51" s="134"/>
+      <c r="J51" s="136"/>
       <c r="K51" s="54"/>
       <c r="L51" s="74" t="s">
         <v>79</v>
       </c>
       <c r="M51" s="75"/>
       <c r="N51" s="76"/>
-      <c r="O51" s="132" t="s">
-        <v>94</v>
-      </c>
-      <c r="P51" s="132"/>
-      <c r="Q51" s="132"/>
+      <c r="O51" s="170" t="s">
+        <v>93</v>
+      </c>
+      <c r="P51" s="170"/>
+      <c r="Q51" s="170"/>
       <c r="R51" s="52"/>
       <c r="S51"/>
       <c r="T51"/>
@@ -3494,16 +3494,16 @@
       <c r="I52" s="57"/>
       <c r="J52" s="28"/>
       <c r="K52" s="14"/>
-      <c r="L52" s="123" t="s">
+      <c r="L52" s="171" t="s">
         <v>77</v>
       </c>
-      <c r="M52" s="124"/>
-      <c r="N52" s="125"/>
-      <c r="O52" s="132" t="s">
-        <v>95</v>
-      </c>
-      <c r="P52" s="132"/>
-      <c r="Q52" s="132"/>
+      <c r="M52" s="172"/>
+      <c r="N52" s="173"/>
+      <c r="O52" s="170" t="s">
+        <v>94</v>
+      </c>
+      <c r="P52" s="170"/>
+      <c r="Q52" s="170"/>
       <c r="S52"/>
       <c r="T52"/>
     </row>
@@ -3514,23 +3514,23 @@
       <c r="B53" s="59"/>
       <c r="C53" s="59"/>
       <c r="D53" s="60"/>
-      <c r="E53" s="113"/>
-      <c r="F53" s="114"/>
-      <c r="G53" s="113"/>
-      <c r="H53" s="114"/>
-      <c r="I53" s="134"/>
-      <c r="J53" s="135"/>
+      <c r="E53" s="134"/>
+      <c r="F53" s="136"/>
+      <c r="G53" s="134"/>
+      <c r="H53" s="136"/>
+      <c r="I53" s="175"/>
+      <c r="J53" s="176"/>
       <c r="K53" s="61"/>
-      <c r="L53" s="123" t="s">
+      <c r="L53" s="171" t="s">
         <v>84</v>
       </c>
-      <c r="M53" s="124"/>
-      <c r="N53" s="125"/>
-      <c r="O53" s="132" t="s">
-        <v>96</v>
-      </c>
-      <c r="P53" s="132"/>
-      <c r="Q53" s="132"/>
+      <c r="M53" s="172"/>
+      <c r="N53" s="173"/>
+      <c r="O53" s="170" t="s">
+        <v>95</v>
+      </c>
+      <c r="P53" s="170"/>
+      <c r="Q53" s="170"/>
       <c r="S53"/>
       <c r="T53"/>
     </row>
@@ -3643,7 +3643,7 @@
     </row>
     <row r="61" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="68" t="s">
-        <v>89</v>
+        <v>102</v>
       </c>
       <c r="B61" s="67"/>
       <c r="C61" s="67"/>
@@ -3663,25 +3663,25 @@
     </row>
     <row r="62" spans="1:20" ht="7.2" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="63" spans="1:20" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="174" t="s">
+      <c r="A63" s="127" t="s">
         <v>85</v>
       </c>
-      <c r="B63" s="174"/>
-      <c r="C63" s="174"/>
-      <c r="D63" s="174"/>
-      <c r="E63" s="174"/>
-      <c r="F63" s="174"/>
-      <c r="G63" s="174"/>
-      <c r="H63" s="174"/>
-      <c r="I63" s="174"/>
-      <c r="J63" s="174"/>
-      <c r="K63" s="174"/>
-      <c r="L63" s="174"/>
-      <c r="M63" s="174"/>
-      <c r="N63" s="174"/>
-      <c r="O63" s="174"/>
-      <c r="P63" s="174"/>
-      <c r="Q63" s="174"/>
+      <c r="B63" s="127"/>
+      <c r="C63" s="127"/>
+      <c r="D63" s="127"/>
+      <c r="E63" s="127"/>
+      <c r="F63" s="127"/>
+      <c r="G63" s="127"/>
+      <c r="H63" s="127"/>
+      <c r="I63" s="127"/>
+      <c r="J63" s="127"/>
+      <c r="K63" s="127"/>
+      <c r="L63" s="127"/>
+      <c r="M63" s="127"/>
+      <c r="N63" s="127"/>
+      <c r="O63" s="127"/>
+      <c r="P63" s="127"/>
+      <c r="Q63" s="127"/>
     </row>
     <row r="64" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="65" ht="15.9" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3691,16 +3691,140 @@
     <protectedRange sqref="C8:C9" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="168">
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="K9:N9"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D2:Q2"/>
-    <mergeCell ref="D3:Q3"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="L46:N46"/>
+    <mergeCell ref="L47:N47"/>
+    <mergeCell ref="L48:N48"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="L38:M39"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="L37:Q37"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="L32:N32"/>
+    <mergeCell ref="O32:Q32"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="E53:F53"/>
+    <mergeCell ref="G53:H53"/>
+    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="L49:N49"/>
+    <mergeCell ref="L52:N52"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="L53:N53"/>
+    <mergeCell ref="O53:Q53"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="O47:Q47"/>
+    <mergeCell ref="O48:Q48"/>
+    <mergeCell ref="O49:Q49"/>
+    <mergeCell ref="O52:Q52"/>
+    <mergeCell ref="O51:Q51"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="O34:Q34"/>
+    <mergeCell ref="I38:J39"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="O50:Q50"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="O46:Q46"/>
+    <mergeCell ref="G48:H48"/>
+    <mergeCell ref="G49:H49"/>
+    <mergeCell ref="G50:H50"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="A37:A39"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="E37:J37"/>
+    <mergeCell ref="E38:F39"/>
+    <mergeCell ref="G38:H39"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="E20:Q20"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="O31:Q31"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="A24:C24"/>
+    <mergeCell ref="D24:G24"/>
+    <mergeCell ref="L44:M44"/>
+    <mergeCell ref="O30:Q30"/>
+    <mergeCell ref="L30:N30"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="L29:N29"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="D26:G26"/>
+    <mergeCell ref="H25:K25"/>
+    <mergeCell ref="H26:K26"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="O33:Q33"/>
+    <mergeCell ref="N38:N39"/>
+    <mergeCell ref="O27:Q27"/>
+    <mergeCell ref="O29:Q29"/>
+    <mergeCell ref="H27:I27"/>
+    <mergeCell ref="J27:K27"/>
     <mergeCell ref="H24:K24"/>
     <mergeCell ref="L24:Q24"/>
     <mergeCell ref="D23:G23"/>
@@ -3725,140 +3849,16 @@
     <mergeCell ref="D21:G21"/>
     <mergeCell ref="A29:C29"/>
     <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A24:C24"/>
-    <mergeCell ref="D24:G24"/>
-    <mergeCell ref="L44:M44"/>
-    <mergeCell ref="O30:Q30"/>
-    <mergeCell ref="L30:N30"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="L29:N29"/>
-    <mergeCell ref="D25:G25"/>
-    <mergeCell ref="D26:G26"/>
-    <mergeCell ref="H25:K25"/>
-    <mergeCell ref="H26:K26"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="O33:Q33"/>
-    <mergeCell ref="N38:N39"/>
-    <mergeCell ref="O27:Q27"/>
-    <mergeCell ref="O29:Q29"/>
-    <mergeCell ref="H27:I27"/>
-    <mergeCell ref="J27:K27"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="E20:Q20"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="A28:Q28"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="A37:A39"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="E37:J37"/>
-    <mergeCell ref="E38:F39"/>
-    <mergeCell ref="G38:H39"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="G49:H49"/>
-    <mergeCell ref="G50:H50"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="L33:N33"/>
-    <mergeCell ref="L34:N34"/>
-    <mergeCell ref="O34:Q34"/>
-    <mergeCell ref="I38:J39"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="L41:M41"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="L43:M43"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="O50:Q50"/>
-    <mergeCell ref="L53:N53"/>
-    <mergeCell ref="O53:Q53"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="O47:Q47"/>
-    <mergeCell ref="O48:Q48"/>
-    <mergeCell ref="O49:Q49"/>
-    <mergeCell ref="O52:Q52"/>
-    <mergeCell ref="O51:Q51"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="O46:Q46"/>
-    <mergeCell ref="G48:H48"/>
-    <mergeCell ref="E53:F53"/>
-    <mergeCell ref="G53:H53"/>
-    <mergeCell ref="I53:J53"/>
-    <mergeCell ref="L49:N49"/>
-    <mergeCell ref="L52:N52"/>
-    <mergeCell ref="E49:F49"/>
-    <mergeCell ref="E50:F50"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="L46:N46"/>
-    <mergeCell ref="L47:N47"/>
-    <mergeCell ref="L48:N48"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="L38:M39"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="L37:Q37"/>
-    <mergeCell ref="E48:F48"/>
-    <mergeCell ref="L32:N32"/>
-    <mergeCell ref="O32:Q32"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G45:H45"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D2:Q2"/>
+    <mergeCell ref="D3:Q3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.39370078740157483" top="0.78740157480314965" bottom="0" header="0" footer="0"/>
@@ -3884,10 +3884,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="181" t="s">
+      <c r="A2" s="185" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="181"/>
+      <c r="B2" s="185"/>
       <c r="C2" s="5" t="s">
         <v>10</v>
       </c>

</xml_diff>

<commit_message>
Revert "fix: update Excel footer template"
This reverts commit 270554f90caba8c43578d28984b477ab805ca0e3.
</commit_message>
<xml_diff>
--- a/app/templates/Temp_CBR_ASTM.xlsx
+++ b/app/templates/Temp_CBR_ASTM.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Documents\crmnew\api-geofal-crm\app\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{280D318E-027D-4178-AB49-43739CC68D3B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8715C8F-9907-45E4-ACB1-FDE61825F565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="723" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -359,6 +359,9 @@
 (visual) (in):</t>
   </si>
   <si>
+    <t>Versión: 02 (11-11-2024)</t>
+  </si>
+  <si>
     <t>EQP-0026</t>
   </si>
   <si>
@@ -396,9 +399,6 @@
   </si>
   <si>
     <t>REALIZADO</t>
-  </si>
-  <si>
-    <t>Versión: 02 (11-11-2026)</t>
   </si>
 </sst>
 </file>
@@ -1075,24 +1075,181 @@
     <xf numFmtId="0" fontId="7" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection hidden="1"/>
+    </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1113,12 +1270,6 @@
     <xf numFmtId="166" fontId="15" fillId="0" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="4" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1147,171 +1298,20 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="10" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="11" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="12" xfId="4" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="4" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="2" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="10" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="11" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="12" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="6">
@@ -2234,43 +2234,43 @@
       <c r="A2" s="81"/>
       <c r="B2" s="82"/>
       <c r="C2" s="83"/>
-      <c r="D2" s="119" t="s">
+      <c r="D2" s="168" t="s">
         <v>15</v>
       </c>
-      <c r="E2" s="120"/>
-      <c r="F2" s="120"/>
-      <c r="G2" s="120"/>
-      <c r="H2" s="120"/>
-      <c r="I2" s="120"/>
-      <c r="J2" s="120"/>
-      <c r="K2" s="120"/>
-      <c r="L2" s="120"/>
-      <c r="M2" s="120"/>
-      <c r="N2" s="120"/>
-      <c r="O2" s="120"/>
-      <c r="P2" s="120"/>
-      <c r="Q2" s="121"/>
+      <c r="E2" s="169"/>
+      <c r="F2" s="169"/>
+      <c r="G2" s="169"/>
+      <c r="H2" s="169"/>
+      <c r="I2" s="169"/>
+      <c r="J2" s="169"/>
+      <c r="K2" s="169"/>
+      <c r="L2" s="169"/>
+      <c r="M2" s="169"/>
+      <c r="N2" s="169"/>
+      <c r="O2" s="169"/>
+      <c r="P2" s="169"/>
+      <c r="Q2" s="170"/>
     </row>
     <row r="3" spans="1:17" ht="12.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="81"/>
       <c r="B3" s="82"/>
       <c r="C3" s="83"/>
-      <c r="D3" s="122" t="s">
+      <c r="D3" s="171" t="s">
         <v>65</v>
       </c>
-      <c r="E3" s="123"/>
-      <c r="F3" s="123"/>
-      <c r="G3" s="123"/>
-      <c r="H3" s="123"/>
-      <c r="I3" s="123"/>
-      <c r="J3" s="123"/>
-      <c r="K3" s="123"/>
-      <c r="L3" s="123"/>
-      <c r="M3" s="123"/>
-      <c r="N3" s="123"/>
-      <c r="O3" s="123"/>
-      <c r="P3" s="123"/>
-      <c r="Q3" s="124"/>
+      <c r="E3" s="172"/>
+      <c r="F3" s="172"/>
+      <c r="G3" s="172"/>
+      <c r="H3" s="172"/>
+      <c r="I3" s="172"/>
+      <c r="J3" s="172"/>
+      <c r="K3" s="172"/>
+      <c r="L3" s="172"/>
+      <c r="M3" s="172"/>
+      <c r="N3" s="172"/>
+      <c r="O3" s="172"/>
+      <c r="P3" s="172"/>
+      <c r="Q3" s="173"/>
     </row>
     <row r="4" spans="1:17" ht="3" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="81"/>
@@ -2349,41 +2349,41 @@
     <row r="8" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="B8" s="32"/>
       <c r="C8" s="32"/>
-      <c r="D8" s="113" t="s">
-        <v>98</v>
-      </c>
-      <c r="E8" s="114"/>
-      <c r="F8" s="113" t="s">
+      <c r="D8" s="166" t="s">
         <v>99</v>
       </c>
-      <c r="G8" s="114"/>
-      <c r="H8" s="113" t="s">
+      <c r="E8" s="167"/>
+      <c r="F8" s="166" t="s">
         <v>100</v>
       </c>
-      <c r="I8" s="118"/>
-      <c r="J8" s="114"/>
-      <c r="K8" s="113" t="s">
+      <c r="G8" s="167"/>
+      <c r="H8" s="166" t="s">
         <v>101</v>
       </c>
-      <c r="L8" s="118"/>
-      <c r="M8" s="118"/>
-      <c r="N8" s="114"/>
+      <c r="I8" s="185"/>
+      <c r="J8" s="167"/>
+      <c r="K8" s="166" t="s">
+        <v>102</v>
+      </c>
+      <c r="L8" s="185"/>
+      <c r="M8" s="185"/>
+      <c r="N8" s="167"/>
     </row>
     <row r="9" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="32"/>
       <c r="B9" s="32"/>
       <c r="C9" s="32"/>
-      <c r="D9" s="115"/>
-      <c r="E9" s="116"/>
-      <c r="F9" s="115"/>
-      <c r="G9" s="116"/>
-      <c r="H9" s="115"/>
-      <c r="I9" s="117"/>
-      <c r="J9" s="116"/>
-      <c r="K9" s="115"/>
-      <c r="L9" s="117"/>
-      <c r="M9" s="117"/>
-      <c r="N9" s="116"/>
+      <c r="D9" s="182"/>
+      <c r="E9" s="184"/>
+      <c r="F9" s="182"/>
+      <c r="G9" s="184"/>
+      <c r="H9" s="182"/>
+      <c r="I9" s="183"/>
+      <c r="J9" s="184"/>
+      <c r="K9" s="182"/>
+      <c r="L9" s="183"/>
+      <c r="M9" s="183"/>
+      <c r="N9" s="184"/>
     </row>
     <row r="10" spans="1:17" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A10" s="32"/>
@@ -2403,46 +2403,46 @@
       <c r="O10" s="35"/>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="128" t="s">
+      <c r="A11" s="175" t="s">
         <v>62</v>
       </c>
-      <c r="B11" s="129"/>
-      <c r="C11" s="129"/>
-      <c r="D11" s="129"/>
-      <c r="E11" s="129"/>
-      <c r="F11" s="129"/>
-      <c r="G11" s="129"/>
-      <c r="H11" s="129"/>
-      <c r="I11" s="129"/>
-      <c r="J11" s="129"/>
-      <c r="K11" s="129"/>
-      <c r="L11" s="129"/>
-      <c r="M11" s="129"/>
-      <c r="N11" s="129"/>
-      <c r="O11" s="129"/>
-      <c r="P11" s="129"/>
-      <c r="Q11" s="130"/>
+      <c r="B11" s="176"/>
+      <c r="C11" s="176"/>
+      <c r="D11" s="176"/>
+      <c r="E11" s="176"/>
+      <c r="F11" s="176"/>
+      <c r="G11" s="176"/>
+      <c r="H11" s="176"/>
+      <c r="I11" s="176"/>
+      <c r="J11" s="176"/>
+      <c r="K11" s="176"/>
+      <c r="L11" s="176"/>
+      <c r="M11" s="176"/>
+      <c r="N11" s="176"/>
+      <c r="O11" s="176"/>
+      <c r="P11" s="176"/>
+      <c r="Q11" s="177"/>
     </row>
     <row r="12" spans="1:17" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="131" t="s">
+      <c r="A12" s="178" t="s">
         <v>63</v>
       </c>
-      <c r="B12" s="132"/>
-      <c r="C12" s="132"/>
-      <c r="D12" s="132"/>
-      <c r="E12" s="132"/>
-      <c r="F12" s="132"/>
-      <c r="G12" s="132"/>
-      <c r="H12" s="132"/>
-      <c r="I12" s="132"/>
-      <c r="J12" s="132"/>
-      <c r="K12" s="132"/>
-      <c r="L12" s="132"/>
-      <c r="M12" s="132"/>
-      <c r="N12" s="132"/>
-      <c r="O12" s="132"/>
-      <c r="P12" s="132"/>
-      <c r="Q12" s="133"/>
+      <c r="B12" s="179"/>
+      <c r="C12" s="179"/>
+      <c r="D12" s="179"/>
+      <c r="E12" s="179"/>
+      <c r="F12" s="179"/>
+      <c r="G12" s="179"/>
+      <c r="H12" s="179"/>
+      <c r="I12" s="179"/>
+      <c r="J12" s="179"/>
+      <c r="K12" s="179"/>
+      <c r="L12" s="179"/>
+      <c r="M12" s="179"/>
+      <c r="N12" s="179"/>
+      <c r="O12" s="179"/>
+      <c r="P12" s="179"/>
+      <c r="Q12" s="180"/>
     </row>
     <row r="13" spans="1:17" ht="11.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="36"/>
@@ -2470,8 +2470,8 @@
       <c r="B14" s="14"/>
       <c r="C14" s="43"/>
       <c r="D14" s="14"/>
-      <c r="E14" s="179"/>
-      <c r="F14" s="179"/>
+      <c r="E14" s="119"/>
+      <c r="F14" s="119"/>
       <c r="G14" s="87" t="s">
         <v>23</v>
       </c>
@@ -2481,8 +2481,8 @@
       <c r="N14" s="45" t="s">
         <v>46</v>
       </c>
-      <c r="O14" s="177"/>
-      <c r="P14" s="178"/>
+      <c r="O14" s="117"/>
+      <c r="P14" s="118"/>
       <c r="Q14" s="27"/>
     </row>
     <row r="15" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2492,8 +2492,8 @@
       <c r="B15" s="14"/>
       <c r="C15" s="14"/>
       <c r="D15" s="14"/>
-      <c r="E15" s="179"/>
-      <c r="F15" s="179"/>
+      <c r="E15" s="119"/>
+      <c r="F15" s="119"/>
       <c r="G15" s="87" t="s">
         <v>25</v>
       </c>
@@ -2503,8 +2503,8 @@
       <c r="N15" s="45" t="s">
         <v>68</v>
       </c>
-      <c r="O15" s="177"/>
-      <c r="P15" s="178"/>
+      <c r="O15" s="117"/>
+      <c r="P15" s="118"/>
       <c r="Q15" s="27"/>
     </row>
     <row r="16" spans="1:17" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
@@ -2524,8 +2524,8 @@
       <c r="N16" s="43" t="s">
         <v>57</v>
       </c>
-      <c r="O16" s="177"/>
-      <c r="P16" s="178"/>
+      <c r="O16" s="117"/>
+      <c r="P16" s="118"/>
       <c r="Q16" s="27"/>
     </row>
     <row r="17" spans="1:20" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.2">
@@ -2543,8 +2543,8 @@
       <c r="N17" s="43" t="s">
         <v>58</v>
       </c>
-      <c r="O17" s="177"/>
-      <c r="P17" s="178"/>
+      <c r="O17" s="117"/>
+      <c r="P17" s="118"/>
       <c r="Q17" s="27"/>
     </row>
     <row r="18" spans="1:20" ht="6" customHeight="1" x14ac:dyDescent="0.2">
@@ -2575,8 +2575,8 @@
       <c r="D19" s="90"/>
       <c r="E19" s="98"/>
       <c r="F19" s="98"/>
-      <c r="G19" s="183"/>
-      <c r="H19" s="183"/>
+      <c r="G19" s="130"/>
+      <c r="H19" s="130"/>
       <c r="I19" s="91"/>
       <c r="J19" s="91"/>
       <c r="K19" s="90"/>
@@ -2594,381 +2594,381 @@
       <c r="B20" s="47"/>
       <c r="C20" s="47"/>
       <c r="D20" s="48"/>
-      <c r="E20" s="150" t="s">
+      <c r="E20" s="153" t="s">
         <v>36</v>
       </c>
-      <c r="F20" s="150"/>
-      <c r="G20" s="150"/>
-      <c r="H20" s="150"/>
-      <c r="I20" s="150"/>
-      <c r="J20" s="150"/>
-      <c r="K20" s="150"/>
-      <c r="L20" s="150"/>
-      <c r="M20" s="150"/>
-      <c r="N20" s="150"/>
-      <c r="O20" s="150"/>
-      <c r="P20" s="150"/>
-      <c r="Q20" s="151"/>
+      <c r="F20" s="153"/>
+      <c r="G20" s="153"/>
+      <c r="H20" s="153"/>
+      <c r="I20" s="153"/>
+      <c r="J20" s="153"/>
+      <c r="K20" s="153"/>
+      <c r="L20" s="153"/>
+      <c r="M20" s="153"/>
+      <c r="N20" s="153"/>
+      <c r="O20" s="153"/>
+      <c r="P20" s="153"/>
+      <c r="Q20" s="154"/>
     </row>
     <row r="21" spans="1:20" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="137" t="s">
+      <c r="A21" s="162" t="s">
         <v>26</v>
       </c>
-      <c r="B21" s="137"/>
-      <c r="C21" s="137"/>
-      <c r="D21" s="137" t="s">
+      <c r="B21" s="162"/>
+      <c r="C21" s="162"/>
+      <c r="D21" s="162" t="s">
         <v>27</v>
       </c>
-      <c r="E21" s="137"/>
-      <c r="F21" s="137"/>
-      <c r="G21" s="137"/>
-      <c r="H21" s="137" t="s">
+      <c r="E21" s="162"/>
+      <c r="F21" s="162"/>
+      <c r="G21" s="162"/>
+      <c r="H21" s="162" t="s">
         <v>28</v>
       </c>
-      <c r="I21" s="137"/>
-      <c r="J21" s="137"/>
-      <c r="K21" s="137"/>
-      <c r="L21" s="137" t="s">
+      <c r="I21" s="162"/>
+      <c r="J21" s="162"/>
+      <c r="K21" s="162"/>
+      <c r="L21" s="162" t="s">
         <v>29</v>
       </c>
-      <c r="M21" s="137"/>
-      <c r="N21" s="137"/>
-      <c r="O21" s="137"/>
-      <c r="P21" s="137"/>
-      <c r="Q21" s="137"/>
+      <c r="M21" s="162"/>
+      <c r="N21" s="162"/>
+      <c r="O21" s="162"/>
+      <c r="P21" s="162"/>
+      <c r="Q21" s="162"/>
       <c r="R21" s="13"/>
     </row>
     <row r="22" spans="1:20" ht="13.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="137" t="s">
+      <c r="A22" s="162" t="s">
         <v>30</v>
       </c>
-      <c r="B22" s="137"/>
-      <c r="C22" s="137"/>
-      <c r="D22" s="137" t="s">
+      <c r="B22" s="162"/>
+      <c r="C22" s="162"/>
+      <c r="D22" s="162" t="s">
         <v>31</v>
       </c>
-      <c r="E22" s="137"/>
-      <c r="F22" s="137" t="s">
+      <c r="E22" s="162"/>
+      <c r="F22" s="162" t="s">
         <v>32</v>
       </c>
-      <c r="G22" s="137"/>
-      <c r="H22" s="137" t="s">
+      <c r="G22" s="162"/>
+      <c r="H22" s="162" t="s">
         <v>31</v>
       </c>
-      <c r="I22" s="137"/>
-      <c r="J22" s="137" t="s">
+      <c r="I22" s="162"/>
+      <c r="J22" s="162" t="s">
         <v>32</v>
       </c>
-      <c r="K22" s="137"/>
-      <c r="L22" s="137" t="s">
+      <c r="K22" s="162"/>
+      <c r="L22" s="162" t="s">
         <v>31</v>
       </c>
-      <c r="M22" s="137"/>
-      <c r="N22" s="137"/>
-      <c r="O22" s="137" t="s">
+      <c r="M22" s="162"/>
+      <c r="N22" s="162"/>
+      <c r="O22" s="162" t="s">
         <v>32</v>
       </c>
-      <c r="P22" s="137"/>
-      <c r="Q22" s="137"/>
+      <c r="P22" s="162"/>
+      <c r="Q22" s="162"/>
       <c r="R22" s="13"/>
     </row>
     <row r="23" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A23" s="141" t="s">
+      <c r="A23" s="146" t="s">
         <v>38</v>
       </c>
-      <c r="B23" s="141"/>
-      <c r="C23" s="141"/>
-      <c r="D23" s="125" t="s">
-        <v>96</v>
-      </c>
-      <c r="E23" s="125"/>
-      <c r="F23" s="125"/>
-      <c r="G23" s="125"/>
-      <c r="H23" s="126">
+      <c r="B23" s="146"/>
+      <c r="C23" s="146"/>
+      <c r="D23" s="163" t="s">
+        <v>97</v>
+      </c>
+      <c r="E23" s="163"/>
+      <c r="F23" s="163"/>
+      <c r="G23" s="163"/>
+      <c r="H23" s="139">
         <v>25</v>
       </c>
-      <c r="I23" s="126"/>
-      <c r="J23" s="126"/>
-      <c r="K23" s="126"/>
-      <c r="L23" s="126">
+      <c r="I23" s="139"/>
+      <c r="J23" s="139"/>
+      <c r="K23" s="139"/>
+      <c r="L23" s="139">
         <v>10</v>
       </c>
-      <c r="M23" s="126"/>
-      <c r="N23" s="126"/>
-      <c r="O23" s="126"/>
-      <c r="P23" s="126"/>
-      <c r="Q23" s="126"/>
+      <c r="M23" s="139"/>
+      <c r="N23" s="139"/>
+      <c r="O23" s="139"/>
+      <c r="P23" s="139"/>
+      <c r="Q23" s="139"/>
     </row>
     <row r="24" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A24" s="141" t="s">
+      <c r="A24" s="146" t="s">
         <v>33</v>
       </c>
-      <c r="B24" s="141"/>
-      <c r="C24" s="141"/>
-      <c r="D24" s="125" t="s">
-        <v>97</v>
-      </c>
-      <c r="E24" s="125"/>
-      <c r="F24" s="125"/>
-      <c r="G24" s="125"/>
-      <c r="H24" s="125" t="s">
-        <v>97</v>
-      </c>
-      <c r="I24" s="125"/>
-      <c r="J24" s="125"/>
-      <c r="K24" s="125"/>
-      <c r="L24" s="126" t="s">
-        <v>97</v>
-      </c>
-      <c r="M24" s="126"/>
-      <c r="N24" s="126"/>
-      <c r="O24" s="126"/>
-      <c r="P24" s="126"/>
-      <c r="Q24" s="126"/>
+      <c r="B24" s="146"/>
+      <c r="C24" s="146"/>
+      <c r="D24" s="163" t="s">
+        <v>98</v>
+      </c>
+      <c r="E24" s="163"/>
+      <c r="F24" s="163"/>
+      <c r="G24" s="163"/>
+      <c r="H24" s="163" t="s">
+        <v>98</v>
+      </c>
+      <c r="I24" s="163"/>
+      <c r="J24" s="163"/>
+      <c r="K24" s="163"/>
+      <c r="L24" s="139" t="s">
+        <v>98</v>
+      </c>
+      <c r="M24" s="139"/>
+      <c r="N24" s="139"/>
+      <c r="O24" s="139"/>
+      <c r="P24" s="139"/>
+      <c r="Q24" s="139"/>
     </row>
     <row r="25" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A25" s="152" t="s">
+      <c r="A25" s="155" t="s">
         <v>69</v>
       </c>
-      <c r="B25" s="153"/>
-      <c r="C25" s="154"/>
-      <c r="D25" s="144"/>
-      <c r="E25" s="145"/>
-      <c r="F25" s="145"/>
-      <c r="G25" s="146"/>
-      <c r="H25" s="144"/>
-      <c r="I25" s="145"/>
-      <c r="J25" s="145"/>
-      <c r="K25" s="146"/>
-      <c r="L25" s="138"/>
-      <c r="M25" s="139"/>
-      <c r="N25" s="139"/>
-      <c r="O25" s="139"/>
-      <c r="P25" s="139"/>
-      <c r="Q25" s="140"/>
+      <c r="B25" s="156"/>
+      <c r="C25" s="157"/>
+      <c r="D25" s="140"/>
+      <c r="E25" s="142"/>
+      <c r="F25" s="142"/>
+      <c r="G25" s="141"/>
+      <c r="H25" s="140"/>
+      <c r="I25" s="142"/>
+      <c r="J25" s="142"/>
+      <c r="K25" s="141"/>
+      <c r="L25" s="136"/>
+      <c r="M25" s="137"/>
+      <c r="N25" s="137"/>
+      <c r="O25" s="137"/>
+      <c r="P25" s="137"/>
+      <c r="Q25" s="138"/>
     </row>
     <row r="26" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A26" s="152" t="s">
+      <c r="A26" s="155" t="s">
         <v>47</v>
       </c>
-      <c r="B26" s="153"/>
-      <c r="C26" s="154"/>
-      <c r="D26" s="144"/>
-      <c r="E26" s="145"/>
-      <c r="F26" s="145"/>
-      <c r="G26" s="146"/>
-      <c r="H26" s="144"/>
-      <c r="I26" s="145"/>
-      <c r="J26" s="145"/>
-      <c r="K26" s="146"/>
-      <c r="L26" s="138"/>
-      <c r="M26" s="139"/>
-      <c r="N26" s="139"/>
-      <c r="O26" s="139"/>
-      <c r="P26" s="139"/>
-      <c r="Q26" s="140"/>
+      <c r="B26" s="156"/>
+      <c r="C26" s="157"/>
+      <c r="D26" s="140"/>
+      <c r="E26" s="142"/>
+      <c r="F26" s="142"/>
+      <c r="G26" s="141"/>
+      <c r="H26" s="140"/>
+      <c r="I26" s="142"/>
+      <c r="J26" s="142"/>
+      <c r="K26" s="141"/>
+      <c r="L26" s="136"/>
+      <c r="M26" s="137"/>
+      <c r="N26" s="137"/>
+      <c r="O26" s="137"/>
+      <c r="P26" s="137"/>
+      <c r="Q26" s="138"/>
       <c r="S26"/>
       <c r="T26"/>
     </row>
     <row r="27" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A27" s="141" t="s">
+      <c r="A27" s="146" t="s">
         <v>39</v>
       </c>
-      <c r="B27" s="141"/>
-      <c r="C27" s="141"/>
-      <c r="D27" s="147"/>
-      <c r="E27" s="147"/>
-      <c r="F27" s="126"/>
-      <c r="G27" s="126"/>
-      <c r="H27" s="144"/>
-      <c r="I27" s="146"/>
-      <c r="J27" s="126"/>
-      <c r="K27" s="126"/>
-      <c r="L27" s="126"/>
-      <c r="M27" s="126"/>
-      <c r="N27" s="126"/>
-      <c r="O27" s="126"/>
-      <c r="P27" s="126"/>
-      <c r="Q27" s="126"/>
+      <c r="B27" s="146"/>
+      <c r="C27" s="146"/>
+      <c r="D27" s="145"/>
+      <c r="E27" s="145"/>
+      <c r="F27" s="139"/>
+      <c r="G27" s="139"/>
+      <c r="H27" s="140"/>
+      <c r="I27" s="141"/>
+      <c r="J27" s="139"/>
+      <c r="K27" s="139"/>
+      <c r="L27" s="139"/>
+      <c r="M27" s="139"/>
+      <c r="N27" s="139"/>
+      <c r="O27" s="139"/>
+      <c r="P27" s="139"/>
+      <c r="Q27" s="139"/>
       <c r="S27"/>
       <c r="T27"/>
     </row>
     <row r="28" spans="1:20" ht="11.4" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="155" t="s">
+      <c r="A28" s="158" t="s">
         <v>40</v>
       </c>
-      <c r="B28" s="156"/>
-      <c r="C28" s="156"/>
-      <c r="D28" s="156"/>
-      <c r="E28" s="156"/>
-      <c r="F28" s="156"/>
-      <c r="G28" s="156"/>
-      <c r="H28" s="156"/>
-      <c r="I28" s="156"/>
-      <c r="J28" s="156"/>
-      <c r="K28" s="156"/>
-      <c r="L28" s="156"/>
-      <c r="M28" s="156"/>
-      <c r="N28" s="156"/>
-      <c r="O28" s="156"/>
-      <c r="P28" s="156"/>
-      <c r="Q28" s="157"/>
+      <c r="B28" s="159"/>
+      <c r="C28" s="159"/>
+      <c r="D28" s="159"/>
+      <c r="E28" s="159"/>
+      <c r="F28" s="159"/>
+      <c r="G28" s="159"/>
+      <c r="H28" s="159"/>
+      <c r="I28" s="159"/>
+      <c r="J28" s="159"/>
+      <c r="K28" s="159"/>
+      <c r="L28" s="159"/>
+      <c r="M28" s="159"/>
+      <c r="N28" s="159"/>
+      <c r="O28" s="159"/>
+      <c r="P28" s="159"/>
+      <c r="Q28" s="160"/>
       <c r="S28"/>
       <c r="T28"/>
     </row>
     <row r="29" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="141" t="s">
+      <c r="A29" s="146" t="s">
         <v>48</v>
       </c>
-      <c r="B29" s="141"/>
-      <c r="C29" s="141"/>
-      <c r="D29" s="147"/>
-      <c r="E29" s="147"/>
-      <c r="F29" s="126"/>
-      <c r="G29" s="126"/>
-      <c r="H29" s="144"/>
-      <c r="I29" s="146"/>
-      <c r="J29" s="126"/>
-      <c r="K29" s="126"/>
-      <c r="L29" s="144"/>
-      <c r="M29" s="145"/>
-      <c r="N29" s="146"/>
-      <c r="O29" s="144"/>
-      <c r="P29" s="145"/>
-      <c r="Q29" s="146"/>
+      <c r="B29" s="146"/>
+      <c r="C29" s="146"/>
+      <c r="D29" s="145"/>
+      <c r="E29" s="145"/>
+      <c r="F29" s="139"/>
+      <c r="G29" s="139"/>
+      <c r="H29" s="140"/>
+      <c r="I29" s="141"/>
+      <c r="J29" s="139"/>
+      <c r="K29" s="139"/>
+      <c r="L29" s="140"/>
+      <c r="M29" s="142"/>
+      <c r="N29" s="141"/>
+      <c r="O29" s="140"/>
+      <c r="P29" s="142"/>
+      <c r="Q29" s="141"/>
       <c r="S29"/>
       <c r="T29"/>
     </row>
     <row r="30" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="141" t="s">
+      <c r="A30" s="146" t="s">
         <v>49</v>
       </c>
-      <c r="B30" s="141"/>
-      <c r="C30" s="141"/>
-      <c r="D30" s="147"/>
-      <c r="E30" s="147"/>
-      <c r="F30" s="126"/>
-      <c r="G30" s="126"/>
-      <c r="H30" s="144"/>
-      <c r="I30" s="146"/>
-      <c r="J30" s="126"/>
-      <c r="K30" s="126"/>
-      <c r="L30" s="144"/>
-      <c r="M30" s="145"/>
-      <c r="N30" s="146"/>
-      <c r="O30" s="144"/>
-      <c r="P30" s="145"/>
-      <c r="Q30" s="146"/>
+      <c r="B30" s="146"/>
+      <c r="C30" s="146"/>
+      <c r="D30" s="145"/>
+      <c r="E30" s="145"/>
+      <c r="F30" s="139"/>
+      <c r="G30" s="139"/>
+      <c r="H30" s="140"/>
+      <c r="I30" s="141"/>
+      <c r="J30" s="139"/>
+      <c r="K30" s="139"/>
+      <c r="L30" s="140"/>
+      <c r="M30" s="142"/>
+      <c r="N30" s="141"/>
+      <c r="O30" s="140"/>
+      <c r="P30" s="142"/>
+      <c r="Q30" s="141"/>
       <c r="S30"/>
       <c r="T30"/>
     </row>
     <row r="31" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="141" t="s">
+      <c r="A31" s="146" t="s">
         <v>50</v>
       </c>
-      <c r="B31" s="141"/>
-      <c r="C31" s="141"/>
-      <c r="D31" s="147"/>
-      <c r="E31" s="147"/>
-      <c r="F31" s="126"/>
-      <c r="G31" s="126"/>
-      <c r="H31" s="144"/>
-      <c r="I31" s="146"/>
-      <c r="J31" s="126"/>
-      <c r="K31" s="126"/>
-      <c r="L31" s="144"/>
-      <c r="M31" s="145"/>
-      <c r="N31" s="146"/>
-      <c r="O31" s="144"/>
-      <c r="P31" s="145"/>
-      <c r="Q31" s="146"/>
+      <c r="B31" s="146"/>
+      <c r="C31" s="146"/>
+      <c r="D31" s="145"/>
+      <c r="E31" s="145"/>
+      <c r="F31" s="139"/>
+      <c r="G31" s="139"/>
+      <c r="H31" s="140"/>
+      <c r="I31" s="141"/>
+      <c r="J31" s="139"/>
+      <c r="K31" s="139"/>
+      <c r="L31" s="140"/>
+      <c r="M31" s="142"/>
+      <c r="N31" s="141"/>
+      <c r="O31" s="140"/>
+      <c r="P31" s="142"/>
+      <c r="Q31" s="141"/>
       <c r="S31"/>
       <c r="T31"/>
     </row>
     <row r="32" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="158" t="s">
+      <c r="A32" s="161" t="s">
         <v>86</v>
       </c>
-      <c r="B32" s="158"/>
-      <c r="C32" s="158"/>
-      <c r="D32" s="147">
+      <c r="B32" s="161"/>
+      <c r="C32" s="161"/>
+      <c r="D32" s="145">
         <f>+D31-D30</f>
         <v>0</v>
       </c>
-      <c r="E32" s="147"/>
-      <c r="F32" s="147">
+      <c r="E32" s="145"/>
+      <c r="F32" s="145">
         <f>+F31-F30</f>
         <v>0</v>
       </c>
-      <c r="G32" s="147"/>
-      <c r="H32" s="147">
+      <c r="G32" s="145"/>
+      <c r="H32" s="145">
         <f>+H31-H30</f>
         <v>0</v>
       </c>
-      <c r="I32" s="147"/>
-      <c r="J32" s="147">
+      <c r="I32" s="145"/>
+      <c r="J32" s="145">
         <f>+J31-J30</f>
         <v>0</v>
       </c>
-      <c r="K32" s="147"/>
-      <c r="L32" s="138">
+      <c r="K32" s="145"/>
+      <c r="L32" s="136">
         <f>+L31-L30</f>
         <v>0</v>
       </c>
-      <c r="M32" s="139"/>
-      <c r="N32" s="140"/>
-      <c r="O32" s="138">
+      <c r="M32" s="137"/>
+      <c r="N32" s="138"/>
+      <c r="O32" s="136">
         <f>+O31-O30</f>
         <v>0</v>
       </c>
-      <c r="P32" s="139"/>
-      <c r="Q32" s="140"/>
+      <c r="P32" s="137"/>
+      <c r="Q32" s="138"/>
       <c r="S32"/>
       <c r="T32"/>
     </row>
     <row r="33" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="141" t="s">
+      <c r="A33" s="146" t="s">
         <v>51</v>
       </c>
-      <c r="B33" s="141"/>
-      <c r="C33" s="141"/>
-      <c r="D33" s="147"/>
-      <c r="E33" s="147"/>
-      <c r="F33" s="126"/>
-      <c r="G33" s="126"/>
-      <c r="H33" s="144"/>
-      <c r="I33" s="146"/>
-      <c r="J33" s="126"/>
-      <c r="K33" s="126"/>
-      <c r="L33" s="144"/>
-      <c r="M33" s="145"/>
-      <c r="N33" s="146"/>
-      <c r="O33" s="144"/>
-      <c r="P33" s="145"/>
-      <c r="Q33" s="146"/>
+      <c r="B33" s="146"/>
+      <c r="C33" s="146"/>
+      <c r="D33" s="145"/>
+      <c r="E33" s="145"/>
+      <c r="F33" s="139"/>
+      <c r="G33" s="139"/>
+      <c r="H33" s="140"/>
+      <c r="I33" s="141"/>
+      <c r="J33" s="139"/>
+      <c r="K33" s="139"/>
+      <c r="L33" s="140"/>
+      <c r="M33" s="142"/>
+      <c r="N33" s="141"/>
+      <c r="O33" s="140"/>
+      <c r="P33" s="142"/>
+      <c r="Q33" s="141"/>
       <c r="S33"/>
       <c r="T33"/>
     </row>
     <row r="34" spans="1:20" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="141" t="s">
+      <c r="A34" s="146" t="s">
         <v>52</v>
       </c>
-      <c r="B34" s="141"/>
-      <c r="C34" s="141"/>
-      <c r="D34" s="147"/>
-      <c r="E34" s="147"/>
-      <c r="F34" s="126"/>
-      <c r="G34" s="126"/>
-      <c r="H34" s="144"/>
-      <c r="I34" s="146"/>
-      <c r="J34" s="126"/>
-      <c r="K34" s="126"/>
-      <c r="L34" s="144"/>
-      <c r="M34" s="145"/>
-      <c r="N34" s="146"/>
-      <c r="O34" s="144"/>
-      <c r="P34" s="145"/>
-      <c r="Q34" s="146"/>
+      <c r="B34" s="146"/>
+      <c r="C34" s="146"/>
+      <c r="D34" s="145"/>
+      <c r="E34" s="145"/>
+      <c r="F34" s="139"/>
+      <c r="G34" s="139"/>
+      <c r="H34" s="140"/>
+      <c r="I34" s="141"/>
+      <c r="J34" s="139"/>
+      <c r="K34" s="139"/>
+      <c r="L34" s="140"/>
+      <c r="M34" s="142"/>
+      <c r="N34" s="141"/>
+      <c r="O34" s="140"/>
+      <c r="P34" s="142"/>
+      <c r="Q34" s="141"/>
       <c r="S34"/>
       <c r="T34"/>
     </row>
@@ -3019,65 +3019,65 @@
       <c r="T36"/>
     </row>
     <row r="37" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="161" t="s">
+      <c r="A37" s="147" t="s">
         <v>74</v>
       </c>
-      <c r="B37" s="134" t="s">
+      <c r="B37" s="113" t="s">
         <v>17</v>
       </c>
-      <c r="C37" s="136"/>
+      <c r="C37" s="114"/>
       <c r="D37" s="20" t="s">
         <v>42</v>
       </c>
-      <c r="E37" s="134" t="s">
+      <c r="E37" s="113" t="s">
         <v>45</v>
       </c>
-      <c r="F37" s="135"/>
-      <c r="G37" s="135"/>
-      <c r="H37" s="135"/>
-      <c r="I37" s="135"/>
-      <c r="J37" s="136"/>
+      <c r="F37" s="152"/>
+      <c r="G37" s="152"/>
+      <c r="H37" s="152"/>
+      <c r="I37" s="152"/>
+      <c r="J37" s="114"/>
       <c r="K37" s="49"/>
-      <c r="L37" s="184" t="s">
+      <c r="L37" s="131" t="s">
         <v>83</v>
       </c>
-      <c r="M37" s="184"/>
-      <c r="N37" s="184"/>
-      <c r="O37" s="184"/>
-      <c r="P37" s="184"/>
-      <c r="Q37" s="184"/>
+      <c r="M37" s="131"/>
+      <c r="N37" s="131"/>
+      <c r="O37" s="131"/>
+      <c r="P37" s="131"/>
+      <c r="Q37" s="131"/>
       <c r="S37"/>
       <c r="T37"/>
     </row>
     <row r="38" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="162"/>
-      <c r="B38" s="164" t="s">
+      <c r="A38" s="148"/>
+      <c r="B38" s="150" t="s">
         <v>70</v>
       </c>
-      <c r="C38" s="164" t="s">
+      <c r="C38" s="150" t="s">
         <v>71</v>
       </c>
       <c r="D38" s="21" t="s">
         <v>43</v>
       </c>
-      <c r="E38" s="166" t="s">
+      <c r="E38" s="126" t="s">
         <v>44</v>
       </c>
-      <c r="F38" s="167"/>
-      <c r="G38" s="166" t="s">
+      <c r="F38" s="127"/>
+      <c r="G38" s="126" t="s">
         <v>44</v>
       </c>
-      <c r="H38" s="167"/>
-      <c r="I38" s="166" t="s">
+      <c r="H38" s="127"/>
+      <c r="I38" s="126" t="s">
         <v>44</v>
       </c>
-      <c r="J38" s="167"/>
+      <c r="J38" s="127"/>
       <c r="K38" s="49"/>
-      <c r="L38" s="166" t="s">
+      <c r="L38" s="126" t="s">
         <v>19</v>
       </c>
-      <c r="M38" s="167"/>
-      <c r="N38" s="148" t="s">
+      <c r="M38" s="127"/>
+      <c r="N38" s="164" t="s">
         <v>34</v>
       </c>
       <c r="O38" s="73" t="s">
@@ -3093,27 +3093,27 @@
       <c r="T38"/>
     </row>
     <row r="39" spans="1:20" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="163"/>
-      <c r="B39" s="165"/>
-      <c r="C39" s="165"/>
+      <c r="A39" s="149"/>
+      <c r="B39" s="151"/>
+      <c r="C39" s="151"/>
       <c r="D39" s="22" t="s">
         <v>72</v>
       </c>
-      <c r="E39" s="168"/>
-      <c r="F39" s="169"/>
-      <c r="G39" s="168"/>
-      <c r="H39" s="169"/>
-      <c r="I39" s="168"/>
-      <c r="J39" s="169"/>
+      <c r="E39" s="128"/>
+      <c r="F39" s="129"/>
+      <c r="G39" s="128"/>
+      <c r="H39" s="129"/>
+      <c r="I39" s="128"/>
+      <c r="J39" s="129"/>
       <c r="K39" s="49"/>
-      <c r="L39" s="168"/>
-      <c r="M39" s="169"/>
-      <c r="N39" s="149"/>
-      <c r="O39" s="134" t="s">
+      <c r="L39" s="128"/>
+      <c r="M39" s="129"/>
+      <c r="N39" s="165"/>
+      <c r="O39" s="113" t="s">
         <v>73</v>
       </c>
-      <c r="P39" s="135"/>
-      <c r="Q39" s="136"/>
+      <c r="P39" s="152"/>
+      <c r="Q39" s="114"/>
       <c r="R39" s="50"/>
       <c r="S39"/>
       <c r="T39"/>
@@ -3129,15 +3129,15 @@
         <v>0</v>
       </c>
       <c r="D40" s="23"/>
-      <c r="E40" s="134"/>
-      <c r="F40" s="136"/>
-      <c r="G40" s="134"/>
-      <c r="H40" s="136"/>
-      <c r="I40" s="134"/>
-      <c r="J40" s="136"/>
+      <c r="E40" s="113"/>
+      <c r="F40" s="114"/>
+      <c r="G40" s="113"/>
+      <c r="H40" s="114"/>
+      <c r="I40" s="113"/>
+      <c r="J40" s="114"/>
       <c r="K40" s="49"/>
-      <c r="L40" s="142"/>
-      <c r="M40" s="143"/>
+      <c r="L40" s="143"/>
+      <c r="M40" s="144"/>
       <c r="N40" s="69"/>
       <c r="O40" s="102"/>
       <c r="P40" s="102"/>
@@ -3157,15 +3157,15 @@
         <v>0.64</v>
       </c>
       <c r="D41" s="23"/>
-      <c r="E41" s="134"/>
-      <c r="F41" s="136"/>
-      <c r="G41" s="134"/>
-      <c r="H41" s="136"/>
-      <c r="I41" s="134"/>
-      <c r="J41" s="136"/>
+      <c r="E41" s="113"/>
+      <c r="F41" s="114"/>
+      <c r="G41" s="113"/>
+      <c r="H41" s="114"/>
+      <c r="I41" s="113"/>
+      <c r="J41" s="114"/>
       <c r="K41" s="51"/>
-      <c r="L41" s="142"/>
-      <c r="M41" s="143"/>
+      <c r="L41" s="143"/>
+      <c r="M41" s="144"/>
       <c r="N41" s="69"/>
       <c r="O41" s="19"/>
       <c r="P41" s="19"/>
@@ -3185,15 +3185,15 @@
         <v>1.3</v>
       </c>
       <c r="D42" s="23"/>
-      <c r="E42" s="134"/>
-      <c r="F42" s="136"/>
-      <c r="G42" s="134"/>
-      <c r="H42" s="136"/>
-      <c r="I42" s="134"/>
-      <c r="J42" s="136"/>
+      <c r="E42" s="113"/>
+      <c r="F42" s="114"/>
+      <c r="G42" s="113"/>
+      <c r="H42" s="114"/>
+      <c r="I42" s="113"/>
+      <c r="J42" s="114"/>
       <c r="K42" s="51"/>
-      <c r="L42" s="142"/>
-      <c r="M42" s="143"/>
+      <c r="L42" s="143"/>
+      <c r="M42" s="144"/>
       <c r="N42" s="69"/>
       <c r="O42" s="19"/>
       <c r="P42" s="19"/>
@@ -3213,15 +3213,15 @@
         <v>1.9</v>
       </c>
       <c r="D43" s="23"/>
-      <c r="E43" s="134"/>
-      <c r="F43" s="136"/>
-      <c r="G43" s="134"/>
-      <c r="H43" s="136"/>
-      <c r="I43" s="134"/>
-      <c r="J43" s="136"/>
+      <c r="E43" s="113"/>
+      <c r="F43" s="114"/>
+      <c r="G43" s="113"/>
+      <c r="H43" s="114"/>
+      <c r="I43" s="113"/>
+      <c r="J43" s="114"/>
       <c r="K43" s="51"/>
-      <c r="L43" s="142"/>
-      <c r="M43" s="143"/>
+      <c r="L43" s="143"/>
+      <c r="M43" s="144"/>
       <c r="N43" s="69"/>
       <c r="O43" s="19"/>
       <c r="P43" s="19"/>
@@ -3243,15 +3243,15 @@
       <c r="D44" s="110">
         <v>1000</v>
       </c>
-      <c r="E44" s="159"/>
-      <c r="F44" s="160"/>
-      <c r="G44" s="159"/>
-      <c r="H44" s="160"/>
-      <c r="I44" s="159"/>
-      <c r="J44" s="160"/>
+      <c r="E44" s="115"/>
+      <c r="F44" s="116"/>
+      <c r="G44" s="115"/>
+      <c r="H44" s="116"/>
+      <c r="I44" s="115"/>
+      <c r="J44" s="116"/>
       <c r="K44" s="51"/>
-      <c r="L44" s="142"/>
-      <c r="M44" s="143"/>
+      <c r="L44" s="143"/>
+      <c r="M44" s="144"/>
       <c r="N44" s="69"/>
       <c r="O44" s="19"/>
       <c r="P44" s="19"/>
@@ -3271,12 +3271,12 @@
         <v>3.18</v>
       </c>
       <c r="D45" s="105"/>
-      <c r="E45" s="159"/>
-      <c r="F45" s="160"/>
-      <c r="G45" s="159"/>
-      <c r="H45" s="160"/>
-      <c r="I45" s="159"/>
-      <c r="J45" s="160"/>
+      <c r="E45" s="115"/>
+      <c r="F45" s="116"/>
+      <c r="G45" s="115"/>
+      <c r="H45" s="116"/>
+      <c r="I45" s="115"/>
+      <c r="J45" s="116"/>
       <c r="K45" s="51"/>
       <c r="L45" s="40"/>
       <c r="M45" s="40"/>
@@ -3299,23 +3299,23 @@
         <v>3.8</v>
       </c>
       <c r="D46" s="105"/>
-      <c r="E46" s="159"/>
-      <c r="F46" s="160"/>
-      <c r="G46" s="159"/>
-      <c r="H46" s="160"/>
-      <c r="I46" s="159"/>
-      <c r="J46" s="160"/>
+      <c r="E46" s="115"/>
+      <c r="F46" s="116"/>
+      <c r="G46" s="115"/>
+      <c r="H46" s="116"/>
+      <c r="I46" s="115"/>
+      <c r="J46" s="116"/>
       <c r="K46" s="51"/>
-      <c r="L46" s="180" t="s">
+      <c r="L46" s="120" t="s">
         <v>75</v>
       </c>
-      <c r="M46" s="181"/>
-      <c r="N46" s="182"/>
-      <c r="O46" s="174" t="s">
+      <c r="M46" s="121"/>
+      <c r="N46" s="122"/>
+      <c r="O46" s="133" t="s">
         <v>76</v>
       </c>
-      <c r="P46" s="174"/>
-      <c r="Q46" s="174"/>
+      <c r="P46" s="133"/>
+      <c r="Q46" s="133"/>
       <c r="R46" s="52"/>
       <c r="S46"/>
       <c r="T46"/>
@@ -3331,23 +3331,23 @@
         <v>4.45</v>
       </c>
       <c r="D47" s="105"/>
-      <c r="E47" s="159"/>
-      <c r="F47" s="160"/>
-      <c r="G47" s="159"/>
-      <c r="H47" s="160"/>
-      <c r="I47" s="159"/>
-      <c r="J47" s="160"/>
+      <c r="E47" s="115"/>
+      <c r="F47" s="116"/>
+      <c r="G47" s="115"/>
+      <c r="H47" s="116"/>
+      <c r="I47" s="115"/>
+      <c r="J47" s="116"/>
       <c r="K47" s="51"/>
-      <c r="L47" s="171" t="s">
+      <c r="L47" s="123" t="s">
         <v>80</v>
       </c>
-      <c r="M47" s="172"/>
-      <c r="N47" s="173"/>
-      <c r="O47" s="170" t="s">
-        <v>89</v>
-      </c>
-      <c r="P47" s="170"/>
-      <c r="Q47" s="170"/>
+      <c r="M47" s="124"/>
+      <c r="N47" s="125"/>
+      <c r="O47" s="132" t="s">
+        <v>90</v>
+      </c>
+      <c r="P47" s="132"/>
+      <c r="Q47" s="132"/>
       <c r="R47" s="52"/>
       <c r="S47"/>
       <c r="T47"/>
@@ -3365,23 +3365,23 @@
       <c r="D48" s="110">
         <v>1500</v>
       </c>
-      <c r="E48" s="159"/>
-      <c r="F48" s="160"/>
-      <c r="G48" s="159"/>
-      <c r="H48" s="160"/>
-      <c r="I48" s="159"/>
-      <c r="J48" s="160"/>
+      <c r="E48" s="115"/>
+      <c r="F48" s="116"/>
+      <c r="G48" s="115"/>
+      <c r="H48" s="116"/>
+      <c r="I48" s="115"/>
+      <c r="J48" s="116"/>
       <c r="K48" s="51"/>
-      <c r="L48" s="171" t="s">
+      <c r="L48" s="123" t="s">
         <v>81</v>
       </c>
-      <c r="M48" s="172"/>
-      <c r="N48" s="173"/>
-      <c r="O48" s="170" t="s">
-        <v>90</v>
-      </c>
-      <c r="P48" s="170"/>
-      <c r="Q48" s="170"/>
+      <c r="M48" s="124"/>
+      <c r="N48" s="125"/>
+      <c r="O48" s="132" t="s">
+        <v>91</v>
+      </c>
+      <c r="P48" s="132"/>
+      <c r="Q48" s="132"/>
       <c r="R48" s="52"/>
       <c r="S48"/>
       <c r="T48"/>
@@ -3397,23 +3397,23 @@
         <v>7.6</v>
       </c>
       <c r="D49" s="23"/>
-      <c r="E49" s="134"/>
-      <c r="F49" s="136"/>
-      <c r="G49" s="134"/>
-      <c r="H49" s="136"/>
-      <c r="I49" s="134"/>
-      <c r="J49" s="136"/>
+      <c r="E49" s="113"/>
+      <c r="F49" s="114"/>
+      <c r="G49" s="113"/>
+      <c r="H49" s="114"/>
+      <c r="I49" s="113"/>
+      <c r="J49" s="114"/>
       <c r="K49" s="53"/>
-      <c r="L49" s="171" t="s">
+      <c r="L49" s="123" t="s">
         <v>82</v>
       </c>
-      <c r="M49" s="172"/>
-      <c r="N49" s="173"/>
-      <c r="O49" s="170" t="s">
-        <v>91</v>
-      </c>
-      <c r="P49" s="170"/>
-      <c r="Q49" s="170"/>
+      <c r="M49" s="124"/>
+      <c r="N49" s="125"/>
+      <c r="O49" s="132" t="s">
+        <v>92</v>
+      </c>
+      <c r="P49" s="132"/>
+      <c r="Q49" s="132"/>
       <c r="R49" s="52"/>
       <c r="S49"/>
       <c r="T49"/>
@@ -3429,23 +3429,23 @@
         <v>10</v>
       </c>
       <c r="D50" s="23"/>
-      <c r="E50" s="134"/>
-      <c r="F50" s="136"/>
-      <c r="G50" s="134"/>
-      <c r="H50" s="136"/>
-      <c r="I50" s="134"/>
-      <c r="J50" s="136"/>
+      <c r="E50" s="113"/>
+      <c r="F50" s="114"/>
+      <c r="G50" s="113"/>
+      <c r="H50" s="114"/>
+      <c r="I50" s="113"/>
+      <c r="J50" s="114"/>
       <c r="K50" s="53"/>
       <c r="L50" s="74" t="s">
         <v>78</v>
       </c>
       <c r="M50" s="75"/>
       <c r="N50" s="76"/>
-      <c r="O50" s="170" t="s">
-        <v>92</v>
-      </c>
-      <c r="P50" s="170"/>
-      <c r="Q50" s="170"/>
+      <c r="O50" s="132" t="s">
+        <v>93</v>
+      </c>
+      <c r="P50" s="132"/>
+      <c r="Q50" s="132"/>
       <c r="R50" s="52"/>
       <c r="S50"/>
       <c r="T50"/>
@@ -3461,23 +3461,23 @@
         <v>13</v>
       </c>
       <c r="D51" s="23"/>
-      <c r="E51" s="134"/>
-      <c r="F51" s="136"/>
-      <c r="G51" s="134"/>
-      <c r="H51" s="136"/>
-      <c r="I51" s="134"/>
-      <c r="J51" s="136"/>
+      <c r="E51" s="113"/>
+      <c r="F51" s="114"/>
+      <c r="G51" s="113"/>
+      <c r="H51" s="114"/>
+      <c r="I51" s="113"/>
+      <c r="J51" s="114"/>
       <c r="K51" s="54"/>
       <c r="L51" s="74" t="s">
         <v>79</v>
       </c>
       <c r="M51" s="75"/>
       <c r="N51" s="76"/>
-      <c r="O51" s="170" t="s">
-        <v>93</v>
-      </c>
-      <c r="P51" s="170"/>
-      <c r="Q51" s="170"/>
+      <c r="O51" s="132" t="s">
+        <v>94</v>
+      </c>
+      <c r="P51" s="132"/>
+      <c r="Q51" s="132"/>
       <c r="R51" s="52"/>
       <c r="S51"/>
       <c r="T51"/>
@@ -3494,16 +3494,16 @@
       <c r="I52" s="57"/>
       <c r="J52" s="28"/>
       <c r="K52" s="14"/>
-      <c r="L52" s="171" t="s">
+      <c r="L52" s="123" t="s">
         <v>77</v>
       </c>
-      <c r="M52" s="172"/>
-      <c r="N52" s="173"/>
-      <c r="O52" s="170" t="s">
-        <v>94</v>
-      </c>
-      <c r="P52" s="170"/>
-      <c r="Q52" s="170"/>
+      <c r="M52" s="124"/>
+      <c r="N52" s="125"/>
+      <c r="O52" s="132" t="s">
+        <v>95</v>
+      </c>
+      <c r="P52" s="132"/>
+      <c r="Q52" s="132"/>
       <c r="S52"/>
       <c r="T52"/>
     </row>
@@ -3514,23 +3514,23 @@
       <c r="B53" s="59"/>
       <c r="C53" s="59"/>
       <c r="D53" s="60"/>
-      <c r="E53" s="134"/>
-      <c r="F53" s="136"/>
-      <c r="G53" s="134"/>
-      <c r="H53" s="136"/>
-      <c r="I53" s="175"/>
-      <c r="J53" s="176"/>
+      <c r="E53" s="113"/>
+      <c r="F53" s="114"/>
+      <c r="G53" s="113"/>
+      <c r="H53" s="114"/>
+      <c r="I53" s="134"/>
+      <c r="J53" s="135"/>
       <c r="K53" s="61"/>
-      <c r="L53" s="171" t="s">
+      <c r="L53" s="123" t="s">
         <v>84</v>
       </c>
-      <c r="M53" s="172"/>
-      <c r="N53" s="173"/>
-      <c r="O53" s="170" t="s">
-        <v>95</v>
-      </c>
-      <c r="P53" s="170"/>
-      <c r="Q53" s="170"/>
+      <c r="M53" s="124"/>
+      <c r="N53" s="125"/>
+      <c r="O53" s="132" t="s">
+        <v>96</v>
+      </c>
+      <c r="P53" s="132"/>
+      <c r="Q53" s="132"/>
       <c r="S53"/>
       <c r="T53"/>
     </row>
@@ -3643,7 +3643,7 @@
     </row>
     <row r="61" spans="1:20" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="68" t="s">
-        <v>102</v>
+        <v>89</v>
       </c>
       <c r="B61" s="67"/>
       <c r="C61" s="67"/>
@@ -3663,25 +3663,25 @@
     </row>
     <row r="62" spans="1:20" ht="7.2" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="63" spans="1:20" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A63" s="127" t="s">
+      <c r="A63" s="174" t="s">
         <v>85</v>
       </c>
-      <c r="B63" s="127"/>
-      <c r="C63" s="127"/>
-      <c r="D63" s="127"/>
-      <c r="E63" s="127"/>
-      <c r="F63" s="127"/>
-      <c r="G63" s="127"/>
-      <c r="H63" s="127"/>
-      <c r="I63" s="127"/>
-      <c r="J63" s="127"/>
-      <c r="K63" s="127"/>
-      <c r="L63" s="127"/>
-      <c r="M63" s="127"/>
-      <c r="N63" s="127"/>
-      <c r="O63" s="127"/>
-      <c r="P63" s="127"/>
-      <c r="Q63" s="127"/>
+      <c r="B63" s="174"/>
+      <c r="C63" s="174"/>
+      <c r="D63" s="174"/>
+      <c r="E63" s="174"/>
+      <c r="F63" s="174"/>
+      <c r="G63" s="174"/>
+      <c r="H63" s="174"/>
+      <c r="I63" s="174"/>
+      <c r="J63" s="174"/>
+      <c r="K63" s="174"/>
+      <c r="L63" s="174"/>
+      <c r="M63" s="174"/>
+      <c r="N63" s="174"/>
+      <c r="O63" s="174"/>
+      <c r="P63" s="174"/>
+      <c r="Q63" s="174"/>
     </row>
     <row r="64" spans="1:20" ht="15.9" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="65" ht="15.9" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -3691,116 +3691,40 @@
     <protectedRange sqref="C8:C9" name="Rango3_3_1_1_1_1_1_2_1"/>
   </protectedRanges>
   <mergeCells count="168">
-    <mergeCell ref="O14:P14"/>
-    <mergeCell ref="O15:P15"/>
-    <mergeCell ref="O16:P16"/>
-    <mergeCell ref="O17:P17"/>
-    <mergeCell ref="E14:F14"/>
-    <mergeCell ref="E15:F15"/>
-    <mergeCell ref="L46:N46"/>
-    <mergeCell ref="L47:N47"/>
-    <mergeCell ref="L48:N48"/>
-    <mergeCell ref="E46:F46"/>
-    <mergeCell ref="E47:F47"/>
-    <mergeCell ref="L38:M39"/>
-    <mergeCell ref="G19:H19"/>
-    <mergeCell ref="L37:Q37"/>
-    <mergeCell ref="E48:F48"/>
-    <mergeCell ref="L32:N32"/>
-    <mergeCell ref="O32:Q32"/>
-    <mergeCell ref="I40:J40"/>
-    <mergeCell ref="G44:H44"/>
-    <mergeCell ref="G45:H45"/>
-    <mergeCell ref="E53:F53"/>
-    <mergeCell ref="G53:H53"/>
-    <mergeCell ref="I53:J53"/>
-    <mergeCell ref="L49:N49"/>
-    <mergeCell ref="L52:N52"/>
-    <mergeCell ref="E49:F49"/>
-    <mergeCell ref="E50:F50"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="L53:N53"/>
-    <mergeCell ref="O53:Q53"/>
-    <mergeCell ref="I47:J47"/>
-    <mergeCell ref="I48:J48"/>
-    <mergeCell ref="I49:J49"/>
-    <mergeCell ref="I50:J50"/>
-    <mergeCell ref="O47:Q47"/>
-    <mergeCell ref="O48:Q48"/>
-    <mergeCell ref="O49:Q49"/>
-    <mergeCell ref="O52:Q52"/>
-    <mergeCell ref="O51:Q51"/>
-    <mergeCell ref="I51:J51"/>
-    <mergeCell ref="L34:N34"/>
-    <mergeCell ref="O34:Q34"/>
-    <mergeCell ref="I38:J39"/>
-    <mergeCell ref="I44:J44"/>
-    <mergeCell ref="L40:M40"/>
-    <mergeCell ref="L41:M41"/>
-    <mergeCell ref="L42:M42"/>
-    <mergeCell ref="L43:M43"/>
-    <mergeCell ref="E51:F51"/>
-    <mergeCell ref="G40:H40"/>
-    <mergeCell ref="O50:Q50"/>
-    <mergeCell ref="G41:H41"/>
-    <mergeCell ref="G42:H42"/>
-    <mergeCell ref="O46:Q46"/>
-    <mergeCell ref="G48:H48"/>
-    <mergeCell ref="G49:H49"/>
-    <mergeCell ref="G50:H50"/>
-    <mergeCell ref="G51:H51"/>
-    <mergeCell ref="I46:J46"/>
-    <mergeCell ref="G46:H46"/>
-    <mergeCell ref="G47:H47"/>
-    <mergeCell ref="J32:K32"/>
-    <mergeCell ref="F33:G33"/>
-    <mergeCell ref="H33:I33"/>
-    <mergeCell ref="J33:K33"/>
-    <mergeCell ref="A34:C34"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="F34:G34"/>
-    <mergeCell ref="H34:I34"/>
-    <mergeCell ref="J34:K34"/>
-    <mergeCell ref="I45:J45"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="A37:A39"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B38:B39"/>
-    <mergeCell ref="C38:C39"/>
-    <mergeCell ref="G43:H43"/>
-    <mergeCell ref="E37:J37"/>
-    <mergeCell ref="E38:F39"/>
-    <mergeCell ref="G38:H39"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="I41:J41"/>
-    <mergeCell ref="I42:J42"/>
-    <mergeCell ref="I43:J43"/>
-    <mergeCell ref="L27:N27"/>
-    <mergeCell ref="E20:Q20"/>
-    <mergeCell ref="A25:C25"/>
-    <mergeCell ref="A26:C26"/>
-    <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A33:C33"/>
-    <mergeCell ref="A31:C31"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="F31:G31"/>
-    <mergeCell ref="H31:I31"/>
-    <mergeCell ref="J31:K31"/>
-    <mergeCell ref="L31:N31"/>
-    <mergeCell ref="O31:Q31"/>
-    <mergeCell ref="A28:Q28"/>
-    <mergeCell ref="A27:C27"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="F27:G27"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="A32:C32"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="F32:G32"/>
-    <mergeCell ref="H32:I32"/>
-    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="F9:G9"/>
+    <mergeCell ref="D9:E9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="D8:E8"/>
+    <mergeCell ref="D2:Q2"/>
+    <mergeCell ref="D3:Q3"/>
+    <mergeCell ref="H24:K24"/>
+    <mergeCell ref="L24:Q24"/>
+    <mergeCell ref="D23:G23"/>
+    <mergeCell ref="H23:K23"/>
+    <mergeCell ref="L23:Q23"/>
+    <mergeCell ref="A63:Q63"/>
+    <mergeCell ref="A11:Q11"/>
+    <mergeCell ref="A12:Q12"/>
+    <mergeCell ref="O39:Q39"/>
+    <mergeCell ref="H21:K21"/>
+    <mergeCell ref="L21:Q21"/>
+    <mergeCell ref="A22:C22"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="L25:Q25"/>
+    <mergeCell ref="L26:Q26"/>
+    <mergeCell ref="L22:N22"/>
+    <mergeCell ref="O22:Q22"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="D21:G21"/>
+    <mergeCell ref="A29:C29"/>
+    <mergeCell ref="A23:C23"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="D24:G24"/>
     <mergeCell ref="L44:M44"/>
@@ -3825,40 +3749,116 @@
     <mergeCell ref="O29:Q29"/>
     <mergeCell ref="H27:I27"/>
     <mergeCell ref="J27:K27"/>
-    <mergeCell ref="H24:K24"/>
-    <mergeCell ref="L24:Q24"/>
-    <mergeCell ref="D23:G23"/>
-    <mergeCell ref="H23:K23"/>
-    <mergeCell ref="L23:Q23"/>
-    <mergeCell ref="A63:Q63"/>
-    <mergeCell ref="A11:Q11"/>
-    <mergeCell ref="A12:Q12"/>
-    <mergeCell ref="O39:Q39"/>
-    <mergeCell ref="H21:K21"/>
-    <mergeCell ref="L21:Q21"/>
-    <mergeCell ref="A22:C22"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="L25:Q25"/>
-    <mergeCell ref="L26:Q26"/>
-    <mergeCell ref="L22:N22"/>
-    <mergeCell ref="O22:Q22"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="D21:G21"/>
-    <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="F9:G9"/>
-    <mergeCell ref="D9:E9"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="K9:N9"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="D8:E8"/>
-    <mergeCell ref="D2:Q2"/>
-    <mergeCell ref="D3:Q3"/>
+    <mergeCell ref="L27:N27"/>
+    <mergeCell ref="E20:Q20"/>
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="A26:C26"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A33:C33"/>
+    <mergeCell ref="A31:C31"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="F31:G31"/>
+    <mergeCell ref="H31:I31"/>
+    <mergeCell ref="J31:K31"/>
+    <mergeCell ref="L31:N31"/>
+    <mergeCell ref="O31:Q31"/>
+    <mergeCell ref="A28:Q28"/>
+    <mergeCell ref="A27:C27"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="F27:G27"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="F32:G32"/>
+    <mergeCell ref="A34:C34"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F34:G34"/>
+    <mergeCell ref="H34:I34"/>
+    <mergeCell ref="J34:K34"/>
+    <mergeCell ref="I45:J45"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="A37:A39"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B38:B39"/>
+    <mergeCell ref="C38:C39"/>
+    <mergeCell ref="G43:H43"/>
+    <mergeCell ref="E37:J37"/>
+    <mergeCell ref="E38:F39"/>
+    <mergeCell ref="G38:H39"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="I41:J41"/>
+    <mergeCell ref="I42:J42"/>
+    <mergeCell ref="I43:J43"/>
+    <mergeCell ref="H32:I32"/>
+    <mergeCell ref="G49:H49"/>
+    <mergeCell ref="G50:H50"/>
+    <mergeCell ref="G51:H51"/>
+    <mergeCell ref="I46:J46"/>
+    <mergeCell ref="G46:H46"/>
+    <mergeCell ref="G47:H47"/>
+    <mergeCell ref="J32:K32"/>
+    <mergeCell ref="F33:G33"/>
+    <mergeCell ref="H33:I33"/>
+    <mergeCell ref="J33:K33"/>
+    <mergeCell ref="L33:N33"/>
+    <mergeCell ref="L34:N34"/>
+    <mergeCell ref="O34:Q34"/>
+    <mergeCell ref="I38:J39"/>
+    <mergeCell ref="I44:J44"/>
+    <mergeCell ref="L40:M40"/>
+    <mergeCell ref="L41:M41"/>
+    <mergeCell ref="L42:M42"/>
+    <mergeCell ref="L43:M43"/>
+    <mergeCell ref="E51:F51"/>
+    <mergeCell ref="G40:H40"/>
+    <mergeCell ref="O50:Q50"/>
+    <mergeCell ref="L53:N53"/>
+    <mergeCell ref="O53:Q53"/>
+    <mergeCell ref="I47:J47"/>
+    <mergeCell ref="I48:J48"/>
+    <mergeCell ref="I49:J49"/>
+    <mergeCell ref="I50:J50"/>
+    <mergeCell ref="O47:Q47"/>
+    <mergeCell ref="O48:Q48"/>
+    <mergeCell ref="O49:Q49"/>
+    <mergeCell ref="O52:Q52"/>
+    <mergeCell ref="O51:Q51"/>
+    <mergeCell ref="I51:J51"/>
+    <mergeCell ref="G41:H41"/>
+    <mergeCell ref="G42:H42"/>
+    <mergeCell ref="O46:Q46"/>
+    <mergeCell ref="G48:H48"/>
+    <mergeCell ref="E53:F53"/>
+    <mergeCell ref="G53:H53"/>
+    <mergeCell ref="I53:J53"/>
+    <mergeCell ref="L49:N49"/>
+    <mergeCell ref="L52:N52"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="O14:P14"/>
+    <mergeCell ref="O15:P15"/>
+    <mergeCell ref="O16:P16"/>
+    <mergeCell ref="O17:P17"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="E15:F15"/>
+    <mergeCell ref="L46:N46"/>
+    <mergeCell ref="L47:N47"/>
+    <mergeCell ref="L48:N48"/>
+    <mergeCell ref="E46:F46"/>
+    <mergeCell ref="E47:F47"/>
+    <mergeCell ref="L38:M39"/>
+    <mergeCell ref="G19:H19"/>
+    <mergeCell ref="L37:Q37"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="L32:N32"/>
+    <mergeCell ref="O32:Q32"/>
+    <mergeCell ref="I40:J40"/>
+    <mergeCell ref="G44:H44"/>
+    <mergeCell ref="G45:H45"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
   <pageMargins left="0" right="0.39370078740157483" top="0.78740157480314965" bottom="0" header="0" footer="0"/>
@@ -3884,10 +3884,10 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="185" t="s">
+      <c r="A2" s="181" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="185"/>
+      <c r="B2" s="181"/>
       <c r="C2" s="5" t="s">
         <v>10</v>
       </c>

</xml_diff>